<commit_message>
Update latest.xlsx 2026-04-24 16:50
</commit_message>
<xml_diff>
--- a/latest.xlsx
+++ b/latest.xlsx
@@ -24,7 +24,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -32,6 +32,7 @@
     <numFmt numFmtId="168" formatCode="0&quot;일&quot;"/>
     <numFmt numFmtId="169" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="170" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="171" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -406,7 +407,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="181">
+  <cellXfs count="192">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -927,6 +928,39 @@
     </xf>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8435,7 +8469,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="15.75" customHeight="1">
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="21" t="n">
         <v>1</v>
       </c>
@@ -8462,25 +8496,17 @@
           <t>EW CP2220</t>
         </is>
       </c>
-      <c r="G3" s="21" t="inlineStr">
-        <is>
-          <t>2025-09-25</t>
-        </is>
-      </c>
-      <c r="H3" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="I3" s="21" t="inlineStr">
-        <is>
-          <t>2025-09-13</t>
-        </is>
-      </c>
-      <c r="J3" s="21" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="G3" s="190" t="n">
+        <v>45925</v>
+      </c>
+      <c r="H3" s="190" t="n">
+        <v>46080</v>
+      </c>
+      <c r="I3" s="190" t="n">
+        <v>45913</v>
+      </c>
+      <c r="J3" s="190" t="n">
+        <v>46262</v>
       </c>
       <c r="K3" s="21" t="inlineStr">
         <is>
@@ -8488,7 +8514,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15.75" customHeight="1">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="21" t="n">
         <v>2</v>
       </c>
@@ -8515,25 +8541,17 @@
           <t>HFR License</t>
         </is>
       </c>
-      <c r="G4" s="21" t="inlineStr">
-        <is>
-          <t>2025-11-21</t>
-        </is>
-      </c>
-      <c r="H4" s="21" t="inlineStr">
-        <is>
-          <t>2025-12-23</t>
-        </is>
-      </c>
-      <c r="I4" s="21" t="inlineStr">
-        <is>
-          <t>2025-12-01</t>
-        </is>
-      </c>
-      <c r="J4" s="21" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
+      <c r="G4" s="190" t="n">
+        <v>45982</v>
+      </c>
+      <c r="H4" s="190" t="n">
+        <v>46014</v>
+      </c>
+      <c r="I4" s="190" t="n">
+        <v>45992</v>
+      </c>
+      <c r="J4" s="190" t="n">
+        <v>46356</v>
       </c>
       <c r="K4" s="21" t="inlineStr">
         <is>
@@ -8541,7 +8559,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15.75" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="21" t="n">
         <v>3</v>
       </c>
@@ -8568,25 +8586,17 @@
           <t>EW CP2309/2315/2320-RGB</t>
         </is>
       </c>
-      <c r="G5" s="21" t="inlineStr">
-        <is>
-          <t>2025-12-02</t>
-        </is>
-      </c>
-      <c r="H5" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-11</t>
-        </is>
-      </c>
-      <c r="I5" s="21" t="inlineStr">
-        <is>
-          <t>2025-12-22</t>
-        </is>
-      </c>
-      <c r="J5" s="21" t="inlineStr">
-        <is>
-          <t>2026-12-21</t>
-        </is>
+      <c r="G5" s="190" t="n">
+        <v>45993</v>
+      </c>
+      <c r="H5" s="190" t="n">
+        <v>46064</v>
+      </c>
+      <c r="I5" s="190" t="n">
+        <v>46013</v>
+      </c>
+      <c r="J5" s="190" t="n">
+        <v>46377</v>
       </c>
       <c r="K5" s="21" t="inlineStr">
         <is>
@@ -8594,7 +8604,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15.75" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="21" t="n">
         <v>4</v>
       </c>
@@ -8621,25 +8631,17 @@
           <t>TMS-2000 EW</t>
         </is>
       </c>
-      <c r="G6" s="21" t="inlineStr">
-        <is>
-          <t>2025-12-16</t>
-        </is>
-      </c>
-      <c r="H6" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-21</t>
-        </is>
-      </c>
-      <c r="I6" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J6" s="21" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="G6" s="190" t="n">
+        <v>46007</v>
+      </c>
+      <c r="H6" s="190" t="n">
+        <v>46043</v>
+      </c>
+      <c r="I6" s="190" t="n">
+        <v>46023</v>
+      </c>
+      <c r="J6" s="190" t="n">
+        <v>46387</v>
       </c>
       <c r="K6" s="21" t="inlineStr">
         <is>
@@ -8647,7 +8649,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15.75" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="21" t="n">
         <v>5</v>
       </c>
@@ -8674,25 +8676,17 @@
           <t>TMS-1000 EW</t>
         </is>
       </c>
-      <c r="G7" s="21" t="inlineStr">
-        <is>
-          <t>2025-12-16</t>
-        </is>
-      </c>
-      <c r="H7" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-21</t>
-        </is>
-      </c>
-      <c r="I7" s="21" t="inlineStr">
-        <is>
-          <t>2025-11-01</t>
-        </is>
-      </c>
-      <c r="J7" s="21" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
+      <c r="G7" s="190" t="n">
+        <v>46007</v>
+      </c>
+      <c r="H7" s="190" t="n">
+        <v>46043</v>
+      </c>
+      <c r="I7" s="190" t="n">
+        <v>45962</v>
+      </c>
+      <c r="J7" s="190" t="n">
+        <v>46325</v>
       </c>
       <c r="K7" s="21" t="inlineStr">
         <is>
@@ -8700,7 +8694,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15.75" customHeight="1">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="21" t="n">
         <v>6</v>
       </c>
@@ -8727,25 +8721,17 @@
           <t>EW 대량 (CP2208~CP4450)</t>
         </is>
       </c>
-      <c r="G8" s="21" t="inlineStr">
-        <is>
-          <t>2025-12-19</t>
-        </is>
-      </c>
-      <c r="H8" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="I8" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J8" s="21" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="G8" s="190" t="n">
+        <v>46010</v>
+      </c>
+      <c r="H8" s="190" t="n">
+        <v>46080</v>
+      </c>
+      <c r="I8" s="190" t="n">
+        <v>46023</v>
+      </c>
+      <c r="J8" s="190" t="n">
+        <v>46387</v>
       </c>
       <c r="K8" s="21" t="inlineStr">
         <is>
@@ -8753,7 +8739,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1">
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="21" t="n">
         <v>7</v>
       </c>
@@ -8780,25 +8766,19 @@
           <t>EW 대량 (SR/SX/TMS)</t>
         </is>
       </c>
-      <c r="G9" s="21" t="inlineStr">
-        <is>
-          <t>2025-12-24</t>
-        </is>
+      <c r="G9" s="190" t="n">
+        <v>46015</v>
       </c>
       <c r="H9" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I9" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J9" s="21" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="I9" s="190" t="n">
+        <v>46023</v>
+      </c>
+      <c r="J9" s="190" t="n">
+        <v>46387</v>
       </c>
       <c r="K9" s="21" t="inlineStr">
         <is>
@@ -8806,7 +8786,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15.75" customHeight="1">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="21" t="n">
         <v>8</v>
       </c>
@@ -8833,25 +8813,17 @@
           <t>EW CP2315/CP4440-RGB</t>
         </is>
       </c>
-      <c r="G10" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-07</t>
-        </is>
-      </c>
-      <c r="H10" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-19</t>
-        </is>
-      </c>
-      <c r="I10" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-30</t>
-        </is>
-      </c>
-      <c r="J10" s="21" t="inlineStr">
-        <is>
-          <t>2027-01-29</t>
-        </is>
+      <c r="G10" s="190" t="n">
+        <v>46029</v>
+      </c>
+      <c r="H10" s="190" t="n">
+        <v>46072</v>
+      </c>
+      <c r="I10" s="190" t="n">
+        <v>46052</v>
+      </c>
+      <c r="J10" s="190" t="n">
+        <v>46416</v>
       </c>
       <c r="K10" s="21" t="inlineStr">
         <is>
@@ -8859,7 +8831,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15.75" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="21" t="n">
         <v>9</v>
       </c>
@@ -8886,10 +8858,8 @@
           <t>EW (홀딩)</t>
         </is>
       </c>
-      <c r="G11" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-07</t>
-        </is>
+      <c r="G11" s="190" t="n">
+        <v>46029</v>
       </c>
       <c r="H11" s="21" t="inlineStr">
         <is>
@@ -8912,7 +8882,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15.75" customHeight="1">
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="21" t="n">
         <v>10</v>
       </c>
@@ -8939,25 +8909,17 @@
           <t>TMS-2000 License</t>
         </is>
       </c>
-      <c r="G12" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-20</t>
-        </is>
-      </c>
-      <c r="H12" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-04</t>
-        </is>
-      </c>
-      <c r="I12" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J12" s="21" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="G12" s="190" t="n">
+        <v>46042</v>
+      </c>
+      <c r="H12" s="190" t="n">
+        <v>46057</v>
+      </c>
+      <c r="I12" s="190" t="n">
+        <v>46023</v>
+      </c>
+      <c r="J12" s="190" t="n">
+        <v>46387</v>
       </c>
       <c r="K12" s="21" t="inlineStr">
         <is>
@@ -8965,7 +8927,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15.75" customHeight="1">
+    <row r="13" ht="16" customHeight="1">
       <c r="A13" s="21" t="n">
         <v>11</v>
       </c>
@@ -8992,25 +8954,17 @@
           <t>SX/SR EW (CGV/Lotte)</t>
         </is>
       </c>
-      <c r="G13" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-20</t>
-        </is>
-      </c>
-      <c r="H13" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-04</t>
-        </is>
-      </c>
-      <c r="I13" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J13" s="21" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="G13" s="190" t="n">
+        <v>46042</v>
+      </c>
+      <c r="H13" s="190" t="n">
+        <v>46057</v>
+      </c>
+      <c r="I13" s="190" t="n">
+        <v>46023</v>
+      </c>
+      <c r="J13" s="190" t="n">
+        <v>46387</v>
       </c>
       <c r="K13" s="21" t="inlineStr">
         <is>
@@ -9018,7 +8972,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15.75" customHeight="1">
+    <row r="14" ht="16" customHeight="1">
       <c r="A14" s="21" t="n">
         <v>12</v>
       </c>
@@ -9045,25 +8999,17 @@
           <t>SR-1000/SX-3000 EW</t>
         </is>
       </c>
-      <c r="G14" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-20</t>
-        </is>
-      </c>
-      <c r="H14" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-04</t>
-        </is>
-      </c>
-      <c r="I14" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J14" s="21" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="G14" s="190" t="n">
+        <v>46042</v>
+      </c>
+      <c r="H14" s="190" t="n">
+        <v>46057</v>
+      </c>
+      <c r="I14" s="190" t="n">
+        <v>46023</v>
+      </c>
+      <c r="J14" s="190" t="n">
+        <v>46387</v>
       </c>
       <c r="K14" s="21" t="inlineStr">
         <is>
@@ -9071,7 +9017,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15.75" customHeight="1">
+    <row r="15" ht="16" customHeight="1">
       <c r="A15" s="21" t="n">
         <v>13</v>
       </c>
@@ -9098,25 +9044,17 @@
           <t>EW (메가박스 외)</t>
         </is>
       </c>
-      <c r="G15" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-04</t>
-        </is>
-      </c>
-      <c r="H15" s="21" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="I15" s="21" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-      <c r="J15" s="95" t="inlineStr">
-        <is>
-          <t>2027-02-28</t>
-        </is>
+      <c r="G15" s="190" t="n">
+        <v>46057</v>
+      </c>
+      <c r="H15" s="190" t="n">
+        <v>46113</v>
+      </c>
+      <c r="I15" s="190" t="n">
+        <v>46082</v>
+      </c>
+      <c r="J15" s="191" t="n">
+        <v>46446</v>
       </c>
       <c r="K15" s="21" t="inlineStr">
         <is>
@@ -9124,7 +9062,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15.75" customHeight="1">
+    <row r="16" ht="16" customHeight="1">
       <c r="A16" s="21" t="n">
         <v>14</v>
       </c>
@@ -9151,25 +9089,17 @@
           <t>SR/SX EW (하남미사 외)</t>
         </is>
       </c>
-      <c r="G16" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-07</t>
-        </is>
-      </c>
-      <c r="H16" s="21" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="I16" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J16" s="95" t="inlineStr">
-        <is>
-          <t>2027-02-22</t>
-        </is>
+      <c r="G16" s="190" t="n">
+        <v>46060</v>
+      </c>
+      <c r="H16" s="190" t="n">
+        <v>46113</v>
+      </c>
+      <c r="I16" s="190" t="n">
+        <v>46023</v>
+      </c>
+      <c r="J16" s="191" t="n">
+        <v>46440</v>
       </c>
       <c r="K16" s="21" t="inlineStr">
         <is>
@@ -9177,7 +9107,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1">
+    <row r="17" ht="16" customHeight="1">
       <c r="A17" s="21" t="n">
         <v>15</v>
       </c>
@@ -9204,25 +9134,17 @@
           <t>TMS-1000 License</t>
         </is>
       </c>
-      <c r="G17" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="H17" s="21" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="I17" s="21" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-      <c r="J17" s="95" t="inlineStr">
-        <is>
-          <t>2027-02-28</t>
-        </is>
+      <c r="G17" s="190" t="n">
+        <v>46080</v>
+      </c>
+      <c r="H17" s="190" t="n">
+        <v>46113</v>
+      </c>
+      <c r="I17" s="190" t="n">
+        <v>46082</v>
+      </c>
+      <c r="J17" s="191" t="n">
+        <v>46446</v>
       </c>
       <c r="K17" s="21" t="inlineStr">
         <is>
@@ -9230,60 +9152,56 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="39" t="n">
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="95" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="39" t="inlineStr">
+      <c r="B18" s="95" t="inlineStr">
         <is>
           <t>GPO471</t>
         </is>
       </c>
-      <c r="C18" s="92" t="inlineStr">
+      <c r="C18" s="181" t="inlineStr">
         <is>
           <t>GDC</t>
         </is>
       </c>
-      <c r="D18" s="92" t="inlineStr">
+      <c r="D18" s="181" t="inlineStr">
         <is>
           <t>라이센스</t>
         </is>
       </c>
-      <c r="E18" s="94" t="n">
+      <c r="E18" s="182" t="n">
         <v>500</v>
       </c>
-      <c r="F18" s="39" t="inlineStr">
+      <c r="F18" s="95" t="inlineStr">
         <is>
           <t>Dolby Atmos License</t>
         </is>
       </c>
-      <c r="G18" s="39" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="H18" s="39" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="I18" s="39" t="inlineStr">
+      <c r="G18" s="191" t="n">
+        <v>46088</v>
+      </c>
+      <c r="H18" s="191" t="n">
+        <v>46113</v>
+      </c>
+      <c r="I18" s="95" t="inlineStr">
         <is>
           <t>미확인</t>
         </is>
       </c>
-      <c r="J18" s="96" t="inlineStr">
+      <c r="J18" s="95" t="inlineStr">
         <is>
           <t>미확인</t>
         </is>
       </c>
-      <c r="K18" s="21" t="inlineStr">
+      <c r="K18" s="95" t="inlineStr">
         <is>
           <t>라이센스</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1">
+    <row r="19" ht="16" customHeight="1">
       <c r="A19" s="21" t="n">
         <v>17</v>
       </c>
@@ -9310,25 +9228,19 @@
           <t>EW (CGV 동백 외 Warranty Extension)</t>
         </is>
       </c>
-      <c r="G19" s="21" t="inlineStr">
-        <is>
-          <t>2026-03-28</t>
-        </is>
+      <c r="G19" s="190" t="n">
+        <v>46109</v>
       </c>
       <c r="H19" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I19" s="21" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="J19" s="95" t="inlineStr">
-        <is>
-          <t>2027-03-31</t>
-        </is>
+      <c r="I19" s="190" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J19" s="191" t="n">
+        <v>46477</v>
       </c>
       <c r="K19" s="21" t="inlineStr">
         <is>
@@ -9336,95 +9248,95 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="150" t="n">
-        <v>17</v>
-      </c>
-      <c r="B20" s="150" t="inlineStr">
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="183" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="183" t="inlineStr">
         <is>
           <t>CPO697</t>
         </is>
       </c>
-      <c r="C20" s="151" t="inlineStr">
+      <c r="C20" s="184" t="inlineStr">
         <is>
           <t>Christie</t>
         </is>
       </c>
-      <c r="D20" s="151" t="inlineStr">
+      <c r="D20" s="184" t="inlineStr">
         <is>
           <t>워런티(EW)</t>
         </is>
       </c>
-      <c r="E20" s="152" t="n">
+      <c r="E20" s="185" t="n">
         <v>15289</v>
       </c>
-      <c r="F20" s="150" t="inlineStr">
+      <c r="F20" s="183" t="inlineStr">
         <is>
           <t>EW CP4425/CP2308/CP2315/CP2309/CP2320 13대</t>
         </is>
       </c>
-      <c r="G20" s="153" t="n">
+      <c r="G20" s="186" t="n">
         <v>46136</v>
       </c>
-      <c r="H20" s="150" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I20" s="153" t="n">
+      <c r="H20" s="186" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="186" t="n">
         <v>46168</v>
       </c>
-      <c r="J20" s="153" t="n">
+      <c r="J20" s="186" t="n">
         <v>46532</v>
       </c>
-      <c r="K20" s="150" t="inlineStr">
+      <c r="K20" s="183" t="inlineStr">
         <is>
           <t>라이센스</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="150" t="n">
-        <v>18</v>
-      </c>
-      <c r="B21" s="150" t="inlineStr">
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="183" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="183" t="inlineStr">
         <is>
           <t>CPO693-2</t>
         </is>
       </c>
-      <c r="C21" s="151" t="inlineStr">
+      <c r="C21" s="184" t="inlineStr">
         <is>
           <t>Christie</t>
         </is>
       </c>
-      <c r="D21" s="151" t="inlineStr">
+      <c r="D21" s="184" t="inlineStr">
         <is>
           <t>워런티(EW)</t>
         </is>
       </c>
-      <c r="E21" s="152" t="n">
+      <c r="E21" s="185" t="n">
         <v>2550</v>
       </c>
-      <c r="F21" s="150" t="inlineStr">
+      <c r="F21" s="183" t="inlineStr">
         <is>
           <t>CP4420-RGB 2년 워런티 (CGV 구미)</t>
         </is>
       </c>
-      <c r="G21" s="153" t="n">
+      <c r="G21" s="186" t="n">
         <v>46133</v>
       </c>
-      <c r="H21" s="150" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I21" s="153" t="n">
+      <c r="H21" s="186" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I21" s="186" t="n">
         <v>46142</v>
       </c>
-      <c r="J21" s="153" t="n">
+      <c r="J21" s="186" t="n">
         <v>46872</v>
       </c>
-      <c r="K21" s="150" t="inlineStr">
+      <c r="K21" s="183" t="inlineStr">
         <is>
           <t>라이센스</t>
         </is>
@@ -10614,185 +10526,185 @@
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="39" t="n">
+      <c r="A3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="39" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>2025.12.01</t>
         </is>
       </c>
-      <c r="C3" s="92" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Christie</t>
         </is>
       </c>
-      <c r="D3" s="39" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>CPO668-3, CPO673</t>
         </is>
       </c>
-      <c r="E3" s="40" t="n">
+      <c r="E3" s="44" t="n">
         <v>35563</v>
       </c>
-      <c r="F3" s="161" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="39" t="n">
+      <c r="F3" s="162" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="H3" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="42">
+      <c r="H3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="9">
         <f>ROUND((E3+G3)*F3+H3+I3,0)</f>
         <v/>
       </c>
-      <c r="L3" s="43">
+      <c r="L3" s="46">
         <f>J3-K3</f>
         <v/>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="39" t="n">
+      <c r="A4" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="39" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>2025.12.02</t>
         </is>
       </c>
-      <c r="C4" s="92" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>GDC</t>
         </is>
       </c>
-      <c r="D4" s="39" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>GPO-445, 446-1, 447, 448</t>
         </is>
       </c>
-      <c r="E4" s="40" t="n">
+      <c r="E4" s="44" t="n">
         <v>55830</v>
       </c>
-      <c r="F4" s="161" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="39" t="n">
+      <c r="F4" s="162" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="H4" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="42">
+      <c r="H4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="9">
         <f>ROUND((E4+G4)*F4+H4+I4,0)</f>
         <v/>
       </c>
-      <c r="L4" s="43">
+      <c r="L4" s="46">
         <f>J4-K4</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="39" t="n">
+      <c r="A5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="39" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>2025.12.02</t>
         </is>
       </c>
-      <c r="C5" s="92" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Thali Consulting</t>
         </is>
       </c>
-      <c r="D5" s="39" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>(PO미기재)</t>
         </is>
       </c>
-      <c r="E5" s="40" t="n">
+      <c r="E5" s="44" t="n">
         <v>9247.690000000001</v>
       </c>
-      <c r="F5" s="161" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="39" t="n">
+      <c r="F5" s="162" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="H5" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="42">
+      <c r="H5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="9">
         <f>ROUND((E5+G5)*F5+H5+I5,0)</f>
         <v/>
       </c>
-      <c r="L5" s="43">
+      <c r="L5" s="46">
         <f>J5-K5</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="39" t="n">
+      <c r="A6" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="39" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>2025.12.02</t>
         </is>
       </c>
-      <c r="C6" s="92" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Christie</t>
         </is>
       </c>
-      <c r="D6" s="39" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>CPO-669</t>
         </is>
       </c>
-      <c r="E6" s="40" t="n">
+      <c r="E6" s="44" t="n">
         <v>7410</v>
       </c>
-      <c r="F6" s="161" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="39" t="n">
+      <c r="F6" s="162" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="H6" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="42">
+      <c r="H6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="9">
         <f>ROUND((E6+G6)*F6+H6+I6,0)</f>
         <v/>
       </c>
-      <c r="L6" s="43">
+      <c r="L6" s="46">
         <f>J6-K6</f>
         <v/>
       </c>
@@ -10982,47 +10894,47 @@
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="13" t="n">
+      <c r="A11" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>2025.12.19</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>GDC(라이센스)</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>/ROC/라이센스</t>
         </is>
       </c>
-      <c r="E11" s="47" t="n">
+      <c r="E11" s="44" t="n">
         <v>1200</v>
       </c>
-      <c r="F11" s="163" t="n">
+      <c r="F11" s="162" t="n">
         <v>1464.9</v>
       </c>
-      <c r="G11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="19">
+      <c r="G11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="9">
         <f>ROUND((E11+G11)*F11+H11+I11,0)</f>
         <v/>
       </c>
-      <c r="L11" s="49">
+      <c r="L11" s="46">
         <f>J11-K11</f>
         <v/>
       </c>
@@ -11718,277 +11630,277 @@
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="13" t="n">
+      <c r="A27" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>2026.04.14</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>GDC</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>GPO468-1, 472, 468-2</t>
+        </is>
+      </c>
+      <c r="E27" s="44" t="n">
+        <v>57650</v>
+      </c>
+      <c r="F27" s="162" t="n">
+        <v>1481.9</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>12500</v>
+      </c>
+      <c r="I27" s="9" t="n">
+        <v>8000</v>
+      </c>
+      <c r="J27" s="9" t="n">
+        <v>85481673</v>
+      </c>
+      <c r="K27" s="9">
+        <f>ROUND((E27+G27)*F27+H27+I27,0)</f>
+        <v/>
+      </c>
+      <c r="L27" s="46">
+        <f>J27-K27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="171" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>2026.04.14</t>
-        </is>
-      </c>
-      <c r="C27" s="14" t="inlineStr">
-        <is>
-          <t>GDC</t>
-        </is>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
-        <is>
-          <t>GPO468-1, 472, 468-2</t>
-        </is>
-      </c>
-      <c r="E27" s="47" t="n">
-        <v>57650</v>
-      </c>
-      <c r="F27" s="163" t="n">
-        <v>1481.9</v>
-      </c>
-      <c r="G27" s="13" t="n">
+      <c r="B28" s="171" t="inlineStr">
+        <is>
+          <t>2026.04.01</t>
+        </is>
+      </c>
+      <c r="C28" s="172" t="inlineStr">
+        <is>
+          <t>Swank</t>
+        </is>
+      </c>
+      <c r="D28" s="171" t="inlineStr">
+        <is>
+          <t>(영화 라이센스)</t>
+        </is>
+      </c>
+      <c r="E28" s="173" t="n">
+        <v>814</v>
+      </c>
+      <c r="F28" s="187" t="n">
+        <v>1505</v>
+      </c>
+      <c r="G28" s="171" t="n">
         <v>20</v>
       </c>
-      <c r="H27" s="19" t="n">
+      <c r="H28" s="176" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I28" s="176" t="n">
+        <v>8000</v>
+      </c>
+      <c r="J28" s="176" t="n">
+        <v>1268170</v>
+      </c>
+      <c r="K28" s="176">
+        <f>ROUND((E28+G28)*F28+H28+I28,0)</f>
+        <v/>
+      </c>
+      <c r="L28" s="177">
+        <f>J28-K28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="27.75" customHeight="1">
+      <c r="A29" s="171" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="171" t="inlineStr">
+        <is>
+          <t>2026.04.02</t>
+        </is>
+      </c>
+      <c r="C29" s="172" t="inlineStr">
+        <is>
+          <t>Monoplex</t>
+        </is>
+      </c>
+      <c r="D29" s="171" t="inlineStr">
+        <is>
+          <t>(영업)</t>
+        </is>
+      </c>
+      <c r="E29" s="173" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F29" s="187" t="n">
+        <v>1520.1</v>
+      </c>
+      <c r="G29" s="171" t="n">
+        <v>20</v>
+      </c>
+      <c r="H29" s="176" t="n">
+        <v>25000</v>
+      </c>
+      <c r="I29" s="176" t="n">
+        <v>8000</v>
+      </c>
+      <c r="J29" s="176" t="n">
+        <v>45666402</v>
+      </c>
+      <c r="K29" s="176">
+        <f>ROUND((E29+G29)*F29+H29+I29,0)</f>
+        <v/>
+      </c>
+      <c r="L29" s="177">
+        <f>J29-K29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="A30" s="171" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="171" t="inlineStr">
+        <is>
+          <t>2026.04.21</t>
+        </is>
+      </c>
+      <c r="C30" s="172" t="inlineStr">
+        <is>
+          <t>Ferco</t>
+        </is>
+      </c>
+      <c r="D30" s="171" t="inlineStr">
+        <is>
+          <t>MONOPLEX20260126-01</t>
+        </is>
+      </c>
+      <c r="E30" s="173" t="n">
+        <v>25976</v>
+      </c>
+      <c r="F30" s="187" t="n">
+        <v>1473.3</v>
+      </c>
+      <c r="G30" s="171" t="n">
+        <v>20</v>
+      </c>
+      <c r="H30" s="176" t="n">
         <v>12500</v>
       </c>
-      <c r="I27" s="19" t="n">
+      <c r="I30" s="176" t="n">
         <v>8000</v>
       </c>
-      <c r="J27" s="19" t="n">
-        <v>85481673</v>
-      </c>
-      <c r="K27" s="19">
-        <f>ROUND((E27+G27)*F27+H27+I27,0)</f>
-        <v/>
-      </c>
-      <c r="L27" s="49">
-        <f>J27-K27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="164" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="164" t="inlineStr">
-        <is>
-          <t>2026.04.01</t>
-        </is>
-      </c>
-      <c r="C28" s="165" t="inlineStr">
-        <is>
-          <t>Swank</t>
-        </is>
-      </c>
-      <c r="D28" s="164" t="inlineStr">
-        <is>
-          <t>(영화 라이센스)</t>
-        </is>
-      </c>
-      <c r="E28" s="166" t="n">
-        <v>814</v>
-      </c>
-      <c r="F28" s="167" t="n">
-        <v>1505</v>
-      </c>
-      <c r="G28" s="164" t="n">
+      <c r="J30" s="176" t="n">
+        <v>38320406</v>
+      </c>
+      <c r="K30" s="176">
+        <f>ROUND((E30+G30)*F30+H30+I30,0)</f>
+        <v/>
+      </c>
+      <c r="L30" s="177">
+        <f>J30-K30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="A31" s="171" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="171" t="inlineStr">
+        <is>
+          <t>2026.04.22</t>
+        </is>
+      </c>
+      <c r="C31" s="172" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="D31" s="171" t="inlineStr">
+        <is>
+          <t>CPO692(692-1, 692-2)</t>
+        </is>
+      </c>
+      <c r="E31" s="173" t="n">
+        <v>297580</v>
+      </c>
+      <c r="F31" s="187" t="n">
+        <v>1482.8</v>
+      </c>
+      <c r="G31" s="171" t="n">
         <v>20</v>
       </c>
-      <c r="H28" s="168" t="n">
-        <v>5000</v>
-      </c>
-      <c r="I28" s="168" t="n">
+      <c r="H31" s="176" t="n">
+        <v>12500</v>
+      </c>
+      <c r="I31" s="176" t="n">
         <v>8000</v>
       </c>
-      <c r="J28" s="168" t="n">
-        <v>1268170</v>
-      </c>
-      <c r="K28" s="168">
-        <f>ROUND((E28+G28)*F28+H28+I28,0)</f>
-        <v/>
-      </c>
-      <c r="L28" s="169">
-        <f>J28-K28</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="27.75" customHeight="1">
-      <c r="A29" s="164" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="164" t="inlineStr">
-        <is>
-          <t>2026.04.02</t>
-        </is>
-      </c>
-      <c r="C29" s="165" t="inlineStr">
-        <is>
-          <t>Monoplex</t>
-        </is>
-      </c>
-      <c r="D29" s="164" t="inlineStr">
-        <is>
-          <t>(영업)</t>
-        </is>
-      </c>
-      <c r="E29" s="166" t="n">
-        <v>30000</v>
-      </c>
-      <c r="F29" s="167" t="n">
-        <v>1520.1</v>
-      </c>
-      <c r="G29" s="164" t="n">
-        <v>20</v>
-      </c>
-      <c r="H29" s="168" t="n">
-        <v>25000</v>
-      </c>
-      <c r="I29" s="168" t="n">
+      <c r="J31" s="176" t="n">
+        <v>441301780</v>
+      </c>
+      <c r="K31" s="176">
+        <f>ROUND((E31+G31)*F31+H31+I31,0)</f>
+        <v/>
+      </c>
+      <c r="L31" s="177">
+        <f>J31-K31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="171" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="171" t="inlineStr">
+        <is>
+          <t>2026.04.22</t>
+        </is>
+      </c>
+      <c r="C32" s="172" t="inlineStr">
+        <is>
+          <t>Elicent (EUR)</t>
+        </is>
+      </c>
+      <c r="D32" s="171" t="inlineStr">
+        <is>
+          <t>EPO18</t>
+        </is>
+      </c>
+      <c r="E32" s="173" t="n">
+        <v>4388.4</v>
+      </c>
+      <c r="F32" s="187" t="n">
+        <v>1741.08</v>
+      </c>
+      <c r="G32" s="171" t="n">
+        <v>25</v>
+      </c>
+      <c r="H32" s="176" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I32" s="176" t="n">
         <v>8000</v>
       </c>
-      <c r="J29" s="168" t="n">
-        <v>45666402</v>
-      </c>
-      <c r="K29" s="168">
-        <f>ROUND((E29+G29)*F29+H29+I29,0)</f>
-        <v/>
-      </c>
-      <c r="L29" s="169">
-        <f>J29-K29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="164" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="164" t="inlineStr">
-        <is>
-          <t>2026.04.21</t>
-        </is>
-      </c>
-      <c r="C30" s="165" t="inlineStr">
-        <is>
-          <t>Ferco</t>
-        </is>
-      </c>
-      <c r="D30" s="164" t="inlineStr">
-        <is>
-          <t>MONOPLEX20260126-01</t>
-        </is>
-      </c>
-      <c r="E30" s="166" t="n">
-        <v>25976</v>
-      </c>
-      <c r="F30" s="167" t="n">
-        <v>1473.3</v>
-      </c>
-      <c r="G30" s="164" t="n">
-        <v>20</v>
-      </c>
-      <c r="H30" s="168" t="n">
-        <v>12500</v>
-      </c>
-      <c r="I30" s="168" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J30" s="168" t="n">
-        <v>38320406</v>
-      </c>
-      <c r="K30" s="168">
-        <f>ROUND((E30+G30)*F30+H30+I30,0)</f>
-        <v/>
-      </c>
-      <c r="L30" s="169">
-        <f>J30-K30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="164" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="164" t="inlineStr">
-        <is>
-          <t>2026.04.22</t>
-        </is>
-      </c>
-      <c r="C31" s="165" t="inlineStr">
-        <is>
-          <t>Christie</t>
-        </is>
-      </c>
-      <c r="D31" s="164" t="inlineStr">
-        <is>
-          <t>CPO692(692-1, 692-2)</t>
-        </is>
-      </c>
-      <c r="E31" s="166" t="n">
-        <v>297580</v>
-      </c>
-      <c r="F31" s="167" t="n">
-        <v>1482.8</v>
-      </c>
-      <c r="G31" s="164" t="n">
-        <v>20</v>
-      </c>
-      <c r="H31" s="168" t="n">
-        <v>12500</v>
-      </c>
-      <c r="I31" s="168" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J31" s="168" t="n">
-        <v>441301780</v>
-      </c>
-      <c r="K31" s="168">
-        <f>ROUND((E31+G31)*F31+H31+I31,0)</f>
-        <v/>
-      </c>
-      <c r="L31" s="169">
-        <f>J31-K31</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="164" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="164" t="inlineStr">
-        <is>
-          <t>2026.04.22</t>
-        </is>
-      </c>
-      <c r="C32" s="165" t="inlineStr">
-        <is>
-          <t>Elicent (EUR)</t>
-        </is>
-      </c>
-      <c r="D32" s="164" t="inlineStr">
-        <is>
-          <t>EPO18</t>
-        </is>
-      </c>
-      <c r="E32" s="166" t="n">
-        <v>4388.4</v>
-      </c>
-      <c r="F32" s="167" t="n">
-        <v>1741.08</v>
-      </c>
-      <c r="G32" s="164" t="n">
-        <v>25</v>
-      </c>
-      <c r="H32" s="168" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I32" s="168" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J32" s="168" t="n">
+      <c r="J32" s="176" t="n">
         <v>7702082</v>
       </c>
-      <c r="K32" s="168">
+      <c r="K32" s="176">
         <f>ROUND((E32+G32)*F32+H32+I32,0)</f>
         <v/>
       </c>
-      <c r="L32" s="169">
+      <c r="L32" s="177">
         <f>J32-K32</f>
         <v/>
       </c>
@@ -12095,31 +12007,32 @@
       <c r="E35" s="44" t="n">
         <v>143557</v>
       </c>
-      <c r="F35" s="170">
-        <f>D30/E30</f>
-        <v/>
-      </c>
-      <c r="G35" s="119" t="n">
-        <v>1479.7</v>
+      <c r="F35" s="188">
+        <f>D35/E35</f>
+        <v/>
+      </c>
+      <c r="G35" s="44">
+        <f>F10</f>
+        <v/>
       </c>
       <c r="H35" s="9">
-        <f>ROUND(D30*G30,0)</f>
+        <f>ROUND(D35*G35,0)</f>
         <v/>
       </c>
       <c r="I35" s="9">
-        <f>ROUND(20*G30*F30,0)</f>
+        <f>ROUND(G10*F35*G35,0)</f>
         <v/>
       </c>
       <c r="J35" s="9">
-        <f>ROUND(H10*F30,0)</f>
+        <f>ROUND(H10*F35,0)</f>
         <v/>
       </c>
       <c r="K35" s="9">
-        <f>ROUND(I10*F30,0)</f>
+        <f>ROUND(I10*F35,0)</f>
         <v/>
       </c>
       <c r="L35" s="46">
-        <f>H30+I30+J30+K30</f>
+        <f>H35+I35+J35+K35</f>
         <v/>
       </c>
     </row>
@@ -12145,31 +12058,32 @@
       <c r="E36" s="44" t="n">
         <v>143557</v>
       </c>
-      <c r="F36" s="170">
-        <f>D31/E31</f>
-        <v/>
-      </c>
-      <c r="G36" s="119" t="n">
-        <v>1479.7</v>
+      <c r="F36" s="188">
+        <f>D36/E36</f>
+        <v/>
+      </c>
+      <c r="G36" s="44">
+        <f>F10</f>
+        <v/>
       </c>
       <c r="H36" s="9">
-        <f>ROUND(D31*G31,0)</f>
+        <f>ROUND(D36*G36,0)</f>
         <v/>
       </c>
       <c r="I36" s="9">
-        <f>ROUND(20*G31*F31,0)</f>
+        <f>ROUND(G10*F36*G36,0)</f>
         <v/>
       </c>
       <c r="J36" s="9">
-        <f>ROUND(H10*F31,0)</f>
+        <f>ROUND(H10*F36,0)</f>
         <v/>
       </c>
       <c r="K36" s="9">
-        <f>ROUND(I10*F31,0)</f>
+        <f>ROUND(I10*F36,0)</f>
         <v/>
       </c>
       <c r="L36" s="46">
-        <f>H31+I31+J31+K31</f>
+        <f>H36+I36+J36+K36</f>
         <v/>
       </c>
     </row>
@@ -12195,31 +12109,32 @@
       <c r="E37" s="44" t="n">
         <v>15040</v>
       </c>
-      <c r="F37" s="170">
-        <f>D32/E32</f>
-        <v/>
-      </c>
-      <c r="G37" s="119" t="n">
-        <v>1480</v>
+      <c r="F37" s="188">
+        <f>D37/E37</f>
+        <v/>
+      </c>
+      <c r="G37" s="44">
+        <f>F9</f>
+        <v/>
       </c>
       <c r="H37" s="9">
-        <f>ROUND(D32*G32,0)</f>
+        <f>ROUND(D37*G37,0)</f>
         <v/>
       </c>
       <c r="I37" s="9">
-        <f>ROUND(20*G32*F32,0)</f>
+        <f>ROUND(G9*F37*G37,0)</f>
         <v/>
       </c>
       <c r="J37" s="9">
-        <f>ROUND(H9*F32,0)</f>
+        <f>ROUND(H9*F37,0)</f>
         <v/>
       </c>
       <c r="K37" s="9">
-        <f>ROUND(I9*F32,0)</f>
+        <f>ROUND(I9*F37,0)</f>
         <v/>
       </c>
       <c r="L37" s="46">
-        <f>H32+I32+J32+K32</f>
+        <f>H37+I37+J37+K37</f>
         <v/>
       </c>
     </row>
@@ -12245,31 +12160,32 @@
       <c r="E38" s="44" t="n">
         <v>13860</v>
       </c>
-      <c r="F38" s="170">
-        <f>D33/E33</f>
-        <v/>
-      </c>
-      <c r="G38" s="119" t="n">
-        <v>1439.1</v>
+      <c r="F38" s="188">
+        <f>D38/E38</f>
+        <v/>
+      </c>
+      <c r="G38" s="44">
+        <f>F12</f>
+        <v/>
       </c>
       <c r="H38" s="9">
-        <f>ROUND(D33*G33,0)</f>
+        <f>ROUND(D38*G38,0)</f>
         <v/>
       </c>
       <c r="I38" s="9">
-        <f>ROUND(20*G33*F33,0)</f>
+        <f>ROUND(G12*F38*G38,0)</f>
         <v/>
       </c>
       <c r="J38" s="9">
-        <f>ROUND(H12*F33,0)</f>
+        <f>ROUND(H12*F38,0)</f>
         <v/>
       </c>
       <c r="K38" s="9">
-        <f>ROUND(I12*F33,0)</f>
+        <f>ROUND(I12*F38,0)</f>
         <v/>
       </c>
       <c r="L38" s="46">
-        <f>H33+I33+J33+K33</f>
+        <f>H38+I38+J38+K38</f>
         <v/>
       </c>
     </row>
@@ -12295,31 +12211,32 @@
       <c r="E39" s="44" t="n">
         <v>13860</v>
       </c>
-      <c r="F39" s="170">
-        <f>D34/E34</f>
-        <v/>
-      </c>
-      <c r="G39" s="119" t="n">
-        <v>1439.1</v>
+      <c r="F39" s="188">
+        <f>D39/E39</f>
+        <v/>
+      </c>
+      <c r="G39" s="44">
+        <f>F12</f>
+        <v/>
       </c>
       <c r="H39" s="9">
-        <f>ROUND(D34*G34,0)</f>
+        <f>ROUND(D39*G39,0)</f>
         <v/>
       </c>
       <c r="I39" s="9">
-        <f>ROUND(20*G34*F34,0)</f>
+        <f>ROUND(G12*F39*G39,0)</f>
         <v/>
       </c>
       <c r="J39" s="9">
-        <f>ROUND(H12*F34,0)</f>
+        <f>ROUND(H12*F39,0)</f>
         <v/>
       </c>
       <c r="K39" s="9">
-        <f>ROUND(I12*F34,0)</f>
+        <f>ROUND(I12*F39,0)</f>
         <v/>
       </c>
       <c r="L39" s="46">
-        <f>H34+I34+J34+K34</f>
+        <f>H39+I39+J39+K39</f>
         <v/>
       </c>
     </row>
@@ -12345,31 +12262,32 @@
       <c r="E40" s="44" t="n">
         <v>252</v>
       </c>
-      <c r="F40" s="170">
-        <f>D35/E35</f>
-        <v/>
-      </c>
-      <c r="G40" s="119" t="n">
-        <v>1479</v>
+      <c r="F40" s="188">
+        <f>D40/E40</f>
+        <v/>
+      </c>
+      <c r="G40" s="44">
+        <f>F14</f>
+        <v/>
       </c>
       <c r="H40" s="9">
-        <f>ROUND(D35*G35,0)</f>
+        <f>ROUND(D40*G40,0)</f>
         <v/>
       </c>
       <c r="I40" s="9">
-        <f>ROUND(20*G35*F35,0)</f>
+        <f>ROUND(G14*F40*G40,0)</f>
         <v/>
       </c>
       <c r="J40" s="9">
-        <f>ROUND(H14*F35,0)</f>
+        <f>ROUND(H14*F40,0)</f>
         <v/>
       </c>
       <c r="K40" s="9">
-        <f>ROUND(I14*F35,0)</f>
+        <f>ROUND(I14*F40,0)</f>
         <v/>
       </c>
       <c r="L40" s="46">
-        <f>H35+I35+J35+K35</f>
+        <f>H40+I40+J40+K40</f>
         <v/>
       </c>
     </row>
@@ -12395,31 +12313,32 @@
       <c r="E41" s="44" t="n">
         <v>3700</v>
       </c>
-      <c r="F41" s="170">
-        <f>D36/E36</f>
-        <v/>
-      </c>
-      <c r="G41" s="119" t="n">
-        <v>1475.7</v>
+      <c r="F41" s="188">
+        <f>D41/E41</f>
+        <v/>
+      </c>
+      <c r="G41" s="44">
+        <f>F15</f>
+        <v/>
       </c>
       <c r="H41" s="9">
-        <f>ROUND(D36*G36,0)</f>
+        <f>ROUND(D41*G41,0)</f>
         <v/>
       </c>
       <c r="I41" s="9">
-        <f>ROUND(20*G36*F36,0)</f>
+        <f>ROUND(G15*F41*G41,0)</f>
         <v/>
       </c>
       <c r="J41" s="9">
-        <f>ROUND(H15*F36,0)</f>
+        <f>ROUND(H15*F41,0)</f>
         <v/>
       </c>
       <c r="K41" s="9">
-        <f>ROUND(I15*F36,0)</f>
+        <f>ROUND(I15*F41,0)</f>
         <v/>
       </c>
       <c r="L41" s="46">
-        <f>H36+I36+J36+K36</f>
+        <f>H41+I41+J41+K41</f>
         <v/>
       </c>
     </row>
@@ -12445,31 +12364,32 @@
       <c r="E42" s="44" t="n">
         <v>3700</v>
       </c>
-      <c r="F42" s="170">
-        <f>D37/E37</f>
-        <v/>
-      </c>
-      <c r="G42" s="119" t="n">
-        <v>1475.7</v>
+      <c r="F42" s="188">
+        <f>D42/E42</f>
+        <v/>
+      </c>
+      <c r="G42" s="44">
+        <f>F15</f>
+        <v/>
       </c>
       <c r="H42" s="9">
-        <f>ROUND(D37*G37,0)</f>
+        <f>ROUND(D42*G42,0)</f>
         <v/>
       </c>
       <c r="I42" s="9">
-        <f>ROUND(20*G37*F37,0)</f>
+        <f>ROUND(G15*F42*G42,0)</f>
         <v/>
       </c>
       <c r="J42" s="9">
-        <f>ROUND(H15*F37,0)</f>
+        <f>ROUND(H15*F42,0)</f>
         <v/>
       </c>
       <c r="K42" s="9">
-        <f>ROUND(I15*F37,0)</f>
+        <f>ROUND(I15*F42,0)</f>
         <v/>
       </c>
       <c r="L42" s="46">
-        <f>H37+I37+J37+K37</f>
+        <f>H42+I42+J42+K42</f>
         <v/>
       </c>
     </row>
@@ -12495,31 +12415,32 @@
       <c r="E43" s="44" t="n">
         <v>3700</v>
       </c>
-      <c r="F43" s="170">
-        <f>D38/E38</f>
-        <v/>
-      </c>
-      <c r="G43" s="119" t="n">
-        <v>1475.7</v>
+      <c r="F43" s="188">
+        <f>D43/E43</f>
+        <v/>
+      </c>
+      <c r="G43" s="44">
+        <f>F15</f>
+        <v/>
       </c>
       <c r="H43" s="9">
-        <f>ROUND(D38*G38,0)</f>
+        <f>ROUND(D43*G43,0)</f>
         <v/>
       </c>
       <c r="I43" s="9">
-        <f>ROUND(20*G38*F38,0)</f>
+        <f>ROUND(G15*F43*G43,0)</f>
         <v/>
       </c>
       <c r="J43" s="9">
-        <f>ROUND(H15*F38,0)</f>
+        <f>ROUND(H15*F43,0)</f>
         <v/>
       </c>
       <c r="K43" s="9">
-        <f>ROUND(I15*F38,0)</f>
+        <f>ROUND(I15*F43,0)</f>
         <v/>
       </c>
       <c r="L43" s="46">
-        <f>H38+I38+J38+K38</f>
+        <f>H43+I43+J43+K43</f>
         <v/>
       </c>
     </row>
@@ -12545,31 +12466,32 @@
       <c r="E44" s="44" t="n">
         <v>9626.35</v>
       </c>
-      <c r="F44" s="170">
-        <f>D39/E39</f>
-        <v/>
-      </c>
-      <c r="G44" s="119" t="n">
-        <v>1476</v>
+      <c r="F44" s="188">
+        <f>D44/E44</f>
+        <v/>
+      </c>
+      <c r="G44" s="44">
+        <f>F16</f>
+        <v/>
       </c>
       <c r="H44" s="9">
-        <f>ROUND(D39*G39,0)</f>
+        <f>ROUND(D44*G44,0)</f>
         <v/>
       </c>
       <c r="I44" s="9">
-        <f>ROUND(20*G39*F39,0)</f>
+        <f>ROUND(G16*F44*G44,0)</f>
         <v/>
       </c>
       <c r="J44" s="9">
-        <f>ROUND(H16*F39,0)</f>
+        <f>ROUND(H16*F44,0)</f>
         <v/>
       </c>
       <c r="K44" s="9">
-        <f>ROUND(I16*F39,0)</f>
+        <f>ROUND(I16*F44,0)</f>
         <v/>
       </c>
       <c r="L44" s="46">
-        <f>H39+I39+J39+K39</f>
+        <f>H44+I44+J44+K44</f>
         <v/>
       </c>
     </row>
@@ -12595,31 +12517,32 @@
       <c r="E45" s="44" t="n">
         <v>5056.8</v>
       </c>
-      <c r="F45" s="170">
-        <f>D40/E40</f>
-        <v/>
-      </c>
-      <c r="G45" s="119" t="n">
-        <v>1445.5</v>
+      <c r="F45" s="188">
+        <f>D45/E45</f>
+        <v/>
+      </c>
+      <c r="G45" s="44">
+        <f>F17</f>
+        <v/>
       </c>
       <c r="H45" s="9">
-        <f>ROUND(D40*G40,0)</f>
+        <f>ROUND(D45*G45,0)</f>
         <v/>
       </c>
       <c r="I45" s="9">
-        <f>ROUND(20*G40*F40,0)</f>
+        <f>ROUND(G17*F45*G45,0)</f>
         <v/>
       </c>
       <c r="J45" s="9">
-        <f>ROUND(H17*F40,0)</f>
+        <f>ROUND(H17*F45,0)</f>
         <v/>
       </c>
       <c r="K45" s="9">
-        <f>ROUND(I17*F40,0)</f>
+        <f>ROUND(I17*F45,0)</f>
         <v/>
       </c>
       <c r="L45" s="46">
-        <f>H40+I40+J40+K40</f>
+        <f>H45+I45+J45+K45</f>
         <v/>
       </c>
     </row>
@@ -12645,31 +12568,32 @@
       <c r="E46" s="44" t="n">
         <v>24794</v>
       </c>
-      <c r="F46" s="170">
-        <f>D41/E41</f>
-        <v/>
-      </c>
-      <c r="G46" s="119" t="n">
-        <v>1454.7</v>
+      <c r="F46" s="188">
+        <f>D46/E46</f>
+        <v/>
+      </c>
+      <c r="G46" s="44">
+        <f>F19</f>
+        <v/>
       </c>
       <c r="H46" s="9">
-        <f>ROUND(D41*G41,0)</f>
+        <f>ROUND(D46*G46,0)</f>
         <v/>
       </c>
       <c r="I46" s="9">
-        <f>ROUND(20*G41*F41,0)</f>
+        <f>ROUND(G19*F46*G46,0)</f>
         <v/>
       </c>
       <c r="J46" s="9">
-        <f>ROUND(H19*F41,0)</f>
+        <f>ROUND(H19*F46,0)</f>
         <v/>
       </c>
       <c r="K46" s="9">
-        <f>ROUND(I19*F41,0)</f>
+        <f>ROUND(I19*F46,0)</f>
         <v/>
       </c>
       <c r="L46" s="46">
-        <f>H41+I41+J41+K41</f>
+        <f>H46+I46+J46+K46</f>
         <v/>
       </c>
     </row>
@@ -12695,31 +12619,32 @@
       <c r="E47" s="44" t="n">
         <v>24794</v>
       </c>
-      <c r="F47" s="170">
-        <f>D42/E42</f>
-        <v/>
-      </c>
-      <c r="G47" s="119" t="n">
-        <v>1454.7</v>
+      <c r="F47" s="188">
+        <f>D47/E47</f>
+        <v/>
+      </c>
+      <c r="G47" s="44">
+        <f>F19</f>
+        <v/>
       </c>
       <c r="H47" s="9">
-        <f>ROUND(D42*G42,0)</f>
+        <f>ROUND(D47*G47,0)</f>
         <v/>
       </c>
       <c r="I47" s="9">
-        <f>ROUND(20*G42*F42,0)</f>
+        <f>ROUND(G19*F47*G47,0)</f>
         <v/>
       </c>
       <c r="J47" s="9">
-        <f>ROUND(H19*F42,0)</f>
+        <f>ROUND(H19*F47,0)</f>
         <v/>
       </c>
       <c r="K47" s="9">
-        <f>ROUND(I19*F42,0)</f>
+        <f>ROUND(I19*F47,0)</f>
         <v/>
       </c>
       <c r="L47" s="46">
-        <f>H42+I42+J42+K42</f>
+        <f>H47+I47+J47+K47</f>
         <v/>
       </c>
     </row>
@@ -12745,31 +12670,32 @@
       <c r="E48" s="44" t="n">
         <v>11599.57</v>
       </c>
-      <c r="F48" s="170">
-        <f>D43/E43</f>
-        <v/>
-      </c>
-      <c r="G48" s="119" t="n">
-        <v>1453.6</v>
+      <c r="F48" s="188">
+        <f>D48/E48</f>
+        <v/>
+      </c>
+      <c r="G48" s="44">
+        <f>F20</f>
+        <v/>
       </c>
       <c r="H48" s="9">
-        <f>ROUND(D43*G43,0)</f>
+        <f>ROUND(D48*G48,0)</f>
         <v/>
       </c>
       <c r="I48" s="9">
-        <f>ROUND(20*G43*F43,0)</f>
+        <f>ROUND(G20*F48*G48,0)</f>
         <v/>
       </c>
       <c r="J48" s="9">
-        <f>ROUND(H20*F43,0)</f>
+        <f>ROUND(H20*F48,0)</f>
         <v/>
       </c>
       <c r="K48" s="9">
-        <f>ROUND(I20*F43,0)</f>
+        <f>ROUND(I20*F48,0)</f>
         <v/>
       </c>
       <c r="L48" s="46">
-        <f>H43+I43+J43+K43</f>
+        <f>H48+I48+J48+K48</f>
         <v/>
       </c>
     </row>
@@ -12795,31 +12721,32 @@
       <c r="E49" s="44" t="n">
         <v>11599.57</v>
       </c>
-      <c r="F49" s="170">
-        <f>D44/E44</f>
-        <v/>
-      </c>
-      <c r="G49" s="119" t="n">
-        <v>1453.6</v>
+      <c r="F49" s="188">
+        <f>D49/E49</f>
+        <v/>
+      </c>
+      <c r="G49" s="44">
+        <f>F20</f>
+        <v/>
       </c>
       <c r="H49" s="9">
-        <f>ROUND(D44*G44,0)</f>
+        <f>ROUND(D49*G49,0)</f>
         <v/>
       </c>
       <c r="I49" s="9">
-        <f>ROUND(20*G44*F44,0)</f>
+        <f>ROUND(G20*F49*G49,0)</f>
         <v/>
       </c>
       <c r="J49" s="9">
-        <f>ROUND(H20*F44,0)</f>
+        <f>ROUND(H20*F49,0)</f>
         <v/>
       </c>
       <c r="K49" s="9">
-        <f>ROUND(I20*F44,0)</f>
+        <f>ROUND(I20*F49,0)</f>
         <v/>
       </c>
       <c r="L49" s="46">
-        <f>H44+I44+J44+K44</f>
+        <f>H49+I49+J49+K49</f>
         <v/>
       </c>
     </row>
@@ -12845,31 +12772,32 @@
       <c r="E50" s="44" t="n">
         <v>11599.57</v>
       </c>
-      <c r="F50" s="170">
-        <f>D45/E45</f>
-        <v/>
-      </c>
-      <c r="G50" s="119" t="n">
-        <v>1453.6</v>
+      <c r="F50" s="188">
+        <f>D50/E50</f>
+        <v/>
+      </c>
+      <c r="G50" s="44">
+        <f>F20</f>
+        <v/>
       </c>
       <c r="H50" s="9">
-        <f>ROUND(D45*G45,0)</f>
+        <f>ROUND(D50*G50,0)</f>
         <v/>
       </c>
       <c r="I50" s="9">
-        <f>ROUND(20*G45*F45,0)</f>
+        <f>ROUND(G20*F50*G50,0)</f>
         <v/>
       </c>
       <c r="J50" s="9">
-        <f>ROUND(H20*F45,0)</f>
+        <f>ROUND(H20*F50,0)</f>
         <v/>
       </c>
       <c r="K50" s="9">
-        <f>ROUND(I20*F45,0)</f>
+        <f>ROUND(I20*F50,0)</f>
         <v/>
       </c>
       <c r="L50" s="46">
-        <f>H45+I45+J45+K45</f>
+        <f>H50+I50+J50+K50</f>
         <v/>
       </c>
     </row>
@@ -12895,31 +12823,32 @@
       <c r="E51" s="44" t="n">
         <v>26358</v>
       </c>
-      <c r="F51" s="170">
-        <f>D46/E46</f>
-        <v/>
-      </c>
-      <c r="G51" s="119" t="n">
-        <v>1460.7</v>
+      <c r="F51" s="188">
+        <f>D51/E51</f>
+        <v/>
+      </c>
+      <c r="G51" s="44">
+        <f>F21</f>
+        <v/>
       </c>
       <c r="H51" s="9">
-        <f>ROUND(D46*G46,0)</f>
+        <f>ROUND(D51*G51,0)</f>
         <v/>
       </c>
       <c r="I51" s="9">
-        <f>ROUND(20*G46*F46,0)</f>
+        <f>ROUND(G21*F51*G51,0)</f>
         <v/>
       </c>
       <c r="J51" s="9">
-        <f>ROUND(H21*F46,0)</f>
+        <f>ROUND(H21*F51,0)</f>
         <v/>
       </c>
       <c r="K51" s="9">
-        <f>ROUND(I21*F46,0)</f>
+        <f>ROUND(I21*F51,0)</f>
         <v/>
       </c>
       <c r="L51" s="46">
-        <f>H46+I46+J46+K46</f>
+        <f>H51+I51+J51+K51</f>
         <v/>
       </c>
     </row>
@@ -12945,31 +12874,32 @@
       <c r="E52" s="44" t="n">
         <v>17538</v>
       </c>
-      <c r="F52" s="170">
-        <f>D47/E47</f>
-        <v/>
-      </c>
-      <c r="G52" s="119" t="n">
-        <v>1451.7</v>
+      <c r="F52" s="188">
+        <f>D52/E52</f>
+        <v/>
+      </c>
+      <c r="G52" s="44">
+        <f>F22</f>
+        <v/>
       </c>
       <c r="H52" s="9">
-        <f>ROUND(D47*G47,0)</f>
+        <f>ROUND(D52*G52,0)</f>
         <v/>
       </c>
       <c r="I52" s="9">
-        <f>ROUND(20*G47*F47,0)</f>
+        <f>ROUND(G22*F52*G52,0)</f>
         <v/>
       </c>
       <c r="J52" s="9">
-        <f>ROUND(H22*F47,0)</f>
+        <f>ROUND(H22*F52,0)</f>
         <v/>
       </c>
       <c r="K52" s="9">
-        <f>ROUND(I22*F47,0)</f>
+        <f>ROUND(I22*F52,0)</f>
         <v/>
       </c>
       <c r="L52" s="46">
-        <f>H47+I47+J47+K47</f>
+        <f>H52+I52+J52+K52</f>
         <v/>
       </c>
     </row>
@@ -12995,30 +12925,34 @@
       <c r="E53" s="44" t="n">
         <v>17538</v>
       </c>
-      <c r="F53" s="170">
-        <f>D48/E48</f>
-        <v/>
-      </c>
-      <c r="G53" s="119" t="n">
-        <v>1451.7</v>
+      <c r="F53" s="188">
+        <f>D53/E53</f>
+        <v/>
+      </c>
+      <c r="G53" s="44">
+        <f>F22</f>
+        <v/>
       </c>
       <c r="H53" s="9">
-        <f>ROUND(D48*G48,0)</f>
+        <f>ROUND(D53*G53,0)</f>
         <v/>
       </c>
       <c r="I53" s="9">
-        <f>ROUND(20*G48*F48,0)</f>
+        <f>ROUND(G22*F53*G53,0)</f>
         <v/>
       </c>
       <c r="J53" s="9">
-        <f>ROUND(H22*F48,0)</f>
+        <f>ROUND(H22*F53,0)</f>
         <v/>
       </c>
       <c r="K53" s="9">
-        <f>ROUND(I22*F48,0)</f>
-        <v/>
-      </c>
-      <c r="L53" s="46" t="n"/>
+        <f>ROUND(I22*F53,0)</f>
+        <v/>
+      </c>
+      <c r="L53" s="46">
+        <f>H53+I53+J53+K53</f>
+        <v/>
+      </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="3" t="inlineStr">
@@ -13042,31 +12976,32 @@
       <c r="E54" s="44" t="n">
         <v>142189</v>
       </c>
-      <c r="F54" s="170">
-        <f>D49/E49</f>
-        <v/>
-      </c>
-      <c r="G54" s="119" t="n">
-        <v>1441.6</v>
+      <c r="F54" s="188">
+        <f>D54/E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="44">
+        <f>F23</f>
+        <v/>
       </c>
       <c r="H54" s="9">
-        <f>ROUND(D49*G49,0)</f>
+        <f>ROUND(D54*G54,0)</f>
         <v/>
       </c>
       <c r="I54" s="9">
-        <f>ROUND(20*G49*F49,0)</f>
+        <f>ROUND(G23*F54*G54,0)</f>
         <v/>
       </c>
       <c r="J54" s="9">
-        <f>ROUND(H23*F49,0)</f>
+        <f>ROUND(H23*F54,0)</f>
         <v/>
       </c>
       <c r="K54" s="9">
-        <f>ROUND(I23*F49,0)</f>
+        <f>ROUND(I23*F54,0)</f>
         <v/>
       </c>
       <c r="L54" s="46">
-        <f>H49+I49+J49+K49</f>
+        <f>H54+I54+J54+K54</f>
         <v/>
       </c>
     </row>
@@ -13092,31 +13027,32 @@
       <c r="E55" s="44" t="n">
         <v>142189</v>
       </c>
-      <c r="F55" s="170">
-        <f>D50/E50</f>
-        <v/>
-      </c>
-      <c r="G55" s="119" t="n">
-        <v>1441.6</v>
+      <c r="F55" s="188">
+        <f>D55/E55</f>
+        <v/>
+      </c>
+      <c r="G55" s="44">
+        <f>F23</f>
+        <v/>
       </c>
       <c r="H55" s="9">
-        <f>ROUND(D50*G50,0)</f>
+        <f>ROUND(D55*G55,0)</f>
         <v/>
       </c>
       <c r="I55" s="9">
-        <f>ROUND(20*G50*F50,0)</f>
+        <f>ROUND(G23*F55*G55,0)</f>
         <v/>
       </c>
       <c r="J55" s="9">
-        <f>ROUND(H23*F50,0)</f>
+        <f>ROUND(H23*F55,0)</f>
         <v/>
       </c>
       <c r="K55" s="9">
-        <f>ROUND(I23*F50,0)</f>
+        <f>ROUND(I23*F55,0)</f>
         <v/>
       </c>
       <c r="L55" s="46">
-        <f>H50+I50+J50+K50</f>
+        <f>H55+I55+J55+K55</f>
         <v/>
       </c>
     </row>
@@ -13142,31 +13078,32 @@
       <c r="E56" s="44" t="n">
         <v>137850</v>
       </c>
-      <c r="F56" s="170">
-        <f>D51/E51</f>
-        <v/>
-      </c>
-      <c r="G56" s="119" t="n">
-        <v>1477.6</v>
+      <c r="F56" s="188">
+        <f>D56/E56</f>
+        <v/>
+      </c>
+      <c r="G56" s="44">
+        <f>F24</f>
+        <v/>
       </c>
       <c r="H56" s="9">
-        <f>ROUND(D51*G51,0)</f>
+        <f>ROUND(D56*G56,0)</f>
         <v/>
       </c>
       <c r="I56" s="9">
-        <f>ROUND(20*G51*F51,0)</f>
+        <f>ROUND(G24*F56*G56,0)</f>
         <v/>
       </c>
       <c r="J56" s="9">
-        <f>ROUND(H24*F51,0)</f>
+        <f>ROUND(H24*F56,0)</f>
         <v/>
       </c>
       <c r="K56" s="9">
-        <f>ROUND(I24*F51,0)</f>
+        <f>ROUND(I24*F56,0)</f>
         <v/>
       </c>
       <c r="L56" s="46">
-        <f>H51+I51+J51+K51</f>
+        <f>H56+I56+J56+K56</f>
         <v/>
       </c>
     </row>
@@ -13192,31 +13129,32 @@
       <c r="E57" s="44" t="n">
         <v>34354</v>
       </c>
-      <c r="F57" s="170">
-        <f>D52/E52</f>
-        <v/>
-      </c>
-      <c r="G57" s="119" t="n">
-        <v>1505.7</v>
+      <c r="F57" s="188">
+        <f>D57/E57</f>
+        <v/>
+      </c>
+      <c r="G57" s="44">
+        <f>F25</f>
+        <v/>
       </c>
       <c r="H57" s="9">
-        <f>ROUND(D52*G52,0)</f>
+        <f>ROUND(D57*G57,0)</f>
         <v/>
       </c>
       <c r="I57" s="9">
-        <f>ROUND(20*G52*F52,0)</f>
+        <f>ROUND(G25*F57*G57,0)</f>
         <v/>
       </c>
       <c r="J57" s="9">
-        <f>ROUND(H25*F52,0)</f>
+        <f>ROUND(H25*F57,0)</f>
         <v/>
       </c>
       <c r="K57" s="9">
-        <f>ROUND(I25*F52,0)</f>
+        <f>ROUND(I25*F57,0)</f>
         <v/>
       </c>
       <c r="L57" s="46">
-        <f>H52+I52+J52+K52</f>
+        <f>H57+I57+J57+K57</f>
         <v/>
       </c>
     </row>
@@ -13242,31 +13180,32 @@
       <c r="E58" s="44" t="n">
         <v>34354</v>
       </c>
-      <c r="F58" s="170">
-        <f>D53/E53</f>
-        <v/>
-      </c>
-      <c r="G58" s="119" t="n">
-        <v>1505.7</v>
+      <c r="F58" s="188">
+        <f>D58/E58</f>
+        <v/>
+      </c>
+      <c r="G58" s="44">
+        <f>F25</f>
+        <v/>
       </c>
       <c r="H58" s="9">
-        <f>ROUND(D53*G53,0)</f>
+        <f>ROUND(D58*G58,0)</f>
         <v/>
       </c>
       <c r="I58" s="9">
-        <f>ROUND(20*G53*F53,0)</f>
+        <f>ROUND(G25*F58*G58,0)</f>
         <v/>
       </c>
       <c r="J58" s="9">
-        <f>ROUND(H25*F53,0)</f>
+        <f>ROUND(H25*F58,0)</f>
         <v/>
       </c>
       <c r="K58" s="9">
-        <f>ROUND(I25*F53,0)</f>
+        <f>ROUND(I25*F58,0)</f>
         <v/>
       </c>
       <c r="L58" s="46">
-        <f>H53+I53+J53+K53</f>
+        <f>H58+I58+J58+K58</f>
         <v/>
       </c>
     </row>
@@ -13292,31 +13231,32 @@
       <c r="E59" s="44" t="n">
         <v>6553.05</v>
       </c>
-      <c r="F59" s="170">
-        <f>D54/E54</f>
-        <v/>
-      </c>
-      <c r="G59" s="119" t="n">
-        <v>1506.4</v>
+      <c r="F59" s="188">
+        <f>D59/E59</f>
+        <v/>
+      </c>
+      <c r="G59" s="44">
+        <f>F26</f>
+        <v/>
       </c>
       <c r="H59" s="9">
-        <f>ROUND(D54*G54,0)</f>
+        <f>ROUND(D59*G59,0)</f>
         <v/>
       </c>
       <c r="I59" s="9">
-        <f>ROUND(20*G54*F54,0)</f>
+        <f>ROUND(G26*F59*G59,0)</f>
         <v/>
       </c>
       <c r="J59" s="9">
-        <f>ROUND(H26*F54,0)</f>
+        <f>ROUND(H26*F59,0)</f>
         <v/>
       </c>
       <c r="K59" s="9">
-        <f>ROUND(I26*F54,0)</f>
+        <f>ROUND(I26*F59,0)</f>
         <v/>
       </c>
       <c r="L59" s="46">
-        <f>H54+I54+J54+K54</f>
+        <f>H59+I59+J59+K59</f>
         <v/>
       </c>
     </row>
@@ -13342,31 +13282,32 @@
       <c r="E60" s="44" t="n">
         <v>6553.05</v>
       </c>
-      <c r="F60" s="170">
-        <f>D55/E55</f>
-        <v/>
-      </c>
-      <c r="G60" s="119" t="n">
-        <v>1506.4</v>
+      <c r="F60" s="188">
+        <f>D60/E60</f>
+        <v/>
+      </c>
+      <c r="G60" s="44">
+        <f>F26</f>
+        <v/>
       </c>
       <c r="H60" s="9">
-        <f>ROUND(D55*G55,0)</f>
+        <f>ROUND(D60*G60,0)</f>
         <v/>
       </c>
       <c r="I60" s="9">
-        <f>ROUND(20*G55*F55,0)</f>
+        <f>ROUND(G26*F60*G60,0)</f>
         <v/>
       </c>
       <c r="J60" s="9">
-        <f>ROUND(H26*F55,0)</f>
+        <f>ROUND(H26*F60,0)</f>
         <v/>
       </c>
       <c r="K60" s="9">
-        <f>ROUND(I26*F55,0)</f>
+        <f>ROUND(I26*F60,0)</f>
         <v/>
       </c>
       <c r="L60" s="46">
-        <f>H55+I55+J55+K55</f>
+        <f>H60+I60+J60+K60</f>
         <v/>
       </c>
     </row>
@@ -13392,31 +13333,32 @@
       <c r="E61" s="44" t="n">
         <v>6553.05</v>
       </c>
-      <c r="F61" s="170">
-        <f>D56/E56</f>
-        <v/>
-      </c>
-      <c r="G61" s="119" t="n">
-        <v>1506.4</v>
+      <c r="F61" s="188">
+        <f>D61/E61</f>
+        <v/>
+      </c>
+      <c r="G61" s="44">
+        <f>F26</f>
+        <v/>
       </c>
       <c r="H61" s="9">
-        <f>ROUND(D56*G56,0)</f>
+        <f>ROUND(D61*G61,0)</f>
         <v/>
       </c>
       <c r="I61" s="9">
-        <f>ROUND(20*G56*F56,0)</f>
+        <f>ROUND(G26*F61*G61,0)</f>
         <v/>
       </c>
       <c r="J61" s="9">
-        <f>ROUND(H26*F56,0)</f>
+        <f>ROUND(H26*F61,0)</f>
         <v/>
       </c>
       <c r="K61" s="9">
-        <f>ROUND(I26*F56,0)</f>
+        <f>ROUND(I26*F61,0)</f>
         <v/>
       </c>
       <c r="L61" s="46">
-        <f>H56+I56+J56+K56</f>
+        <f>H61+I61+J61+K61</f>
         <v/>
       </c>
     </row>
@@ -13442,31 +13384,32 @@
       <c r="E62" s="44" t="n">
         <v>6553.05</v>
       </c>
-      <c r="F62" s="170">
-        <f>D57/E57</f>
-        <v/>
-      </c>
-      <c r="G62" s="119" t="n">
-        <v>1506.4</v>
+      <c r="F62" s="188">
+        <f>D62/E62</f>
+        <v/>
+      </c>
+      <c r="G62" s="44">
+        <f>F26</f>
+        <v/>
       </c>
       <c r="H62" s="9">
-        <f>ROUND(D57*G57,0)</f>
+        <f>ROUND(D62*G62,0)</f>
         <v/>
       </c>
       <c r="I62" s="9">
-        <f>ROUND(20*G57*F57,0)</f>
+        <f>ROUND(G26*F62*G62,0)</f>
         <v/>
       </c>
       <c r="J62" s="9">
-        <f>ROUND(H26*F57,0)</f>
+        <f>ROUND(H26*F62,0)</f>
         <v/>
       </c>
       <c r="K62" s="9">
-        <f>ROUND(I26*F57,0)</f>
+        <f>ROUND(I26*F62,0)</f>
         <v/>
       </c>
       <c r="L62" s="46">
-        <f>H57+I57+J57+K57</f>
+        <f>H62+I62+J62+K62</f>
         <v/>
       </c>
     </row>
@@ -13492,31 +13435,32 @@
       <c r="E63" s="44" t="n">
         <v>57650</v>
       </c>
-      <c r="F63" s="170">
-        <f>D58/E58</f>
-        <v/>
-      </c>
-      <c r="G63" s="119" t="n">
-        <v>1481.9</v>
+      <c r="F63" s="188">
+        <f>D63/E63</f>
+        <v/>
+      </c>
+      <c r="G63" s="44">
+        <f>F27</f>
+        <v/>
       </c>
       <c r="H63" s="9">
-        <f>ROUND(D58*G58,0)</f>
+        <f>ROUND(D63*G63,0)</f>
         <v/>
       </c>
       <c r="I63" s="9">
-        <f>ROUND(20*G58*F58,0)</f>
+        <f>ROUND(G27*F63*G63,0)</f>
         <v/>
       </c>
       <c r="J63" s="9">
-        <f>ROUND(H27*F58,0)</f>
+        <f>ROUND(H27*F63,0)</f>
         <v/>
       </c>
       <c r="K63" s="9">
-        <f>ROUND(I27*F58,0)</f>
+        <f>ROUND(I27*F63,0)</f>
         <v/>
       </c>
       <c r="L63" s="46">
-        <f>H58+I58+J58+K58</f>
+        <f>H63+I63+J63+K63</f>
         <v/>
       </c>
     </row>
@@ -13542,31 +13486,32 @@
       <c r="E64" s="44" t="n">
         <v>57650</v>
       </c>
-      <c r="F64" s="170">
-        <f>D59/E59</f>
-        <v/>
-      </c>
-      <c r="G64" s="119" t="n">
-        <v>1481.9</v>
+      <c r="F64" s="188">
+        <f>D64/E64</f>
+        <v/>
+      </c>
+      <c r="G64" s="44">
+        <f>F27</f>
+        <v/>
       </c>
       <c r="H64" s="9">
-        <f>ROUND(D59*G59,0)</f>
+        <f>ROUND(D64*G64,0)</f>
         <v/>
       </c>
       <c r="I64" s="9">
-        <f>ROUND(20*G59*F59,0)</f>
+        <f>ROUND(G27*F64*G64,0)</f>
         <v/>
       </c>
       <c r="J64" s="9">
-        <f>ROUND(H27*F59,0)</f>
+        <f>ROUND(H27*F64,0)</f>
         <v/>
       </c>
       <c r="K64" s="9">
-        <f>ROUND(I27*F59,0)</f>
+        <f>ROUND(I27*F64,0)</f>
         <v/>
       </c>
       <c r="L64" s="46">
-        <f>H59+I59+J59+K59</f>
+        <f>H64+I64+J64+K64</f>
         <v/>
       </c>
     </row>
@@ -13592,31 +13537,32 @@
       <c r="E65" s="44" t="n">
         <v>57650</v>
       </c>
-      <c r="F65" s="170">
-        <f>D60/E60</f>
-        <v/>
-      </c>
-      <c r="G65" s="119" t="n">
-        <v>1481.9</v>
+      <c r="F65" s="188">
+        <f>D65/E65</f>
+        <v/>
+      </c>
+      <c r="G65" s="44">
+        <f>F27</f>
+        <v/>
       </c>
       <c r="H65" s="9">
-        <f>ROUND(D60*G60,0)</f>
+        <f>ROUND(D65*G65,0)</f>
         <v/>
       </c>
       <c r="I65" s="9">
-        <f>ROUND(20*G60*F60,0)</f>
+        <f>ROUND(G27*F65*G65,0)</f>
         <v/>
       </c>
       <c r="J65" s="9">
-        <f>ROUND(H27*F60,0)</f>
+        <f>ROUND(H27*F65,0)</f>
         <v/>
       </c>
       <c r="K65" s="9">
-        <f>ROUND(I27*F60,0)</f>
+        <f>ROUND(I27*F65,0)</f>
         <v/>
       </c>
       <c r="L65" s="46">
-        <f>H60+I60+J60+K60</f>
+        <f>H65+I65+J65+K65</f>
         <v/>
       </c>
     </row>
@@ -13642,26 +13588,33 @@
       <c r="E66" s="173" t="n">
         <v>297580</v>
       </c>
-      <c r="F66" s="174" t="n">
-        <v>0.03696484978829222</v>
-      </c>
-      <c r="G66" s="175" t="n">
-        <v>1482.8</v>
-      </c>
-      <c r="H66" s="176" t="n">
-        <v>16310800</v>
-      </c>
-      <c r="I66" s="176" t="n">
-        <v>1096</v>
-      </c>
-      <c r="J66" s="176" t="n">
-        <v>462</v>
-      </c>
-      <c r="K66" s="176" t="n">
-        <v>296</v>
-      </c>
-      <c r="L66" s="177" t="n">
-        <v>16312654</v>
+      <c r="F66" s="189">
+        <f>D66/E66</f>
+        <v/>
+      </c>
+      <c r="G66" s="173">
+        <f>F31</f>
+        <v/>
+      </c>
+      <c r="H66" s="176">
+        <f>ROUND(D66*G66,0)</f>
+        <v/>
+      </c>
+      <c r="I66" s="176">
+        <f>ROUND(G31*F66*G66,0)</f>
+        <v/>
+      </c>
+      <c r="J66" s="176">
+        <f>ROUND(H31*F66,0)</f>
+        <v/>
+      </c>
+      <c r="K66" s="176">
+        <f>ROUND(I31*F66,0)</f>
+        <v/>
+      </c>
+      <c r="L66" s="177">
+        <f>H66+I66+J66+K66</f>
+        <v/>
       </c>
     </row>
     <row r="67">
@@ -13686,26 +13639,33 @@
       <c r="E67" s="173" t="n">
         <v>297580</v>
       </c>
-      <c r="F67" s="174" t="n">
-        <v>0.9630351502117078</v>
-      </c>
-      <c r="G67" s="175" t="n">
-        <v>1482.8</v>
-      </c>
-      <c r="H67" s="176" t="n">
-        <v>424990980</v>
-      </c>
-      <c r="I67" s="176" t="n">
-        <v>28560</v>
-      </c>
-      <c r="J67" s="176" t="n">
-        <v>12038</v>
-      </c>
-      <c r="K67" s="176" t="n">
-        <v>7704</v>
-      </c>
-      <c r="L67" s="177" t="n">
-        <v>425039282</v>
+      <c r="F67" s="189">
+        <f>D67/E67</f>
+        <v/>
+      </c>
+      <c r="G67" s="173">
+        <f>F31</f>
+        <v/>
+      </c>
+      <c r="H67" s="176">
+        <f>ROUND(D67*G67,0)</f>
+        <v/>
+      </c>
+      <c r="I67" s="176">
+        <f>ROUND(G31*F67*G67,0)</f>
+        <v/>
+      </c>
+      <c r="J67" s="176">
+        <f>ROUND(H31*F67,0)</f>
+        <v/>
+      </c>
+      <c r="K67" s="176">
+        <f>ROUND(I31*F67,0)</f>
+        <v/>
+      </c>
+      <c r="L67" s="177">
+        <f>H67+I67+J67+K67</f>
+        <v/>
       </c>
     </row>
     <row r="68">
@@ -13730,26 +13690,33 @@
       <c r="E68" s="173" t="n">
         <v>4388.4</v>
       </c>
-      <c r="F68" s="174" t="n">
-        <v>1</v>
-      </c>
-      <c r="G68" s="175" t="n">
-        <v>1741.08</v>
-      </c>
-      <c r="H68" s="176" t="n">
-        <v>7702082</v>
-      </c>
-      <c r="I68" s="176" t="n">
-        <v>43527</v>
-      </c>
-      <c r="J68" s="176" t="n">
-        <v>10000</v>
-      </c>
-      <c r="K68" s="176" t="n">
-        <v>8000</v>
-      </c>
-      <c r="L68" s="177" t="n">
-        <v>7763609</v>
+      <c r="F68" s="189">
+        <f>D68/E68</f>
+        <v/>
+      </c>
+      <c r="G68" s="173">
+        <f>F32</f>
+        <v/>
+      </c>
+      <c r="H68" s="176">
+        <f>ROUND(D68*G68,0)</f>
+        <v/>
+      </c>
+      <c r="I68" s="176">
+        <f>ROUND(G32*F68*G68,0)</f>
+        <v/>
+      </c>
+      <c r="J68" s="176">
+        <f>ROUND(H32*F68,0)</f>
+        <v/>
+      </c>
+      <c r="K68" s="176">
+        <f>ROUND(I32*F68,0)</f>
+        <v/>
+      </c>
+      <c r="L68" s="177">
+        <f>H68+I68+J68+K68</f>
+        <v/>
       </c>
     </row>
     <row r="76">

</xml_diff>

<commit_message>
latest 20260610 2026-06-10 13:19
</commit_message>
<xml_diff>
--- a/latest.xlsx
+++ b/latest.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" tabRatio="500" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PO별 개당 수입원가" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="라이센스_워런티" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="합배송_비용안분" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="외화송금내역" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usance_LC" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="환율" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="PO별 개당 수입원가" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="라이센스_워런티" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="합배송_비용안분" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="외화송금내역" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Usance_LC" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="환율" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="RemitTable1">'외화송금내역'!$A$3:$L$39</definedName>
-    <definedName name="RemitTable2">'외화송금내역'!$A$42:$L$87</definedName>
-    <definedName name="FxRateTable">'환율'!$A$7:$D$41</definedName>
+    <definedName name="RemitTable1">'외화송금내역'!$A$3:$L$40</definedName>
+    <definedName name="RemitTable2">'외화송금내역'!$A$43:$L$91</definedName>
+    <definedName name="FxRateTable">'환율'!$A$7:$D$42</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -24,11 +24,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0&quot;일&quot;"/>
+    <numFmt numFmtId="168" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -432,7 +433,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="233">
+  <cellXfs count="241">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1100,6 +1101,30 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="20" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="20" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1546,7 +1571,7 @@
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="170" t="inlineStr">
         <is>
-          <t>회계처리용 통합 데이터  |  기준일: 2026-06-02  |  노란색=미확인  |  보라색=라이센스/워런티  |  날짜→해당항목 좌측 배치</t>
+          <t>회계처리용 통합 데이터  |  기준일: 2026-06-10  |  노란색=미확인  |  보라색=라이센스/워런티  |  날짜→해당항목 좌측 배치</t>
         </is>
       </c>
       <c r="B2" s="148" t="n"/>
@@ -5834,10 +5859,8 @@
       <c r="F37" s="209" t="n">
         <v>46113</v>
       </c>
-      <c r="G37" s="210" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G37" s="210" t="n">
+        <v>46183</v>
       </c>
       <c r="H37" s="211" t="n">
         <v>69160</v>
@@ -5955,10 +5978,8 @@
       <c r="F38" s="209" t="n">
         <v>46113</v>
       </c>
-      <c r="G38" s="210" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G38" s="210" t="n">
+        <v>46183</v>
       </c>
       <c r="H38" s="211" t="n">
         <v>49400</v>
@@ -8763,10 +8784,8 @@
       <c r="F60" s="188" t="n">
         <v>46152</v>
       </c>
-      <c r="G60" s="132" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G60" s="233" t="n">
+        <v>46183</v>
       </c>
       <c r="H60" s="134" t="n">
         <v>500</v>
@@ -8835,7 +8854,11 @@
         <f>ROUND(AA60/AB60,0)</f>
         <v/>
       </c>
-      <c r="AD60" s="137" t="n"/>
+      <c r="AD60" s="137" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
       <c r="AE60" s="137" t="n"/>
       <c r="AF60" s="137" t="n"/>
     </row>
@@ -10825,10 +10848,8 @@
       <c r="G24" s="227" t="n">
         <v>46152</v>
       </c>
-      <c r="H24" s="227" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="H24" s="227" t="n">
+        <v>46183</v>
       </c>
       <c r="I24" s="227" t="inlineStr">
         <is>
@@ -12142,7 +12163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M87"/>
+  <dimension ref="A1:M91"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="12.83203125" customWidth="1" style="160" min="1" max="1"/>
@@ -13975,143 +13996,137 @@
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="169" t="inlineStr">
+      <c r="A40" s="234" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="234" t="inlineStr">
+        <is>
+          <t>2026.06.10</t>
+        </is>
+      </c>
+      <c r="C40" s="235" t="inlineStr">
+        <is>
+          <t>GDC</t>
+        </is>
+      </c>
+      <c r="D40" s="234" t="inlineStr">
+        <is>
+          <t>GPO481, GPO473-2, GPO473-3</t>
+        </is>
+      </c>
+      <c r="E40" s="236" t="n">
+        <v>119060</v>
+      </c>
+      <c r="F40" s="237" t="n">
+        <v>1525.3</v>
+      </c>
+      <c r="G40" s="236" t="n">
+        <v>20</v>
+      </c>
+      <c r="H40" s="238" t="n">
+        <v>12500</v>
+      </c>
+      <c r="I40" s="238" t="n">
+        <v>8000</v>
+      </c>
+      <c r="J40" s="238" t="n">
+        <v>181653224</v>
+      </c>
+      <c r="K40" s="238">
+        <f>ROUND((E40+G40)*F40+H40+I40,0)</f>
+        <v/>
+      </c>
+      <c r="L40" s="239">
+        <f>J40-K40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="169" t="inlineStr">
         <is>
           <t>② PO별 비용 안분 내역</t>
         </is>
       </c>
-      <c r="B40" s="148" t="n"/>
-      <c r="C40" s="148" t="n"/>
-      <c r="D40" s="148" t="n"/>
-      <c r="E40" s="148" t="n"/>
-      <c r="F40" s="148" t="n"/>
-      <c r="G40" s="148" t="n"/>
-      <c r="H40" s="148" t="n"/>
-      <c r="I40" s="148" t="n"/>
-      <c r="J40" s="148" t="n"/>
-      <c r="K40" s="148" t="n"/>
-      <c r="L40" s="149" t="n"/>
-      <c r="M40" s="115" t="n"/>
-    </row>
-    <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="150" t="inlineStr">
+      <c r="B41" s="148" t="n"/>
+      <c r="C41" s="148" t="n"/>
+      <c r="D41" s="148" t="n"/>
+      <c r="E41" s="148" t="n"/>
+      <c r="F41" s="148" t="n"/>
+      <c r="G41" s="148" t="n"/>
+      <c r="H41" s="148" t="n"/>
+      <c r="I41" s="148" t="n"/>
+      <c r="J41" s="148" t="n"/>
+      <c r="K41" s="148" t="n"/>
+      <c r="L41" s="149" t="n"/>
+      <c r="M41" s="115" t="n"/>
+    </row>
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="A42" s="150" t="inlineStr">
         <is>
           <t>PO No.</t>
         </is>
       </c>
-      <c r="B41" s="150" t="inlineStr">
+      <c r="B42" s="150" t="inlineStr">
         <is>
           <t>송금일</t>
         </is>
       </c>
-      <c r="C41" s="150" t="inlineStr">
+      <c r="C42" s="150" t="inlineStr">
         <is>
           <t>업체</t>
         </is>
       </c>
-      <c r="D41" s="150" t="inlineStr">
+      <c r="D42" s="150" t="inlineStr">
         <is>
           <t>PO USD</t>
         </is>
       </c>
-      <c r="E41" s="150" t="inlineStr">
+      <c r="E42" s="150" t="inlineStr">
         <is>
           <t>그룹총USD</t>
         </is>
       </c>
-      <c r="F41" s="150" t="inlineStr">
+      <c r="F42" s="150" t="inlineStr">
         <is>
           <t>배부비율</t>
         </is>
       </c>
-      <c r="G41" s="150" t="inlineStr">
+      <c r="G42" s="150" t="inlineStr">
         <is>
           <t>적용환율</t>
         </is>
       </c>
-      <c r="H41" s="150" t="inlineStr">
+      <c r="H42" s="150" t="inlineStr">
         <is>
           <t>원화환산액</t>
         </is>
       </c>
-      <c r="I41" s="150" t="inlineStr">
+      <c r="I42" s="150" t="inlineStr">
         <is>
           <t>중개수수료안분</t>
         </is>
       </c>
-      <c r="J41" s="150" t="inlineStr">
+      <c r="J42" s="150" t="inlineStr">
         <is>
           <t>수수료안분</t>
         </is>
       </c>
-      <c r="K41" s="150" t="inlineStr">
+      <c r="K42" s="150" t="inlineStr">
         <is>
           <t>전신료안분</t>
         </is>
       </c>
-      <c r="L41" s="150" t="inlineStr">
+      <c r="L42" s="150" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
-      </c>
-      <c r="M41" s="115" t="n"/>
-    </row>
-    <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="116" t="inlineStr">
-        <is>
-          <t>CPO678-1</t>
-        </is>
-      </c>
-      <c r="B42" s="116" t="inlineStr">
-        <is>
-          <t>2025.12.16</t>
-        </is>
-      </c>
-      <c r="C42" s="117" t="inlineStr">
-        <is>
-          <t>Christie</t>
-        </is>
-      </c>
-      <c r="D42" s="118" t="n">
-        <v>139083</v>
-      </c>
-      <c r="E42" s="118" t="n">
-        <v>143557</v>
-      </c>
-      <c r="F42" s="122">
-        <f>D42/E42</f>
-        <v/>
-      </c>
-      <c r="G42" s="118">
-        <f>F10</f>
-        <v/>
-      </c>
-      <c r="H42" s="120">
-        <f>ROUND(D42*G42,0)</f>
-        <v/>
-      </c>
-      <c r="I42" s="120">
-        <f>ROUND(G10*F42*G42,0)</f>
-        <v/>
-      </c>
-      <c r="J42" s="120">
-        <f>ROUND(H10*F42,0)</f>
-        <v/>
-      </c>
-      <c r="K42" s="120">
-        <f>ROUND(I10*F42,0)</f>
-        <v/>
-      </c>
-      <c r="L42" s="121">
-        <f>H42+I42+J42+K42</f>
-        <v/>
       </c>
       <c r="M42" s="115" t="n"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="116" t="inlineStr">
         <is>
-          <t>CPO679</t>
+          <t>CPO678-1</t>
         </is>
       </c>
       <c r="B43" s="116" t="inlineStr">
@@ -14125,7 +14140,7 @@
         </is>
       </c>
       <c r="D43" s="118" t="n">
-        <v>4474</v>
+        <v>139083</v>
       </c>
       <c r="E43" s="118" t="n">
         <v>143557</v>
@@ -14163,7 +14178,7 @@
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="116" t="inlineStr">
         <is>
-          <t>MPO65</t>
+          <t>CPO679</t>
         </is>
       </c>
       <c r="B44" s="116" t="inlineStr">
@@ -14173,21 +14188,21 @@
       </c>
       <c r="C44" s="117" t="inlineStr">
         <is>
-          <t>MAG</t>
+          <t>Christie</t>
         </is>
       </c>
       <c r="D44" s="118" t="n">
-        <v>4936</v>
+        <v>4474</v>
       </c>
       <c r="E44" s="118" t="n">
-        <v>15040</v>
+        <v>143557</v>
       </c>
       <c r="F44" s="122">
         <f>D44/E44</f>
         <v/>
       </c>
       <c r="G44" s="118">
-        <f>F9</f>
+        <f>F10</f>
         <v/>
       </c>
       <c r="H44" s="120">
@@ -14195,15 +14210,15 @@
         <v/>
       </c>
       <c r="I44" s="120">
-        <f>ROUND(G9*F44*G44,0)</f>
+        <f>ROUND(G10*F44*G44,0)</f>
         <v/>
       </c>
       <c r="J44" s="120">
-        <f>ROUND(H9*F44,0)</f>
+        <f>ROUND(H10*F44,0)</f>
         <v/>
       </c>
       <c r="K44" s="120">
-        <f>ROUND(I9*F44,0)</f>
+        <f>ROUND(I10*F44,0)</f>
         <v/>
       </c>
       <c r="L44" s="121">
@@ -14215,31 +14230,31 @@
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="116" t="inlineStr">
         <is>
-          <t>GPO451</t>
+          <t>MPO65</t>
         </is>
       </c>
       <c r="B45" s="116" t="inlineStr">
         <is>
-          <t>2025.12.29</t>
+          <t>2025.12.16</t>
         </is>
       </c>
       <c r="C45" s="117" t="inlineStr">
         <is>
-          <t>GDC</t>
+          <t>MAG</t>
         </is>
       </c>
       <c r="D45" s="118" t="n">
-        <v>9060</v>
+        <v>4936</v>
       </c>
       <c r="E45" s="118" t="n">
-        <v>13860</v>
+        <v>15040</v>
       </c>
       <c r="F45" s="122">
         <f>D45/E45</f>
         <v/>
       </c>
       <c r="G45" s="118">
-        <f>F12</f>
+        <f>F9</f>
         <v/>
       </c>
       <c r="H45" s="120">
@@ -14247,15 +14262,15 @@
         <v/>
       </c>
       <c r="I45" s="120">
-        <f>ROUND(G12*F45*G45,0)</f>
+        <f>ROUND(G9*F45*G45,0)</f>
         <v/>
       </c>
       <c r="J45" s="120">
-        <f>ROUND(H12*F45,0)</f>
+        <f>ROUND(H9*F45,0)</f>
         <v/>
       </c>
       <c r="K45" s="120">
-        <f>ROUND(I12*F45,0)</f>
+        <f>ROUND(I9*F45,0)</f>
         <v/>
       </c>
       <c r="L45" s="121">
@@ -14267,7 +14282,7 @@
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="116" t="inlineStr">
         <is>
-          <t>GPO458</t>
+          <t>GPO451</t>
         </is>
       </c>
       <c r="B46" s="116" t="inlineStr">
@@ -14281,7 +14296,7 @@
         </is>
       </c>
       <c r="D46" s="118" t="n">
-        <v>350</v>
+        <v>9060</v>
       </c>
       <c r="E46" s="118" t="n">
         <v>13860</v>
@@ -14319,31 +14334,31 @@
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="116" t="inlineStr">
         <is>
-          <t>CPO680</t>
+          <t>GPO458</t>
         </is>
       </c>
       <c r="B47" s="116" t="inlineStr">
         <is>
-          <t>2026.01.13</t>
+          <t>2025.12.29</t>
         </is>
       </c>
       <c r="C47" s="117" t="inlineStr">
         <is>
-          <t>Christie</t>
+          <t>GDC</t>
         </is>
       </c>
       <c r="D47" s="118" t="n">
-        <v>252</v>
+        <v>350</v>
       </c>
       <c r="E47" s="118" t="n">
-        <v>252</v>
+        <v>13860</v>
       </c>
       <c r="F47" s="122">
         <f>D47/E47</f>
         <v/>
       </c>
       <c r="G47" s="118">
-        <f>F14</f>
+        <f>F12</f>
         <v/>
       </c>
       <c r="H47" s="120">
@@ -14351,15 +14366,15 @@
         <v/>
       </c>
       <c r="I47" s="120">
-        <f>ROUND(G14*F47*G47,0)</f>
+        <f>ROUND(G12*F47*G47,0)</f>
         <v/>
       </c>
       <c r="J47" s="120">
-        <f>ROUND(H14*F47,0)</f>
+        <f>ROUND(H12*F47,0)</f>
         <v/>
       </c>
       <c r="K47" s="120">
-        <f>ROUND(I14*F47,0)</f>
+        <f>ROUND(I12*F47,0)</f>
         <v/>
       </c>
       <c r="L47" s="121">
@@ -14371,31 +14386,31 @@
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="116" t="inlineStr">
         <is>
-          <t>GPO459</t>
+          <t>CPO680</t>
         </is>
       </c>
       <c r="B48" s="116" t="inlineStr">
         <is>
-          <t>2026.01.21</t>
+          <t>2026.01.13</t>
         </is>
       </c>
       <c r="C48" s="117" t="inlineStr">
         <is>
-          <t>GDC</t>
+          <t>Christie</t>
         </is>
       </c>
       <c r="D48" s="118" t="n">
-        <v>450</v>
+        <v>252</v>
       </c>
       <c r="E48" s="118" t="n">
-        <v>3700</v>
+        <v>252</v>
       </c>
       <c r="F48" s="122">
         <f>D48/E48</f>
         <v/>
       </c>
       <c r="G48" s="118">
-        <f>F15</f>
+        <f>F14</f>
         <v/>
       </c>
       <c r="H48" s="120">
@@ -14403,15 +14418,15 @@
         <v/>
       </c>
       <c r="I48" s="120">
-        <f>ROUND(G15*F48*G48,0)</f>
+        <f>ROUND(G14*F48*G48,0)</f>
         <v/>
       </c>
       <c r="J48" s="120">
-        <f>ROUND(H15*F48,0)</f>
+        <f>ROUND(H14*F48,0)</f>
         <v/>
       </c>
       <c r="K48" s="120">
-        <f>ROUND(I15*F48,0)</f>
+        <f>ROUND(I14*F48,0)</f>
         <v/>
       </c>
       <c r="L48" s="121">
@@ -14423,7 +14438,7 @@
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="116" t="inlineStr">
         <is>
-          <t>GPO460</t>
+          <t>GPO459</t>
         </is>
       </c>
       <c r="B49" s="116" t="inlineStr">
@@ -14437,7 +14452,7 @@
         </is>
       </c>
       <c r="D49" s="118" t="n">
-        <v>2710</v>
+        <v>450</v>
       </c>
       <c r="E49" s="118" t="n">
         <v>3700</v>
@@ -14475,7 +14490,7 @@
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="116" t="inlineStr">
         <is>
-          <t>GPO461</t>
+          <t>GPO460</t>
         </is>
       </c>
       <c r="B50" s="116" t="inlineStr">
@@ -14489,7 +14504,7 @@
         </is>
       </c>
       <c r="D50" s="118" t="n">
-        <v>540</v>
+        <v>2710</v>
       </c>
       <c r="E50" s="118" t="n">
         <v>3700</v>
@@ -14527,7 +14542,7 @@
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="116" t="inlineStr">
         <is>
-          <t>MPO66</t>
+          <t>GPO461</t>
         </is>
       </c>
       <c r="B51" s="116" t="inlineStr">
@@ -14537,21 +14552,21 @@
       </c>
       <c r="C51" s="117" t="inlineStr">
         <is>
-          <t>MAG</t>
+          <t>GDC</t>
         </is>
       </c>
       <c r="D51" s="118" t="n">
-        <v>9626.35</v>
+        <v>540</v>
       </c>
       <c r="E51" s="118" t="n">
-        <v>9626.35</v>
+        <v>3700</v>
       </c>
       <c r="F51" s="122">
         <f>D51/E51</f>
         <v/>
       </c>
       <c r="G51" s="118">
-        <f>F16</f>
+        <f>F15</f>
         <v/>
       </c>
       <c r="H51" s="120">
@@ -14559,15 +14574,15 @@
         <v/>
       </c>
       <c r="I51" s="120">
-        <f>ROUND(G16*F51*G51,0)</f>
+        <f>ROUND(G15*F51*G51,0)</f>
         <v/>
       </c>
       <c r="J51" s="120">
-        <f>ROUND(H16*F51,0)</f>
+        <f>ROUND(H15*F51,0)</f>
         <v/>
       </c>
       <c r="K51" s="120">
-        <f>ROUND(I16*F51,0)</f>
+        <f>ROUND(I15*F51,0)</f>
         <v/>
       </c>
       <c r="L51" s="121">
@@ -14579,31 +14594,31 @@
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="116" t="inlineStr">
         <is>
-          <t>LPO001</t>
+          <t>MPO66</t>
         </is>
       </c>
       <c r="B52" s="116" t="inlineStr">
         <is>
-          <t>2026.01.30</t>
+          <t>2026.01.21</t>
         </is>
       </c>
       <c r="C52" s="117" t="inlineStr">
         <is>
-          <t>Lemon</t>
+          <t>MAG</t>
         </is>
       </c>
       <c r="D52" s="118" t="n">
-        <v>5056.8</v>
+        <v>9626.35</v>
       </c>
       <c r="E52" s="118" t="n">
-        <v>5056.8</v>
+        <v>9626.35</v>
       </c>
       <c r="F52" s="122">
         <f>D52/E52</f>
         <v/>
       </c>
       <c r="G52" s="118">
-        <f>F17</f>
+        <f>F16</f>
         <v/>
       </c>
       <c r="H52" s="120">
@@ -14611,15 +14626,15 @@
         <v/>
       </c>
       <c r="I52" s="120">
-        <f>ROUND(G17*F52*G52,0)</f>
+        <f>ROUND(G16*F52*G52,0)</f>
         <v/>
       </c>
       <c r="J52" s="120">
-        <f>ROUND(H17*F52,0)</f>
+        <f>ROUND(H16*F52,0)</f>
         <v/>
       </c>
       <c r="K52" s="120">
-        <f>ROUND(I17*F52,0)</f>
+        <f>ROUND(I16*F52,0)</f>
         <v/>
       </c>
       <c r="L52" s="121">
@@ -14631,31 +14646,31 @@
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="116" t="inlineStr">
         <is>
-          <t>CPO682</t>
+          <t>LPO001</t>
         </is>
       </c>
       <c r="B53" s="116" t="inlineStr">
         <is>
-          <t>2026.02.04</t>
+          <t>2026.01.30</t>
         </is>
       </c>
       <c r="C53" s="117" t="inlineStr">
         <is>
-          <t>Christie</t>
+          <t>Lemon</t>
         </is>
       </c>
       <c r="D53" s="118" t="n">
-        <v>20174</v>
+        <v>5056.8</v>
       </c>
       <c r="E53" s="118" t="n">
-        <v>24794</v>
+        <v>5056.8</v>
       </c>
       <c r="F53" s="122">
         <f>D53/E53</f>
         <v/>
       </c>
       <c r="G53" s="118">
-        <f>F19</f>
+        <f>F17</f>
         <v/>
       </c>
       <c r="H53" s="120">
@@ -14663,15 +14678,15 @@
         <v/>
       </c>
       <c r="I53" s="120">
-        <f>ROUND(G19*F53*G53,0)</f>
+        <f>ROUND(G17*F53*G53,0)</f>
         <v/>
       </c>
       <c r="J53" s="120">
-        <f>ROUND(H19*F53,0)</f>
+        <f>ROUND(H17*F53,0)</f>
         <v/>
       </c>
       <c r="K53" s="120">
-        <f>ROUND(I19*F53,0)</f>
+        <f>ROUND(I17*F53,0)</f>
         <v/>
       </c>
       <c r="L53" s="121">
@@ -14683,7 +14698,7 @@
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="116" t="inlineStr">
         <is>
-          <t>CPO683</t>
+          <t>CPO682</t>
         </is>
       </c>
       <c r="B54" s="116" t="inlineStr">
@@ -14697,7 +14712,7 @@
         </is>
       </c>
       <c r="D54" s="118" t="n">
-        <v>4620</v>
+        <v>20174</v>
       </c>
       <c r="E54" s="118" t="n">
         <v>24794</v>
@@ -14735,7 +14750,7 @@
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="116" t="inlineStr">
         <is>
-          <t>GPO462</t>
+          <t>CPO683</t>
         </is>
       </c>
       <c r="B55" s="116" t="inlineStr">
@@ -14745,21 +14760,21 @@
       </c>
       <c r="C55" s="117" t="inlineStr">
         <is>
-          <t>GDC</t>
+          <t>Christie</t>
         </is>
       </c>
       <c r="D55" s="118" t="n">
-        <v>1440</v>
+        <v>4620</v>
       </c>
       <c r="E55" s="118" t="n">
-        <v>11599.57</v>
+        <v>24794</v>
       </c>
       <c r="F55" s="122">
         <f>D55/E55</f>
         <v/>
       </c>
       <c r="G55" s="118">
-        <f>F20</f>
+        <f>F19</f>
         <v/>
       </c>
       <c r="H55" s="120">
@@ -14767,15 +14782,15 @@
         <v/>
       </c>
       <c r="I55" s="120">
-        <f>ROUND(G20*F55*G55,0)</f>
+        <f>ROUND(G19*F55*G55,0)</f>
         <v/>
       </c>
       <c r="J55" s="120">
-        <f>ROUND(H20*F55,0)</f>
+        <f>ROUND(H19*F55,0)</f>
         <v/>
       </c>
       <c r="K55" s="120">
-        <f>ROUND(I20*F55,0)</f>
+        <f>ROUND(I19*F55,0)</f>
         <v/>
       </c>
       <c r="L55" s="121">
@@ -14787,7 +14802,7 @@
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="116" t="inlineStr">
         <is>
-          <t>GPO463</t>
+          <t>GPO462</t>
         </is>
       </c>
       <c r="B56" s="116" t="inlineStr">
@@ -14801,7 +14816,7 @@
         </is>
       </c>
       <c r="D56" s="118" t="n">
-        <v>4489</v>
+        <v>1440</v>
       </c>
       <c r="E56" s="118" t="n">
         <v>11599.57</v>
@@ -14839,7 +14854,7 @@
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="116" t="inlineStr">
         <is>
-          <t>GPO464</t>
+          <t>GPO463</t>
         </is>
       </c>
       <c r="B57" s="116" t="inlineStr">
@@ -14853,7 +14868,7 @@
         </is>
       </c>
       <c r="D57" s="118" t="n">
-        <v>5670.57</v>
+        <v>4489</v>
       </c>
       <c r="E57" s="118" t="n">
         <v>11599.57</v>
@@ -14891,31 +14906,31 @@
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="116" t="inlineStr">
         <is>
-          <t>CPO681</t>
+          <t>GPO464</t>
         </is>
       </c>
       <c r="B58" s="116" t="inlineStr">
         <is>
-          <t>2026.02.11</t>
+          <t>2026.02.04</t>
         </is>
       </c>
       <c r="C58" s="117" t="inlineStr">
         <is>
-          <t>Christie</t>
+          <t>GDC</t>
         </is>
       </c>
       <c r="D58" s="118" t="n">
-        <v>26358</v>
+        <v>5670.57</v>
       </c>
       <c r="E58" s="118" t="n">
-        <v>26358</v>
+        <v>11599.57</v>
       </c>
       <c r="F58" s="122">
         <f>D58/E58</f>
         <v/>
       </c>
       <c r="G58" s="118">
-        <f>F21</f>
+        <f>F20</f>
         <v/>
       </c>
       <c r="H58" s="120">
@@ -14923,15 +14938,15 @@
         <v/>
       </c>
       <c r="I58" s="120">
-        <f>ROUND(G21*F58*G58,0)</f>
+        <f>ROUND(G20*F58*G58,0)</f>
         <v/>
       </c>
       <c r="J58" s="120">
-        <f>ROUND(H21*F58,0)</f>
+        <f>ROUND(H20*F58,0)</f>
         <v/>
       </c>
       <c r="K58" s="120">
-        <f>ROUND(I21*F58,0)</f>
+        <f>ROUND(I20*F58,0)</f>
         <v/>
       </c>
       <c r="L58" s="121">
@@ -14943,12 +14958,12 @@
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="116" t="inlineStr">
         <is>
-          <t>CPO686</t>
+          <t>CPO681</t>
         </is>
       </c>
       <c r="B59" s="116" t="inlineStr">
         <is>
-          <t>2026.02.19</t>
+          <t>2026.02.11</t>
         </is>
       </c>
       <c r="C59" s="117" t="inlineStr">
@@ -14957,17 +14972,17 @@
         </is>
       </c>
       <c r="D59" s="118" t="n">
-        <v>14793</v>
+        <v>26358</v>
       </c>
       <c r="E59" s="118" t="n">
-        <v>17538</v>
+        <v>26358</v>
       </c>
       <c r="F59" s="122">
         <f>D59/E59</f>
         <v/>
       </c>
       <c r="G59" s="118">
-        <f>F22</f>
+        <f>F21</f>
         <v/>
       </c>
       <c r="H59" s="120">
@@ -14975,15 +14990,15 @@
         <v/>
       </c>
       <c r="I59" s="120">
-        <f>ROUND(G22*F59*G59,0)</f>
+        <f>ROUND(G21*F59*G59,0)</f>
         <v/>
       </c>
       <c r="J59" s="120">
-        <f>ROUND(H22*F59,0)</f>
+        <f>ROUND(H21*F59,0)</f>
         <v/>
       </c>
       <c r="K59" s="120">
-        <f>ROUND(I22*F59,0)</f>
+        <f>ROUND(I21*F59,0)</f>
         <v/>
       </c>
       <c r="L59" s="121">
@@ -14995,7 +15010,7 @@
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="116" t="inlineStr">
         <is>
-          <t>CPO689</t>
+          <t>CPO686</t>
         </is>
       </c>
       <c r="B60" s="116" t="inlineStr">
@@ -15009,7 +15024,7 @@
         </is>
       </c>
       <c r="D60" s="118" t="n">
-        <v>2745</v>
+        <v>14793</v>
       </c>
       <c r="E60" s="118" t="n">
         <v>17538</v>
@@ -15047,12 +15062,12 @@
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="116" t="inlineStr">
         <is>
-          <t>CPO667</t>
+          <t>CPO689</t>
         </is>
       </c>
       <c r="B61" s="116" t="inlineStr">
         <is>
-          <t>2026.02.27</t>
+          <t>2026.02.19</t>
         </is>
       </c>
       <c r="C61" s="117" t="inlineStr">
@@ -15061,17 +15076,17 @@
         </is>
       </c>
       <c r="D61" s="118" t="n">
-        <v>5673</v>
+        <v>2745</v>
       </c>
       <c r="E61" s="118" t="n">
-        <v>142189</v>
+        <v>17538</v>
       </c>
       <c r="F61" s="122">
         <f>D61/E61</f>
         <v/>
       </c>
       <c r="G61" s="118">
-        <f>F23</f>
+        <f>F22</f>
         <v/>
       </c>
       <c r="H61" s="120">
@@ -15079,15 +15094,15 @@
         <v/>
       </c>
       <c r="I61" s="120">
-        <f>ROUND(G23*F61*G61,0)</f>
+        <f>ROUND(G22*F61*G61,0)</f>
         <v/>
       </c>
       <c r="J61" s="120">
-        <f>ROUND(H23*F61,0)</f>
+        <f>ROUND(H22*F61,0)</f>
         <v/>
       </c>
       <c r="K61" s="120">
-        <f>ROUND(I23*F61,0)</f>
+        <f>ROUND(I22*F61,0)</f>
         <v/>
       </c>
       <c r="L61" s="121">
@@ -15099,7 +15114,7 @@
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="116" t="inlineStr">
         <is>
-          <t>CPO685</t>
+          <t>CPO667</t>
         </is>
       </c>
       <c r="B62" s="116" t="inlineStr">
@@ -15113,7 +15128,7 @@
         </is>
       </c>
       <c r="D62" s="118" t="n">
-        <v>136516</v>
+        <v>5673</v>
       </c>
       <c r="E62" s="118" t="n">
         <v>142189</v>
@@ -15151,12 +15166,12 @@
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="116" t="inlineStr">
         <is>
-          <t>CPO678-2</t>
+          <t>CPO685</t>
         </is>
       </c>
       <c r="B63" s="116" t="inlineStr">
         <is>
-          <t>2026.03.06</t>
+          <t>2026.02.27</t>
         </is>
       </c>
       <c r="C63" s="117" t="inlineStr">
@@ -15165,17 +15180,17 @@
         </is>
       </c>
       <c r="D63" s="118" t="n">
-        <v>137850</v>
+        <v>136516</v>
       </c>
       <c r="E63" s="118" t="n">
-        <v>137850</v>
+        <v>142189</v>
       </c>
       <c r="F63" s="122">
         <f>D63/E63</f>
         <v/>
       </c>
       <c r="G63" s="118">
-        <f>F24</f>
+        <f>F23</f>
         <v/>
       </c>
       <c r="H63" s="120">
@@ -15183,15 +15198,15 @@
         <v/>
       </c>
       <c r="I63" s="120">
-        <f>ROUND(G24*F63*G63,0)</f>
+        <f>ROUND(G23*F63*G63,0)</f>
         <v/>
       </c>
       <c r="J63" s="120">
-        <f>ROUND(H24*F63,0)</f>
+        <f>ROUND(H23*F63,0)</f>
         <v/>
       </c>
       <c r="K63" s="120">
-        <f>ROUND(I24*F63,0)</f>
+        <f>ROUND(I23*F63,0)</f>
         <v/>
       </c>
       <c r="L63" s="121">
@@ -15203,12 +15218,12 @@
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="116" t="inlineStr">
         <is>
-          <t>CPO690</t>
+          <t>CPO678-2</t>
         </is>
       </c>
       <c r="B64" s="116" t="inlineStr">
         <is>
-          <t>2026.04.01</t>
+          <t>2026.03.06</t>
         </is>
       </c>
       <c r="C64" s="117" t="inlineStr">
@@ -15217,17 +15232,17 @@
         </is>
       </c>
       <c r="D64" s="118" t="n">
-        <v>9740</v>
+        <v>137850</v>
       </c>
       <c r="E64" s="118" t="n">
-        <v>34354</v>
+        <v>137850</v>
       </c>
       <c r="F64" s="122">
         <f>D64/E64</f>
         <v/>
       </c>
       <c r="G64" s="118">
-        <f>F25</f>
+        <f>F24</f>
         <v/>
       </c>
       <c r="H64" s="120">
@@ -15235,15 +15250,15 @@
         <v/>
       </c>
       <c r="I64" s="120">
-        <f>ROUND(G25*F64*G64,0)</f>
+        <f>ROUND(G24*F64*G64,0)</f>
         <v/>
       </c>
       <c r="J64" s="120">
-        <f>ROUND(H25*F64,0)</f>
+        <f>ROUND(H24*F64,0)</f>
         <v/>
       </c>
       <c r="K64" s="120">
-        <f>ROUND(I25*F64,0)</f>
+        <f>ROUND(I24*F64,0)</f>
         <v/>
       </c>
       <c r="L64" s="121">
@@ -15255,7 +15270,7 @@
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="116" t="inlineStr">
         <is>
-          <t>CPO691</t>
+          <t>CPO690</t>
         </is>
       </c>
       <c r="B65" s="116" t="inlineStr">
@@ -15269,7 +15284,7 @@
         </is>
       </c>
       <c r="D65" s="118" t="n">
-        <v>24614</v>
+        <v>9740</v>
       </c>
       <c r="E65" s="118" t="n">
         <v>34354</v>
@@ -15307,7 +15322,7 @@
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="116" t="inlineStr">
         <is>
-          <t>GPO467</t>
+          <t>CPO691</t>
         </is>
       </c>
       <c r="B66" s="116" t="inlineStr">
@@ -15317,21 +15332,21 @@
       </c>
       <c r="C66" s="117" t="inlineStr">
         <is>
-          <t>GDC</t>
+          <t>Christie</t>
         </is>
       </c>
       <c r="D66" s="118" t="n">
-        <v>1700</v>
+        <v>24614</v>
       </c>
       <c r="E66" s="118" t="n">
-        <v>6553.05</v>
+        <v>34354</v>
       </c>
       <c r="F66" s="122">
         <f>D66/E66</f>
         <v/>
       </c>
       <c r="G66" s="118">
-        <f>F26</f>
+        <f>F25</f>
         <v/>
       </c>
       <c r="H66" s="120">
@@ -15339,15 +15354,15 @@
         <v/>
       </c>
       <c r="I66" s="120">
-        <f>ROUND(G26*F66*G66,0)</f>
+        <f>ROUND(G25*F66*G66,0)</f>
         <v/>
       </c>
       <c r="J66" s="120">
-        <f>ROUND(H26*F66,0)</f>
+        <f>ROUND(H25*F66,0)</f>
         <v/>
       </c>
       <c r="K66" s="120">
-        <f>ROUND(I26*F66,0)</f>
+        <f>ROUND(I25*F66,0)</f>
         <v/>
       </c>
       <c r="L66" s="121">
@@ -15359,7 +15374,7 @@
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="116" t="inlineStr">
         <is>
-          <t>GPO469</t>
+          <t>GPO467</t>
         </is>
       </c>
       <c r="B67" s="116" t="inlineStr">
@@ -15373,7 +15388,7 @@
         </is>
       </c>
       <c r="D67" s="118" t="n">
-        <v>3993.05</v>
+        <v>1700</v>
       </c>
       <c r="E67" s="118" t="n">
         <v>6553.05</v>
@@ -15411,7 +15426,7 @@
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="116" t="inlineStr">
         <is>
-          <t>GPO470</t>
+          <t>GPO469</t>
         </is>
       </c>
       <c r="B68" s="116" t="inlineStr">
@@ -15425,7 +15440,7 @@
         </is>
       </c>
       <c r="D68" s="118" t="n">
-        <v>360</v>
+        <v>3993.05</v>
       </c>
       <c r="E68" s="118" t="n">
         <v>6553.05</v>
@@ -15463,7 +15478,7 @@
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="116" t="inlineStr">
         <is>
-          <t>GPO471</t>
+          <t>GPO470</t>
         </is>
       </c>
       <c r="B69" s="116" t="inlineStr">
@@ -15477,7 +15492,7 @@
         </is>
       </c>
       <c r="D69" s="118" t="n">
-        <v>500</v>
+        <v>360</v>
       </c>
       <c r="E69" s="118" t="n">
         <v>6553.05</v>
@@ -15515,12 +15530,12 @@
     <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="116" t="inlineStr">
         <is>
-          <t>GPO468-1</t>
+          <t>GPO471</t>
         </is>
       </c>
       <c r="B70" s="116" t="inlineStr">
         <is>
-          <t>2026.04.14</t>
+          <t>2026.04.01</t>
         </is>
       </c>
       <c r="C70" s="117" t="inlineStr">
@@ -15529,17 +15544,17 @@
         </is>
       </c>
       <c r="D70" s="118" t="n">
-        <v>36190</v>
+        <v>500</v>
       </c>
       <c r="E70" s="118" t="n">
-        <v>57650</v>
+        <v>6553.05</v>
       </c>
       <c r="F70" s="122">
         <f>D70/E70</f>
         <v/>
       </c>
       <c r="G70" s="118">
-        <f>F27</f>
+        <f>F26</f>
         <v/>
       </c>
       <c r="H70" s="120">
@@ -15547,15 +15562,15 @@
         <v/>
       </c>
       <c r="I70" s="120">
-        <f>ROUND(G27*F70*G70,0)</f>
+        <f>ROUND(G26*F70*G70,0)</f>
         <v/>
       </c>
       <c r="J70" s="120">
-        <f>ROUND(H27*F70,0)</f>
+        <f>ROUND(H26*F70,0)</f>
         <v/>
       </c>
       <c r="K70" s="120">
-        <f>ROUND(I27*F70,0)</f>
+        <f>ROUND(I26*F70,0)</f>
         <v/>
       </c>
       <c r="L70" s="121">
@@ -15567,7 +15582,7 @@
     <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="116" t="inlineStr">
         <is>
-          <t>GPO472</t>
+          <t>GPO468-1</t>
         </is>
       </c>
       <c r="B71" s="116" t="inlineStr">
@@ -15581,7 +15596,7 @@
         </is>
       </c>
       <c r="D71" s="118" t="n">
-        <v>180</v>
+        <v>36190</v>
       </c>
       <c r="E71" s="118" t="n">
         <v>57650</v>
@@ -15619,7 +15634,7 @@
     <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="116" t="inlineStr">
         <is>
-          <t>GPO468-2</t>
+          <t>GPO472</t>
         </is>
       </c>
       <c r="B72" s="116" t="inlineStr">
@@ -15633,7 +15648,7 @@
         </is>
       </c>
       <c r="D72" s="118" t="n">
-        <v>21280</v>
+        <v>180</v>
       </c>
       <c r="E72" s="118" t="n">
         <v>57650</v>
@@ -15671,31 +15686,31 @@
     <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="116" t="inlineStr">
         <is>
-          <t>CPO692-1</t>
+          <t>GPO468-2</t>
         </is>
       </c>
       <c r="B73" s="116" t="inlineStr">
         <is>
-          <t>2026.04.22</t>
+          <t>2026.04.14</t>
         </is>
       </c>
       <c r="C73" s="117" t="inlineStr">
         <is>
-          <t>Christie</t>
+          <t>GDC</t>
         </is>
       </c>
       <c r="D73" s="118" t="n">
-        <v>11000</v>
+        <v>21280</v>
       </c>
       <c r="E73" s="118" t="n">
-        <v>297580</v>
+        <v>57650</v>
       </c>
       <c r="F73" s="122">
         <f>D73/E73</f>
         <v/>
       </c>
       <c r="G73" s="118">
-        <f>F31</f>
+        <f>F27</f>
         <v/>
       </c>
       <c r="H73" s="120">
@@ -15703,15 +15718,15 @@
         <v/>
       </c>
       <c r="I73" s="120">
-        <f>ROUND(G31*F73*G73,0)</f>
+        <f>ROUND(G27*F73*G73,0)</f>
         <v/>
       </c>
       <c r="J73" s="120">
-        <f>ROUND(H31*F73,0)</f>
+        <f>ROUND(H27*F73,0)</f>
         <v/>
       </c>
       <c r="K73" s="120">
-        <f>ROUND(I31*F73,0)</f>
+        <f>ROUND(I27*F73,0)</f>
         <v/>
       </c>
       <c r="L73" s="121">
@@ -15723,7 +15738,7 @@
     <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="116" t="inlineStr">
         <is>
-          <t>CPO692-2</t>
+          <t>CPO692-1</t>
         </is>
       </c>
       <c r="B74" s="116" t="inlineStr">
@@ -15737,7 +15752,7 @@
         </is>
       </c>
       <c r="D74" s="118" t="n">
-        <v>286580</v>
+        <v>11000</v>
       </c>
       <c r="E74" s="118" t="n">
         <v>297580</v>
@@ -15775,7 +15790,7 @@
     <row r="75" ht="15.75" customHeight="1">
       <c r="A75" s="116" t="inlineStr">
         <is>
-          <t>EPO18</t>
+          <t>CPO692-2</t>
         </is>
       </c>
       <c r="B75" s="116" t="inlineStr">
@@ -15785,21 +15800,21 @@
       </c>
       <c r="C75" s="117" t="inlineStr">
         <is>
-          <t>MAICO Italia</t>
+          <t>Christie</t>
         </is>
       </c>
       <c r="D75" s="118" t="n">
-        <v>4388.4</v>
+        <v>286580</v>
       </c>
       <c r="E75" s="118" t="n">
-        <v>4388.4</v>
+        <v>297580</v>
       </c>
       <c r="F75" s="122">
         <f>D75/E75</f>
         <v/>
       </c>
       <c r="G75" s="118">
-        <f>F32</f>
+        <f>F31</f>
         <v/>
       </c>
       <c r="H75" s="120">
@@ -15807,50 +15822,51 @@
         <v/>
       </c>
       <c r="I75" s="120">
-        <f>ROUND(G32*F75*G75,0)</f>
+        <f>ROUND(G31*F75*G75,0)</f>
         <v/>
       </c>
       <c r="J75" s="120">
-        <f>ROUND(H32*F75,0)</f>
+        <f>ROUND(H31*F75,0)</f>
         <v/>
       </c>
       <c r="K75" s="120">
-        <f>ROUND(I32*F75,0)</f>
+        <f>ROUND(I31*F75,0)</f>
         <v/>
       </c>
       <c r="L75" s="121">
         <f>H75+I75+J75+K75</f>
         <v/>
       </c>
+      <c r="M75" s="115" t="n"/>
     </row>
     <row r="76" ht="15.75" customHeight="1">
       <c r="A76" s="116" t="inlineStr">
         <is>
-          <t>CPO694</t>
+          <t>EPO18</t>
         </is>
       </c>
       <c r="B76" s="116" t="inlineStr">
         <is>
-          <t>2026.05.04</t>
+          <t>2026.04.22</t>
         </is>
       </c>
       <c r="C76" s="117" t="inlineStr">
         <is>
-          <t>Christie</t>
+          <t>MAICO Italia</t>
         </is>
       </c>
       <c r="D76" s="118" t="n">
-        <v>17404</v>
+        <v>4388.4</v>
       </c>
       <c r="E76" s="118" t="n">
-        <v>21439</v>
+        <v>4388.4</v>
       </c>
       <c r="F76" s="122">
         <f>D76/E76</f>
         <v/>
       </c>
       <c r="G76" s="118">
-        <f>F33</f>
+        <f>F32</f>
         <v/>
       </c>
       <c r="H76" s="120">
@@ -15858,15 +15874,15 @@
         <v/>
       </c>
       <c r="I76" s="120">
-        <f>ROUND(G33*F76*G76,0)</f>
+        <f>ROUND(G32*F76*G76,0)</f>
         <v/>
       </c>
       <c r="J76" s="120">
-        <f>ROUND(H33*F76,0)</f>
+        <f>ROUND(H32*F76,0)</f>
         <v/>
       </c>
       <c r="K76" s="120">
-        <f>ROUND(I33*F76,0)</f>
+        <f>ROUND(I32*F76,0)</f>
         <v/>
       </c>
       <c r="L76" s="121">
@@ -15877,7 +15893,7 @@
     <row r="77" ht="15.75" customHeight="1">
       <c r="A77" s="116" t="inlineStr">
         <is>
-          <t>CPO695-1</t>
+          <t>CPO694</t>
         </is>
       </c>
       <c r="B77" s="116" t="inlineStr">
@@ -15891,7 +15907,7 @@
         </is>
       </c>
       <c r="D77" s="118" t="n">
-        <v>2058</v>
+        <v>17404</v>
       </c>
       <c r="E77" s="118" t="n">
         <v>21439</v>
@@ -15928,7 +15944,7 @@
     <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="116" t="inlineStr">
         <is>
-          <t>CPO695-2</t>
+          <t>CPO695-1</t>
         </is>
       </c>
       <c r="B78" s="116" t="inlineStr">
@@ -15942,7 +15958,7 @@
         </is>
       </c>
       <c r="D78" s="118" t="n">
-        <v>1977</v>
+        <v>2058</v>
       </c>
       <c r="E78" s="118" t="n">
         <v>21439</v>
@@ -15979,7 +15995,7 @@
     <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="116" t="inlineStr">
         <is>
-          <t>IPO016</t>
+          <t>CPO695-2</t>
         </is>
       </c>
       <c r="B79" s="116" t="inlineStr">
@@ -15989,21 +16005,21 @@
       </c>
       <c r="C79" s="117" t="inlineStr">
         <is>
-          <t>Integ</t>
+          <t>Christie</t>
         </is>
       </c>
       <c r="D79" s="118" t="n">
-        <v>6800</v>
+        <v>1977</v>
       </c>
       <c r="E79" s="118" t="n">
-        <v>6800</v>
+        <v>21439</v>
       </c>
       <c r="F79" s="122">
         <f>D79/E79</f>
         <v/>
       </c>
       <c r="G79" s="118">
-        <f>F34</f>
+        <f>F33</f>
         <v/>
       </c>
       <c r="H79" s="120">
@@ -16011,15 +16027,15 @@
         <v/>
       </c>
       <c r="I79" s="120">
-        <f>ROUND(G34*F79*G79,0)</f>
+        <f>ROUND(G33*F79*G79,0)</f>
         <v/>
       </c>
       <c r="J79" s="120">
-        <f>ROUND(H34*F79,0)</f>
+        <f>ROUND(H33*F79,0)</f>
         <v/>
       </c>
       <c r="K79" s="120">
-        <f>ROUND(I34*F79,0)</f>
+        <f>ROUND(I33*F79,0)</f>
         <v/>
       </c>
       <c r="L79" s="121">
@@ -16030,31 +16046,31 @@
     <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="116" t="inlineStr">
         <is>
-          <t>GPO478</t>
+          <t>IPO016</t>
         </is>
       </c>
       <c r="B80" s="116" t="inlineStr">
         <is>
-          <t>2026.05.19</t>
+          <t>2026.05.04</t>
         </is>
       </c>
       <c r="C80" s="117" t="inlineStr">
         <is>
-          <t>GDC</t>
+          <t>Integ</t>
         </is>
       </c>
       <c r="D80" s="118" t="n">
-        <v>180</v>
+        <v>6800</v>
       </c>
       <c r="E80" s="118" t="n">
-        <v>180</v>
+        <v>6800</v>
       </c>
       <c r="F80" s="122">
         <f>D80/E80</f>
         <v/>
       </c>
       <c r="G80" s="118">
-        <f>F36</f>
+        <f>F34</f>
         <v/>
       </c>
       <c r="H80" s="120">
@@ -16062,15 +16078,15 @@
         <v/>
       </c>
       <c r="I80" s="120">
-        <f>ROUND(G36*F80*G80,0)</f>
+        <f>ROUND(G34*F80*G80,0)</f>
         <v/>
       </c>
       <c r="J80" s="120">
-        <f>ROUND(H36*F80,0)</f>
+        <f>ROUND(H34*F80,0)</f>
         <v/>
       </c>
       <c r="K80" s="120">
-        <f>ROUND(I36*F80,0)</f>
+        <f>ROUND(I34*F80,0)</f>
         <v/>
       </c>
       <c r="L80" s="121">
@@ -16081,31 +16097,31 @@
     <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="116" t="inlineStr">
         <is>
-          <t>CPO698</t>
+          <t>GPO478</t>
         </is>
       </c>
       <c r="B81" s="116" t="inlineStr">
         <is>
-          <t>2026.05.20</t>
+          <t>2026.05.19</t>
         </is>
       </c>
       <c r="C81" s="117" t="inlineStr">
         <is>
-          <t>Christie</t>
+          <t>GDC</t>
         </is>
       </c>
       <c r="D81" s="118" t="n">
-        <v>4290</v>
+        <v>180</v>
       </c>
       <c r="E81" s="118" t="n">
-        <v>4290</v>
+        <v>180</v>
       </c>
       <c r="F81" s="122">
         <f>D81/E81</f>
         <v/>
       </c>
       <c r="G81" s="118">
-        <f>F37</f>
+        <f>F36</f>
         <v/>
       </c>
       <c r="H81" s="120">
@@ -16113,51 +16129,50 @@
         <v/>
       </c>
       <c r="I81" s="120">
-        <f>ROUND(G37*F81*G81,0)</f>
+        <f>ROUND(G36*F81*G81,0)</f>
         <v/>
       </c>
       <c r="J81" s="120">
-        <f>ROUND(H37*F81,0)</f>
+        <f>ROUND(H36*F81,0)</f>
         <v/>
       </c>
       <c r="K81" s="120">
-        <f>ROUND(I37*F81,0)</f>
+        <f>ROUND(I36*F81,0)</f>
         <v/>
       </c>
       <c r="L81" s="121">
         <f>H81+I81+J81+K81</f>
         <v/>
       </c>
-      <c r="M81" s="40" t="n"/>
     </row>
     <row r="82" ht="15.75" customHeight="1">
       <c r="A82" s="116" t="inlineStr">
         <is>
-          <t>GPO473-1</t>
+          <t>CPO698</t>
         </is>
       </c>
       <c r="B82" s="116" t="inlineStr">
         <is>
-          <t>2026.05.29</t>
+          <t>2026.05.20</t>
         </is>
       </c>
       <c r="C82" s="117" t="inlineStr">
         <is>
-          <t>GDC</t>
+          <t>Christie</t>
         </is>
       </c>
       <c r="D82" s="118" t="n">
-        <v>98800</v>
+        <v>4290</v>
       </c>
       <c r="E82" s="118" t="n">
-        <v>99140</v>
+        <v>4290</v>
       </c>
       <c r="F82" s="122">
         <f>D82/E82</f>
         <v/>
       </c>
       <c r="G82" s="118">
-        <f>F38</f>
+        <f>F37</f>
         <v/>
       </c>
       <c r="H82" s="120">
@@ -16165,26 +16180,27 @@
         <v/>
       </c>
       <c r="I82" s="120">
-        <f>ROUND(G38*F82*G82,0)</f>
+        <f>ROUND(G37*F82*G82,0)</f>
         <v/>
       </c>
       <c r="J82" s="120">
-        <f>ROUND(H38*F82,0)</f>
+        <f>ROUND(H37*F82,0)</f>
         <v/>
       </c>
       <c r="K82" s="120">
-        <f>ROUND(I38*F82,0)</f>
+        <f>ROUND(I37*F82,0)</f>
         <v/>
       </c>
       <c r="L82" s="121">
         <f>H82+I82+J82+K82</f>
         <v/>
       </c>
+      <c r="M82" s="40" t="n"/>
     </row>
     <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="116" t="inlineStr">
         <is>
-          <t>GPO480</t>
+          <t>GPO473-1</t>
         </is>
       </c>
       <c r="B83" s="116" t="inlineStr">
@@ -16198,7 +16214,7 @@
         </is>
       </c>
       <c r="D83" s="118" t="n">
-        <v>250</v>
+        <v>98800</v>
       </c>
       <c r="E83" s="118" t="n">
         <v>99140</v>
@@ -16235,7 +16251,7 @@
     <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="116" t="inlineStr">
         <is>
-          <t>GPO479</t>
+          <t>GPO480</t>
         </is>
       </c>
       <c r="B84" s="116" t="inlineStr">
@@ -16249,7 +16265,7 @@
         </is>
       </c>
       <c r="D84" s="118" t="n">
-        <v>90</v>
+        <v>250</v>
       </c>
       <c r="E84" s="118" t="n">
         <v>99140</v>
@@ -16286,7 +16302,7 @@
     <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="116" t="inlineStr">
         <is>
-          <t>CPO697</t>
+          <t>GPO479</t>
         </is>
       </c>
       <c r="B85" s="116" t="inlineStr">
@@ -16296,21 +16312,21 @@
       </c>
       <c r="C85" s="117" t="inlineStr">
         <is>
-          <t>Christie</t>
+          <t>GDC</t>
         </is>
       </c>
       <c r="D85" s="118" t="n">
-        <v>15289</v>
+        <v>90</v>
       </c>
       <c r="E85" s="118" t="n">
-        <v>101638</v>
+        <v>99140</v>
       </c>
       <c r="F85" s="122">
         <f>D85/E85</f>
         <v/>
       </c>
       <c r="G85" s="118">
-        <f>F39</f>
+        <f>F38</f>
         <v/>
       </c>
       <c r="H85" s="120">
@@ -16318,15 +16334,15 @@
         <v/>
       </c>
       <c r="I85" s="120">
-        <f>ROUND(G39*F85*G85,0)</f>
+        <f>ROUND(G38*F85*G85,0)</f>
         <v/>
       </c>
       <c r="J85" s="120">
-        <f>ROUND(H39*F85,0)</f>
+        <f>ROUND(H38*F85,0)</f>
         <v/>
       </c>
       <c r="K85" s="120">
-        <f>ROUND(I39*F85,0)</f>
+        <f>ROUND(I38*F85,0)</f>
         <v/>
       </c>
       <c r="L85" s="121">
@@ -16337,7 +16353,7 @@
     <row r="86" ht="15.75" customHeight="1">
       <c r="A86" s="116" t="inlineStr">
         <is>
-          <t>CPO696-1</t>
+          <t>CPO697</t>
         </is>
       </c>
       <c r="B86" s="116" t="inlineStr">
@@ -16351,7 +16367,7 @@
         </is>
       </c>
       <c r="D86" s="118" t="n">
-        <v>78209</v>
+        <v>15289</v>
       </c>
       <c r="E86" s="118" t="n">
         <v>101638</v>
@@ -16388,7 +16404,7 @@
     <row r="87" ht="15.75" customHeight="1">
       <c r="A87" s="116" t="inlineStr">
         <is>
-          <t>CPO696-2</t>
+          <t>CPO696-1</t>
         </is>
       </c>
       <c r="B87" s="116" t="inlineStr">
@@ -16402,7 +16418,7 @@
         </is>
       </c>
       <c r="D87" s="118" t="n">
-        <v>8140</v>
+        <v>78209</v>
       </c>
       <c r="E87" s="118" t="n">
         <v>101638</v>
@@ -16436,9 +16452,213 @@
         <v/>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" s="116" t="inlineStr">
+        <is>
+          <t>CPO696-2</t>
+        </is>
+      </c>
+      <c r="B88" s="116" t="inlineStr">
+        <is>
+          <t>2026.05.29</t>
+        </is>
+      </c>
+      <c r="C88" s="117" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="D88" s="118" t="n">
+        <v>8140</v>
+      </c>
+      <c r="E88" s="118" t="n">
+        <v>101638</v>
+      </c>
+      <c r="F88" s="122">
+        <f>D88/E88</f>
+        <v/>
+      </c>
+      <c r="G88" s="118">
+        <f>F39</f>
+        <v/>
+      </c>
+      <c r="H88" s="120">
+        <f>ROUND(D88*G88,0)</f>
+        <v/>
+      </c>
+      <c r="I88" s="120">
+        <f>ROUND(G39*F88*G88,0)</f>
+        <v/>
+      </c>
+      <c r="J88" s="120">
+        <f>ROUND(H39*F88,0)</f>
+        <v/>
+      </c>
+      <c r="K88" s="120">
+        <f>ROUND(I39*F88,0)</f>
+        <v/>
+      </c>
+      <c r="L88" s="121">
+        <f>H88+I88+J88+K88</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="234" t="inlineStr">
+        <is>
+          <t>GPO481</t>
+        </is>
+      </c>
+      <c r="B89" s="234" t="inlineStr">
+        <is>
+          <t>2026.06.10</t>
+        </is>
+      </c>
+      <c r="C89" s="235" t="inlineStr">
+        <is>
+          <t>GDC</t>
+        </is>
+      </c>
+      <c r="D89" s="236" t="n">
+        <v>500</v>
+      </c>
+      <c r="E89" s="236" t="n">
+        <v>119060</v>
+      </c>
+      <c r="F89" s="240">
+        <f>D89/E89</f>
+        <v/>
+      </c>
+      <c r="G89" s="236">
+        <f>F40</f>
+        <v/>
+      </c>
+      <c r="H89" s="238">
+        <f>ROUND(D89*G89,0)</f>
+        <v/>
+      </c>
+      <c r="I89" s="238">
+        <f>ROUND(G40*F89*G89,0)</f>
+        <v/>
+      </c>
+      <c r="J89" s="238">
+        <f>ROUND(H40*F89,0)</f>
+        <v/>
+      </c>
+      <c r="K89" s="238">
+        <f>ROUND(I40*F89,0)</f>
+        <v/>
+      </c>
+      <c r="L89" s="239">
+        <f>H89+I89+J89+K89</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="234" t="inlineStr">
+        <is>
+          <t>GPO473-2</t>
+        </is>
+      </c>
+      <c r="B90" s="234" t="inlineStr">
+        <is>
+          <t>2026.06.10</t>
+        </is>
+      </c>
+      <c r="C90" s="235" t="inlineStr">
+        <is>
+          <t>GDC</t>
+        </is>
+      </c>
+      <c r="D90" s="236" t="n">
+        <v>69160</v>
+      </c>
+      <c r="E90" s="236" t="n">
+        <v>119060</v>
+      </c>
+      <c r="F90" s="240">
+        <f>D90/E90</f>
+        <v/>
+      </c>
+      <c r="G90" s="236">
+        <f>F40</f>
+        <v/>
+      </c>
+      <c r="H90" s="238">
+        <f>ROUND(D90*G90,0)</f>
+        <v/>
+      </c>
+      <c r="I90" s="238">
+        <f>ROUND(G40*F90*G90,0)</f>
+        <v/>
+      </c>
+      <c r="J90" s="238">
+        <f>ROUND(H40*F90,0)</f>
+        <v/>
+      </c>
+      <c r="K90" s="238">
+        <f>ROUND(I40*F90,0)</f>
+        <v/>
+      </c>
+      <c r="L90" s="239">
+        <f>H90+I90+J90+K90</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="234" t="inlineStr">
+        <is>
+          <t>GPO473-3</t>
+        </is>
+      </c>
+      <c r="B91" s="234" t="inlineStr">
+        <is>
+          <t>2026.06.10</t>
+        </is>
+      </c>
+      <c r="C91" s="235" t="inlineStr">
+        <is>
+          <t>GDC</t>
+        </is>
+      </c>
+      <c r="D91" s="236" t="n">
+        <v>49400</v>
+      </c>
+      <c r="E91" s="236" t="n">
+        <v>119060</v>
+      </c>
+      <c r="F91" s="240">
+        <f>D91/E91</f>
+        <v/>
+      </c>
+      <c r="G91" s="236">
+        <f>F40</f>
+        <v/>
+      </c>
+      <c r="H91" s="238">
+        <f>ROUND(D91*G91,0)</f>
+        <v/>
+      </c>
+      <c r="I91" s="238">
+        <f>ROUND(G40*F91*G91,0)</f>
+        <v/>
+      </c>
+      <c r="J91" s="238">
+        <f>ROUND(H40*F91,0)</f>
+        <v/>
+      </c>
+      <c r="K91" s="238">
+        <f>ROUND(I40*F91,0)</f>
+        <v/>
+      </c>
+      <c r="L91" s="239">
+        <f>H91+I91+J91+K91</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A40:L40"/>
+    <mergeCell ref="A41:L41"/>
     <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -16498,7 +16718,7 @@
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="163" t="inlineStr">
         <is>
-          <t>기준일: 2026-06-02  |  미상환 건만 표시  |  상환예정일 = 신한은행 PDF 만기일 기준</t>
+          <t>기준일: 2026-06-10  |  미상환 건만 표시  |  상환예정일 = 신한은행 PDF 만기일 기준</t>
         </is>
       </c>
     </row>
@@ -16899,10 +17119,18 @@
       <c r="L17" s="200" t="n">
         <v>60</v>
       </c>
-      <c r="M17" s="59" t="n"/>
+      <c r="M17" s="59" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="N17" s="201" t="n"/>
       <c r="O17" s="63" t="n"/>
-      <c r="P17" s="59" t="n"/>
+      <c r="P17" s="59" t="inlineStr">
+        <is>
+          <t>6/9 만기 상환 완료 (USD 190,470)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="56" t="inlineStr">
@@ -18445,7 +18673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="15" customWidth="1" style="40" min="1" max="2"/>
@@ -19076,6 +19304,22 @@
       </c>
       <c r="D41" s="211" t="n">
         <v>1507.15</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="210" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B42" s="210" t="n">
+        <v>46186</v>
+      </c>
+      <c r="C42" s="207" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D42" s="211" t="n">
+        <v>1514.68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
latest: Usance 상환 명세
</commit_message>
<xml_diff>
--- a/latest.xlsx
+++ b/latest.xlsx
@@ -24,14 +24,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0&quot;일&quot;"/>
     <numFmt numFmtId="168" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="169" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="27">
     <font>
       <name val="맑은 고딕"/>
       <charset val="129"/>
@@ -193,8 +195,22 @@
       <sz val="11"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color theme="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -292,8 +308,23 @@
         <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -429,11 +460,17 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="245">
+  <cellXfs count="272">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1138,6 +1175,87 @@
     </xf>
     <xf numFmtId="3" fontId="3" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="24" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="24" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="24" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="26" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="26" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="26" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="25" fillId="20" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="25" fillId="20" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="26" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="26" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="26" fillId="20" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="20" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="25" fillId="20" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="25" fillId="20" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1387,6 +1505,28 @@
 </comments>
 </file>
 
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>RNR 재무팀</author>
+  </authors>
+  <commentList>
+    <comment ref="N17" authorId="0" shapeId="0">
+      <text>
+        <t>은행 원금 상환 전표(원화 출금) 미수취
+전표 수취 후 상환환율과 KRW 확정 기입</t>
+      </text>
+    </comment>
+    <comment ref="C27" authorId="0" shapeId="0">
+      <text>
+        <t>신한은행 원금 상환 전표(원화 출금액) 미수취
+수취 즉시 환율/KRW 기입 예정</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -17187,7 +17327,7 @@
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="163" t="inlineStr">
         <is>
-          <t>기준일: 2026-06-10  |  미상환 건만 표시  |  상환예정일 = 신한은행 PDF 만기일 기준</t>
+          <t>기준일: 2026-06-10  |  상환 완료 건은 초록색 표시  |  상환예정일 = 신한은행 PDF 만기일 기준</t>
         </is>
       </c>
     </row>
@@ -17372,7 +17512,7 @@
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="199" t="inlineStr">
         <is>
-          <t>&lt; 미상환 L/C 현황 &gt;</t>
+          <t>&lt; Usance L/C 현황 (상환완료 포함) &gt;</t>
         </is>
       </c>
       <c r="B14" s="148" t="n"/>
@@ -17534,70 +17674,70 @@
       <c r="P16" s="59" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="59" t="n">
+      <c r="A17" s="245" t="n">
         <v>2</v>
       </c>
-      <c r="B17" s="59" t="inlineStr">
+      <c r="B17" s="245" t="inlineStr">
         <is>
           <t>GPO-446-2</t>
         </is>
       </c>
-      <c r="C17" s="74" t="inlineStr">
+      <c r="C17" s="246" t="inlineStr">
         <is>
           <t>GDC</t>
         </is>
       </c>
-      <c r="D17" s="60" t="n">
+      <c r="D17" s="247" t="n">
         <v>190470</v>
       </c>
-      <c r="E17" s="59" t="inlineStr">
+      <c r="E17" s="245" t="inlineStr">
         <is>
           <t>신한은행</t>
         </is>
       </c>
-      <c r="F17" s="59" t="inlineStr">
+      <c r="F17" s="245" t="inlineStr">
         <is>
           <t>M88JX2511NU00018</t>
         </is>
       </c>
-      <c r="G17" s="59" t="inlineStr">
+      <c r="G17" s="245" t="inlineStr">
         <is>
           <t>2025-11-11</t>
         </is>
       </c>
-      <c r="H17" s="59" t="inlineStr">
+      <c r="H17" s="245" t="inlineStr">
         <is>
           <t>2026-05-10</t>
         </is>
       </c>
-      <c r="I17" s="59" t="inlineStr">
+      <c r="I17" s="245" t="inlineStr">
         <is>
           <t>180 Days</t>
         </is>
       </c>
-      <c r="J17" s="59" t="inlineStr">
+      <c r="J17" s="245" t="inlineStr">
         <is>
           <t>2025-12-08</t>
         </is>
       </c>
-      <c r="K17" s="59" t="inlineStr">
+      <c r="K17" s="245" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="L17" s="200" t="n">
-        <v>60</v>
-      </c>
-      <c r="M17" s="59" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="N17" s="201" t="n"/>
-      <c r="O17" s="63" t="n"/>
-      <c r="P17" s="59" t="inlineStr">
-        <is>
-          <t>6/9 만기 상환 완료 (USD 190,470)</t>
+      <c r="L17" s="248" t="inlineStr">
+        <is>
+          <t>상환완료</t>
+        </is>
+      </c>
+      <c r="M17" s="249" t="n">
+        <v>46182</v>
+      </c>
+      <c r="N17" s="250" t="n"/>
+      <c r="O17" s="251" t="n"/>
+      <c r="P17" s="245" t="inlineStr">
+        <is>
+          <t>6/9 만기 상환 완료, 하단 정산 명세 참조</t>
         </is>
       </c>
     </row>
@@ -17855,7 +17995,11 @@
       <c r="P24" s="65" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="65" t="n"/>
+      <c r="A25" s="252" t="inlineStr">
+        <is>
+          <t>&lt; GPO-446-2 상환 정산 및 수수료 명세 (신한은행, 출처: 은행 수수료 내역서 2026-06-09 조회) &gt;</t>
+        </is>
+      </c>
       <c r="B25" s="65" t="n"/>
       <c r="C25" s="66" t="n"/>
       <c r="D25" s="65" t="n"/>
@@ -17873,12 +18017,36 @@
       <c r="P25" s="65" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="65" t="n"/>
-      <c r="B26" s="65" t="n"/>
-      <c r="C26" s="66" t="n"/>
-      <c r="D26" s="65" t="n"/>
-      <c r="E26" s="65" t="n"/>
-      <c r="F26" s="65" t="n"/>
+      <c r="A26" s="253" t="inlineStr">
+        <is>
+          <t>상환일</t>
+        </is>
+      </c>
+      <c r="B26" s="253" t="inlineStr">
+        <is>
+          <t>상환원금(USD)</t>
+        </is>
+      </c>
+      <c r="C26" s="253" t="inlineStr">
+        <is>
+          <t>상환환율(₩)</t>
+        </is>
+      </c>
+      <c r="D26" s="253" t="inlineStr">
+        <is>
+          <t>상환금액(KRW)</t>
+        </is>
+      </c>
+      <c r="E26" s="253" t="inlineStr">
+        <is>
+          <t>L/C No.</t>
+        </is>
+      </c>
+      <c r="F26" s="253" t="inlineStr">
+        <is>
+          <t>회계처리(권장)</t>
+        </is>
+      </c>
       <c r="G26" s="65" t="n"/>
       <c r="H26" s="65" t="n"/>
       <c r="I26" s="65" t="n"/>
@@ -17891,12 +18059,32 @@
       <c r="P26" s="65" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1">
-      <c r="A27" s="65" t="n"/>
-      <c r="B27" s="65" t="n"/>
-      <c r="C27" s="66" t="n"/>
-      <c r="D27" s="65" t="n"/>
-      <c r="E27" s="65" t="n"/>
-      <c r="F27" s="70" t="n"/>
+      <c r="A27" s="254" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B27" s="255" t="n">
+        <v>190470</v>
+      </c>
+      <c r="C27" s="256" t="inlineStr">
+        <is>
+          <t>전표 확인 필요</t>
+        </is>
+      </c>
+      <c r="D27" s="256" t="inlineStr">
+        <is>
+          <t>전표 확인 필요</t>
+        </is>
+      </c>
+      <c r="E27" s="257" t="inlineStr">
+        <is>
+          <t>M88JX2511NU00018</t>
+        </is>
+      </c>
+      <c r="F27" s="258" t="inlineStr">
+        <is>
+          <t>차변 외화매입채무 190,470 USD, 대변 보통예금(상환환율), 차액 외환차손익</t>
+        </is>
+      </c>
       <c r="G27" s="71" t="n"/>
       <c r="H27" s="65" t="n"/>
       <c r="I27" s="65" t="n"/>
@@ -17927,16 +18115,56 @@
       <c r="P28" s="65" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="65" t="n"/>
-      <c r="B29" s="65" t="n"/>
-      <c r="C29" s="66" t="n"/>
-      <c r="D29" s="65" t="n"/>
-      <c r="E29" s="65" t="n"/>
-      <c r="F29" s="70" t="n"/>
-      <c r="G29" s="71" t="n"/>
-      <c r="H29" s="65" t="n"/>
-      <c r="I29" s="65" t="n"/>
-      <c r="J29" s="65" t="n"/>
+      <c r="A29" s="253" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B29" s="253" t="inlineStr">
+        <is>
+          <t>징수일</t>
+        </is>
+      </c>
+      <c r="C29" s="253" t="inlineStr">
+        <is>
+          <t>수수료 구분</t>
+        </is>
+      </c>
+      <c r="D29" s="253" t="inlineStr">
+        <is>
+          <t>이율(%)</t>
+        </is>
+      </c>
+      <c r="E29" s="253" t="inlineStr">
+        <is>
+          <t>수수료 기간</t>
+        </is>
+      </c>
+      <c r="F29" s="259" t="inlineStr">
+        <is>
+          <t>일수</t>
+        </is>
+      </c>
+      <c r="G29" s="260" t="inlineStr">
+        <is>
+          <t>대상금액(USD)</t>
+        </is>
+      </c>
+      <c r="H29" s="253" t="inlineStr">
+        <is>
+          <t>USD 상당액</t>
+        </is>
+      </c>
+      <c r="I29" s="253" t="inlineStr">
+        <is>
+          <t>징수액(KRW)</t>
+        </is>
+      </c>
+      <c r="J29" s="253" t="inlineStr">
+        <is>
+          <t>회계처리(권장)</t>
+        </is>
+      </c>
       <c r="K29" s="65" t="n"/>
       <c r="L29" s="65" t="n"/>
       <c r="M29" s="65" t="n"/>
@@ -17945,16 +18173,42 @@
       <c r="P29" s="65" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="65" t="n"/>
-      <c r="B30" s="65" t="n"/>
-      <c r="C30" s="66" t="n"/>
-      <c r="D30" s="65" t="n"/>
-      <c r="E30" s="65" t="n"/>
-      <c r="F30" s="70" t="n"/>
-      <c r="G30" s="71" t="n"/>
-      <c r="H30" s="65" t="n"/>
-      <c r="I30" s="65" t="n"/>
-      <c r="J30" s="65" t="n"/>
+      <c r="A30" s="257" t="n">
+        <v>1</v>
+      </c>
+      <c r="B30" s="254" t="n">
+        <v>45971</v>
+      </c>
+      <c r="C30" s="261" t="inlineStr">
+        <is>
+          <t>수입신용장 기간수수료(발행수수료, 360일 단위)</t>
+        </is>
+      </c>
+      <c r="D30" s="262" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E30" s="257" t="inlineStr">
+        <is>
+          <t>2025-11-10 ~ 2025-12-26</t>
+        </is>
+      </c>
+      <c r="F30" s="263" t="n">
+        <v>47</v>
+      </c>
+      <c r="G30" s="255" t="n">
+        <v>190470</v>
+      </c>
+      <c r="H30" s="255" t="n">
+        <v>198.94</v>
+      </c>
+      <c r="I30" s="264" t="n">
+        <v>289132</v>
+      </c>
+      <c r="J30" s="257" t="inlineStr">
+        <is>
+          <t>지급수수료</t>
+        </is>
+      </c>
       <c r="K30" s="65" t="n"/>
       <c r="L30" s="65" t="n"/>
       <c r="M30" s="65" t="n"/>
@@ -17963,16 +18217,32 @@
       <c r="P30" s="65" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1">
-      <c r="A31" s="65" t="n"/>
-      <c r="B31" s="65" t="n"/>
-      <c r="C31" s="66" t="n"/>
-      <c r="D31" s="65" t="n"/>
-      <c r="E31" s="65" t="n"/>
-      <c r="F31" s="70" t="n"/>
-      <c r="G31" s="71" t="n"/>
-      <c r="H31" s="65" t="n"/>
-      <c r="I31" s="65" t="n"/>
-      <c r="J31" s="65" t="n"/>
+      <c r="A31" s="257" t="n">
+        <v>2</v>
+      </c>
+      <c r="B31" s="254" t="n">
+        <v>45971</v>
+      </c>
+      <c r="C31" s="261" t="inlineStr">
+        <is>
+          <t>전신료(일반신용장 USANCE)</t>
+        </is>
+      </c>
+      <c r="D31" s="262" t="n"/>
+      <c r="E31" s="257" t="inlineStr"/>
+      <c r="F31" s="263" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="255" t="n"/>
+      <c r="H31" s="255" t="n"/>
+      <c r="I31" s="264" t="n">
+        <v>13750</v>
+      </c>
+      <c r="J31" s="257" t="inlineStr">
+        <is>
+          <t>지급수수료</t>
+        </is>
+      </c>
       <c r="K31" s="65" t="n"/>
       <c r="L31" s="65" t="n"/>
       <c r="M31" s="65" t="n"/>
@@ -17981,16 +18251,32 @@
       <c r="P31" s="65" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1">
-      <c r="A32" s="65" t="n"/>
-      <c r="B32" s="65" t="n"/>
-      <c r="C32" s="66" t="n"/>
-      <c r="D32" s="65" t="n"/>
-      <c r="E32" s="65" t="n"/>
-      <c r="F32" s="70" t="n"/>
-      <c r="G32" s="71" t="n"/>
-      <c r="H32" s="65" t="n"/>
-      <c r="I32" s="65" t="n"/>
-      <c r="J32" s="65" t="n"/>
+      <c r="A32" s="257" t="n">
+        <v>3</v>
+      </c>
+      <c r="B32" s="254" t="n">
+        <v>45980</v>
+      </c>
+      <c r="C32" s="261" t="inlineStr">
+        <is>
+          <t>수입화물선취보증서(L/G) 발급수수료</t>
+        </is>
+      </c>
+      <c r="D32" s="262" t="n"/>
+      <c r="E32" s="257" t="inlineStr"/>
+      <c r="F32" s="263" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="255" t="n"/>
+      <c r="H32" s="255" t="n"/>
+      <c r="I32" s="264" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J32" s="257" t="inlineStr">
+        <is>
+          <t>지급수수료</t>
+        </is>
+      </c>
       <c r="K32" s="65" t="n"/>
       <c r="L32" s="65" t="n"/>
       <c r="M32" s="65" t="n"/>
@@ -17999,16 +18285,42 @@
       <c r="P32" s="65" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1">
-      <c r="A33" s="65" t="n"/>
-      <c r="B33" s="65" t="n"/>
-      <c r="C33" s="66" t="n"/>
-      <c r="D33" s="65" t="n"/>
-      <c r="E33" s="65" t="n"/>
-      <c r="F33" s="70" t="n"/>
-      <c r="G33" s="71" t="n"/>
-      <c r="H33" s="65" t="n"/>
-      <c r="I33" s="65" t="n"/>
-      <c r="J33" s="65" t="n"/>
+      <c r="A33" s="257" t="n">
+        <v>4</v>
+      </c>
+      <c r="B33" s="254" t="n">
+        <v>45999</v>
+      </c>
+      <c r="C33" s="261" t="inlineStr">
+        <is>
+          <t>수입화물선취보증료(외화)</t>
+        </is>
+      </c>
+      <c r="D33" s="262" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" s="257" t="inlineStr">
+        <is>
+          <t>2025-11-19 ~ 2025-12-07</t>
+        </is>
+      </c>
+      <c r="F33" s="263" t="n">
+        <v>19</v>
+      </c>
+      <c r="G33" s="255" t="n">
+        <v>190470</v>
+      </c>
+      <c r="H33" s="255" t="n">
+        <v>301.58</v>
+      </c>
+      <c r="I33" s="264" t="n">
+        <v>442866</v>
+      </c>
+      <c r="J33" s="257" t="inlineStr">
+        <is>
+          <t>지급수수료</t>
+        </is>
+      </c>
       <c r="K33" s="65" t="n"/>
       <c r="L33" s="65" t="n"/>
       <c r="M33" s="65" t="n"/>
@@ -18017,16 +18329,42 @@
       <c r="P33" s="65" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1">
-      <c r="A34" s="65" t="n"/>
-      <c r="B34" s="65" t="n"/>
-      <c r="C34" s="66" t="n"/>
-      <c r="D34" s="65" t="n"/>
-      <c r="E34" s="65" t="n"/>
-      <c r="F34" s="70" t="n"/>
-      <c r="G34" s="71" t="n"/>
-      <c r="H34" s="65" t="n"/>
-      <c r="I34" s="65" t="n"/>
-      <c r="J34" s="65" t="n"/>
+      <c r="A34" s="257" t="n">
+        <v>5</v>
+      </c>
+      <c r="B34" s="254" t="n">
+        <v>45999</v>
+      </c>
+      <c r="C34" s="261" t="inlineStr">
+        <is>
+          <t>수입인수수수료(360일 단위)</t>
+        </is>
+      </c>
+      <c r="D34" s="262" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E34" s="257" t="inlineStr">
+        <is>
+          <t>2025-12-08 ~ 2026-05-31</t>
+        </is>
+      </c>
+      <c r="F34" s="263" t="n">
+        <v>175</v>
+      </c>
+      <c r="G34" s="255" t="n">
+        <v>190470</v>
+      </c>
+      <c r="H34" s="255" t="n">
+        <v>1111.08</v>
+      </c>
+      <c r="I34" s="264" t="n">
+        <v>1631613</v>
+      </c>
+      <c r="J34" s="257" t="inlineStr">
+        <is>
+          <t>이자비용</t>
+        </is>
+      </c>
       <c r="K34" s="65" t="n"/>
       <c r="L34" s="65" t="n"/>
       <c r="M34" s="65" t="n"/>
@@ -18035,16 +18373,42 @@
       <c r="P34" s="65" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1">
-      <c r="A35" s="65" t="n"/>
-      <c r="B35" s="65" t="n"/>
-      <c r="C35" s="66" t="n"/>
-      <c r="D35" s="65" t="n"/>
-      <c r="E35" s="65" t="n"/>
-      <c r="F35" s="70" t="n"/>
-      <c r="G35" s="71" t="n"/>
-      <c r="H35" s="65" t="n"/>
-      <c r="I35" s="65" t="n"/>
-      <c r="J35" s="65" t="n"/>
+      <c r="A35" s="257" t="n">
+        <v>6</v>
+      </c>
+      <c r="B35" s="254" t="n">
+        <v>45999</v>
+      </c>
+      <c r="C35" s="261" t="inlineStr">
+        <is>
+          <t>수입기간수수료 환급(-)</t>
+        </is>
+      </c>
+      <c r="D35" s="262" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E35" s="257" t="inlineStr">
+        <is>
+          <t>2025-12-08 ~ 2025-12-26</t>
+        </is>
+      </c>
+      <c r="F35" s="263" t="n">
+        <v>19</v>
+      </c>
+      <c r="G35" s="255" t="n">
+        <v>190470</v>
+      </c>
+      <c r="H35" s="255" t="n">
+        <v>-80.42</v>
+      </c>
+      <c r="I35" s="264" t="n">
+        <v>-116883</v>
+      </c>
+      <c r="J35" s="257" t="inlineStr">
+        <is>
+          <t>지급수수료 차감</t>
+        </is>
+      </c>
       <c r="K35" s="65" t="n"/>
       <c r="L35" s="65" t="n"/>
       <c r="M35" s="65" t="n"/>
@@ -18053,16 +18417,42 @@
       <c r="P35" s="65" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1">
-      <c r="A36" s="65" t="n"/>
-      <c r="B36" s="65" t="n"/>
-      <c r="C36" s="66" t="n"/>
-      <c r="D36" s="65" t="n"/>
-      <c r="E36" s="65" t="n"/>
-      <c r="F36" s="70" t="n"/>
-      <c r="G36" s="71" t="n"/>
-      <c r="H36" s="65" t="n"/>
-      <c r="I36" s="65" t="n"/>
-      <c r="J36" s="65" t="n"/>
+      <c r="A36" s="257" t="n">
+        <v>7</v>
+      </c>
+      <c r="B36" s="254" t="n">
+        <v>46182</v>
+      </c>
+      <c r="C36" s="261" t="inlineStr">
+        <is>
+          <t>수입인수수수료(만기연장 8일분)</t>
+        </is>
+      </c>
+      <c r="D36" s="262" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E36" s="257" t="inlineStr">
+        <is>
+          <t>2026-06-01 ~ 2026-06-08</t>
+        </is>
+      </c>
+      <c r="F36" s="263" t="n">
+        <v>8</v>
+      </c>
+      <c r="G36" s="255" t="n">
+        <v>190470</v>
+      </c>
+      <c r="H36" s="255" t="n">
+        <v>50.79</v>
+      </c>
+      <c r="I36" s="264" t="n">
+        <v>77732</v>
+      </c>
+      <c r="J36" s="257" t="inlineStr">
+        <is>
+          <t>이자비용</t>
+        </is>
+      </c>
       <c r="K36" s="65" t="n"/>
       <c r="L36" s="65" t="n"/>
       <c r="M36" s="65" t="n"/>
@@ -18071,16 +18461,28 @@
       <c r="P36" s="65" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1">
-      <c r="A37" s="65" t="n"/>
-      <c r="B37" s="65" t="n"/>
-      <c r="C37" s="66" t="n"/>
-      <c r="D37" s="65" t="n"/>
-      <c r="E37" s="65" t="n"/>
-      <c r="F37" s="70" t="n"/>
-      <c r="G37" s="71" t="n"/>
-      <c r="H37" s="65" t="n"/>
-      <c r="I37" s="65" t="n"/>
-      <c r="J37" s="65" t="n"/>
+      <c r="A37" s="253" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+      <c r="B37" s="265" t="n"/>
+      <c r="C37" s="266" t="n"/>
+      <c r="D37" s="265" t="n"/>
+      <c r="E37" s="265" t="n"/>
+      <c r="F37" s="267" t="n"/>
+      <c r="G37" s="268" t="n"/>
+      <c r="H37" s="269" t="n">
+        <v>1581.97</v>
+      </c>
+      <c r="I37" s="270" t="n">
+        <v>2343210</v>
+      </c>
+      <c r="J37" s="253" t="inlineStr">
+        <is>
+          <t>이자비용 1,709,345 + 지급수수료 633,865</t>
+        </is>
+      </c>
       <c r="K37" s="65" t="n"/>
       <c r="L37" s="65" t="n"/>
       <c r="M37" s="65" t="n"/>
@@ -18089,7 +18491,11 @@
       <c r="P37" s="65" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="65" t="n"/>
+      <c r="A38" s="271" t="inlineStr">
+        <is>
+          <t>주1: USD 상당액 = 대상금액 x 이율 x 일수/360 (정액 항목인 전신료, 발급수수료는 KRW 정액 징수로 USD 산식 없음)</t>
+        </is>
+      </c>
       <c r="B38" s="65" t="n"/>
       <c r="C38" s="66" t="n"/>
       <c r="D38" s="65" t="n"/>
@@ -18107,7 +18513,11 @@
       <c r="P38" s="65" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1">
-      <c r="A39" s="65" t="n"/>
+      <c r="A39" s="271" t="inlineStr">
+        <is>
+          <t>주2: 수수료는 전액 KRW로 기징수됨 (징수일 기준). 회계처리 시 징수일자 전표로 계상</t>
+        </is>
+      </c>
       <c r="B39" s="65" t="n"/>
       <c r="C39" s="66" t="n"/>
       <c r="D39" s="65" t="n"/>
@@ -18125,7 +18535,11 @@
       <c r="P39" s="65" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1">
-      <c r="A40" s="65" t="n"/>
+      <c r="A40" s="271" t="inlineStr">
+        <is>
+          <t>주3: 원금 상환(6/9) 전표 수취 후 상환환율, KRW 확정 기입 예정. 회계처리는 외화매입채무 제거 및 외환차손익 인식</t>
+        </is>
+      </c>
       <c r="B40" s="65" t="n"/>
       <c r="C40" s="66" t="n"/>
       <c r="D40" s="65" t="n"/>
@@ -19133,6 +19547,7 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
latest: GPO-446-2 상환 확정
</commit_message>
<xml_diff>
--- a/latest.xlsx
+++ b/latest.xlsx
@@ -24,7 +24,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -32,6 +32,7 @@
     <numFmt numFmtId="168" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="169" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
+    <numFmt numFmtId="171" formatCode="0.00000"/>
   </numFmts>
   <fonts count="27">
     <font>
@@ -324,7 +325,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -466,11 +467,12 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="272">
+  <cellXfs count="276">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1257,6 +1259,16 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="3" fontId="24" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="26" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -1505,28 +1517,6 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>RNR 재무팀</author>
-  </authors>
-  <commentList>
-    <comment ref="N17" authorId="0" shapeId="0">
-      <text>
-        <t>은행 원금 상환 전표(원화 출금) 미수취
-전표 수취 후 상환환율과 KRW 확정 기입</t>
-      </text>
-    </comment>
-    <comment ref="C27" authorId="0" shapeId="0">
-      <text>
-        <t>신한은행 원금 상환 전표(원화 출금액) 미수취
-수취 즉시 환율/KRW 기입 예정</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -17733,11 +17723,15 @@
       <c r="M17" s="249" t="n">
         <v>46182</v>
       </c>
-      <c r="N17" s="250" t="n"/>
-      <c r="O17" s="251" t="n"/>
+      <c r="N17" s="247" t="n">
+        <v>1535.1</v>
+      </c>
+      <c r="O17" s="272" t="n">
+        <v>292390497</v>
+      </c>
       <c r="P17" s="245" t="inlineStr">
         <is>
-          <t>6/9 만기 상환 완료, 하단 정산 명세 참조</t>
+          <t>6/9 만기 상환 완료 (전표 2026-06-09, 승인 402875686), 하단 정산 명세 참조</t>
         </is>
       </c>
     </row>
@@ -18065,15 +18059,11 @@
       <c r="B27" s="255" t="n">
         <v>190470</v>
       </c>
-      <c r="C27" s="256" t="inlineStr">
-        <is>
-          <t>전표 확인 필요</t>
-        </is>
-      </c>
-      <c r="D27" s="256" t="inlineStr">
-        <is>
-          <t>전표 확인 필요</t>
-        </is>
+      <c r="C27" s="255" t="n">
+        <v>1535.1</v>
+      </c>
+      <c r="D27" s="264" t="n">
+        <v>292390497</v>
       </c>
       <c r="E27" s="257" t="inlineStr">
         <is>
@@ -18082,7 +18072,7 @@
       </c>
       <c r="F27" s="258" t="inlineStr">
         <is>
-          <t>차변 외화매입채무 190,470 USD, 대변 보통예금(상환환율), 차액 외환차손익</t>
+          <t>차변 외화매입채무(USANCE) 190,470 USD 제거 + 외환차손익, 대변 보통예금 292,390,497</t>
         </is>
       </c>
       <c r="G27" s="71" t="n"/>
@@ -18461,26 +18451,36 @@
       <c r="P36" s="65" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1">
-      <c r="A37" s="253" t="inlineStr">
-        <is>
-          <t>합계</t>
-        </is>
-      </c>
-      <c r="B37" s="265" t="n"/>
-      <c r="C37" s="266" t="n"/>
-      <c r="D37" s="265" t="n"/>
-      <c r="E37" s="265" t="n"/>
-      <c r="F37" s="267" t="n"/>
-      <c r="G37" s="268" t="n"/>
-      <c r="H37" s="269" t="n">
-        <v>1581.97</v>
-      </c>
-      <c r="I37" s="270" t="n">
-        <v>2343210</v>
-      </c>
-      <c r="J37" s="253" t="inlineStr">
-        <is>
-          <t>이자비용 1,709,345 + 지급수수료 633,865</t>
+      <c r="A37" s="257" t="n">
+        <v>8</v>
+      </c>
+      <c r="B37" s="254" t="n">
+        <v>46182</v>
+      </c>
+      <c r="C37" s="261" t="inlineStr">
+        <is>
+          <t>지체료 (인수수수료 연체이자 7%, 8일)</t>
+        </is>
+      </c>
+      <c r="D37" s="262" t="n">
+        <v>7</v>
+      </c>
+      <c r="E37" s="257" t="inlineStr">
+        <is>
+          <t>2026-06-01 ~ 2026-06-08</t>
+        </is>
+      </c>
+      <c r="F37" s="263" t="n">
+        <v>8</v>
+      </c>
+      <c r="G37" s="255" t="n"/>
+      <c r="H37" s="255" t="n"/>
+      <c r="I37" s="264" t="n">
+        <v>119</v>
+      </c>
+      <c r="J37" s="257" t="inlineStr">
+        <is>
+          <t>이자비용</t>
         </is>
       </c>
       <c r="K37" s="65" t="n"/>
@@ -18491,20 +18491,42 @@
       <c r="P37" s="65" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="271" t="inlineStr">
-        <is>
-          <t>주1: USD 상당액 = 대상금액 x 이율 x 일수/360 (정액 항목인 전신료, 발급수수료는 KRW 정액 징수로 USD 산식 없음)</t>
-        </is>
-      </c>
-      <c r="B38" s="65" t="n"/>
-      <c r="C38" s="66" t="n"/>
-      <c r="D38" s="65" t="n"/>
-      <c r="E38" s="65" t="n"/>
-      <c r="F38" s="70" t="n"/>
-      <c r="G38" s="71" t="n"/>
-      <c r="H38" s="65" t="n"/>
-      <c r="I38" s="65" t="n"/>
-      <c r="J38" s="65" t="n"/>
+      <c r="A38" s="257" t="n">
+        <v>9</v>
+      </c>
+      <c r="B38" s="254" t="n">
+        <v>46182</v>
+      </c>
+      <c r="C38" s="261" t="inlineStr">
+        <is>
+          <t>해외수수료 (해외은행 인수금융 이자 5.57788%, 180일)</t>
+        </is>
+      </c>
+      <c r="D38" s="273" t="n">
+        <v>5.57788</v>
+      </c>
+      <c r="E38" s="257" t="inlineStr">
+        <is>
+          <t>2025-12-11 ~ 2026-06-09</t>
+        </is>
+      </c>
+      <c r="F38" s="263" t="n">
+        <v>180</v>
+      </c>
+      <c r="G38" s="255" t="n">
+        <v>190400</v>
+      </c>
+      <c r="H38" s="255" t="n">
+        <v>5310.14</v>
+      </c>
+      <c r="I38" s="264" t="n">
+        <v>8154250</v>
+      </c>
+      <c r="J38" s="257" t="inlineStr">
+        <is>
+          <t>이자비용</t>
+        </is>
+      </c>
       <c r="K38" s="65" t="n"/>
       <c r="L38" s="65" t="n"/>
       <c r="M38" s="65" t="n"/>
@@ -18513,20 +18535,28 @@
       <c r="P38" s="65" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1">
-      <c r="A39" s="271" t="inlineStr">
-        <is>
-          <t>주2: 수수료는 전액 KRW로 기징수됨 (징수일 기준). 회계처리 시 징수일자 전표로 계상</t>
-        </is>
-      </c>
-      <c r="B39" s="65" t="n"/>
-      <c r="C39" s="66" t="n"/>
-      <c r="D39" s="65" t="n"/>
-      <c r="E39" s="65" t="n"/>
-      <c r="F39" s="65" t="n"/>
-      <c r="G39" s="71" t="n"/>
-      <c r="H39" s="65" t="n"/>
-      <c r="I39" s="65" t="n"/>
-      <c r="J39" s="65" t="n"/>
+      <c r="A39" s="253" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+      <c r="B39" s="265" t="n"/>
+      <c r="C39" s="266" t="n"/>
+      <c r="D39" s="265" t="n"/>
+      <c r="E39" s="265" t="n"/>
+      <c r="F39" s="265" t="n"/>
+      <c r="G39" s="268" t="n"/>
+      <c r="H39" s="269" t="n">
+        <v>6892.11</v>
+      </c>
+      <c r="I39" s="270" t="n">
+        <v>10497579</v>
+      </c>
+      <c r="J39" s="253" t="inlineStr">
+        <is>
+          <t>이자비용 9,863,714 + 지급수수료 633,865</t>
+        </is>
+      </c>
       <c r="K39" s="65" t="n"/>
       <c r="L39" s="65" t="n"/>
       <c r="M39" s="65" t="n"/>
@@ -18535,9 +18565,9 @@
       <c r="P39" s="65" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1">
-      <c r="A40" s="271" t="inlineStr">
-        <is>
-          <t>주3: 원금 상환(6/9) 전표 수취 후 상환환율, KRW 확정 기입 예정. 회계처리는 외화매입채무 제거 및 외환차손익 인식</t>
+      <c r="A40" s="274" t="inlineStr">
+        <is>
+          <t>주1: USD 상당액 = 대상금액 x 이율 x 일수/360 (전신료, 발급수수료, 지체료는 KRW 정액 또는 KRW 기준 산출)</t>
         </is>
       </c>
       <c r="B40" s="65" t="n"/>
@@ -18557,7 +18587,11 @@
       <c r="P40" s="65" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1">
-      <c r="A41" s="65" t="n"/>
+      <c r="A41" s="274" t="inlineStr">
+        <is>
+          <t>주2: No.1~6 수수료는 징수일에 KRW 기징수, No.7~9는 상환일(6/9) 출금. 회계처리는 각 징수일자 전표로 계상</t>
+        </is>
+      </c>
       <c r="B41" s="65" t="n"/>
       <c r="C41" s="66" t="n"/>
       <c r="D41" s="65" t="n"/>
@@ -18574,8 +18608,20 @@
       <c r="O41" s="65" t="n"/>
       <c r="P41" s="65" t="n"/>
     </row>
-    <row r="42" ht="15.75" customHeight="1"/>
-    <row r="43" ht="15.75" customHeight="1"/>
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="A42" s="275" t="inlineStr">
+        <is>
+          <t>주3: 원금 상환 확정 (외국환 거래계산서 2026-06-09, 승인번호 402875686, REF M88JX2511NU00018): 원금 USD 190,470.00 x 1,535.10 = 292,390,497원</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="A43" s="275" t="inlineStr">
+        <is>
+          <t>주4: 6/9 실제 출금 합계 300,622,598원 = 원금분 292,468,348 (원금 + 인수수수료 77,732 + 지체료 119) + 해외수수료분 8,154,250</t>
+        </is>
+      </c>
+    </row>
     <row r="44" ht="15.75" customHeight="1"/>
     <row r="45" ht="15.75" customHeight="1"/>
     <row r="46" ht="15.75" customHeight="1"/>
@@ -19547,7 +19593,6 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Update latest.xlsx 2026-06-16 15:21
</commit_message>
<xml_diff>
--- a/latest.xlsx
+++ b/latest.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" tabRatio="500" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="PO별 개당 수입원가" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="라이센스_워런티" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="합배송_비용안분" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="외화송금내역" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Usance_LC" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="환율" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PO별 개당 수입원가" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="라이센스_워런티" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="합배송_비용안분" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="외화송금내역" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usance_LC" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="환율" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="RemitTable1">'외화송금내역'!$A$3:$L$40</definedName>
     <definedName name="RemitTable2">'외화송금내역'!$A$43:$L$91</definedName>
-    <definedName name="FxRateTable">'환율'!$A$7:$D$42</definedName>
+    <definedName name="FxRateTable">환율!$A$7:$D$43</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="276">
+  <cellXfs count="283">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1269,6 +1269,27 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="24" fillId="18" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="24" fillId="18" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="18" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="24" fillId="18" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -1767,7 +1788,7 @@
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="170" t="inlineStr">
         <is>
-          <t>회계처리용 통합 데이터  |  기준일: 2026-06-10  |  노란색=미확인  |  보라색=라이센스/워런티  |  날짜→해당항목 좌측 배치</t>
+          <t>회계처리용 통합 데이터  |  기준일: 2026-06-16  |  노란색=미확인  |  보라색=라이센스/워런티  |  날짜→해당항목 좌측 배치</t>
         </is>
       </c>
       <c r="B2" s="148" t="n"/>
@@ -2055,24 +2076,20 @@
       <c r="H5" s="7" t="n">
         <v>6800</v>
       </c>
-      <c r="I5" s="33">
-        <f>IFERROR(VLOOKUP(B5,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I5" s="33" t="n">
+        <v>1475.2</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="9">
-        <f>IFERROR(ROUND(H5*I5,0),0)</f>
-        <v/>
-      </c>
-      <c r="L5" s="9">
-        <f>IFERROR(VLOOKUP(B5,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M5" s="9">
-        <f>IFERROR(VLOOKUP(B5,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>10031360</v>
+      </c>
+      <c r="K5" s="9" t="n">
+        <v>10031360</v>
+      </c>
+      <c r="L5" s="9" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M5" s="9" t="n">
+        <v>8000</v>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
@@ -2184,24 +2201,20 @@
       <c r="H6" s="7" t="n">
         <v>139083</v>
       </c>
-      <c r="I6" s="33">
-        <f>IFERROR(VLOOKUP(B6,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I6" s="33" t="n">
+        <v>1479.7</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>212471386</v>
-      </c>
-      <c r="K6" s="9">
-        <f>IFERROR(ROUND(H6*I6,0),0)</f>
-        <v/>
-      </c>
-      <c r="L6" s="9">
-        <f>IFERROR(VLOOKUP(B6,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M6" s="9">
-        <f>IFERROR(VLOOKUP(B6,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>205801115</v>
+      </c>
+      <c r="K6" s="9" t="n">
+        <v>205801115</v>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>12110</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>7751</v>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
@@ -2315,24 +2328,20 @@
       <c r="H7" s="7" t="n">
         <v>9060</v>
       </c>
-      <c r="I7" s="33">
-        <f>IFERROR(VLOOKUP(B7,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I7" s="33" t="n">
+        <v>1439.1</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>18264679</v>
-      </c>
-      <c r="K7" s="9">
-        <f>IFERROR(ROUND(H7*I7,0),0)</f>
-        <v/>
-      </c>
-      <c r="L7" s="9">
-        <f>IFERROR(VLOOKUP(B7,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M7" s="9">
-        <f>IFERROR(VLOOKUP(B7,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>13038246</v>
+      </c>
+      <c r="K7" s="9" t="n">
+        <v>13038246</v>
+      </c>
+      <c r="L7" s="9" t="n">
+        <v>6537</v>
+      </c>
+      <c r="M7" s="9" t="n">
+        <v>5229</v>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
@@ -2446,24 +2455,20 @@
       <c r="H8" s="7" t="n">
         <v>4474</v>
       </c>
-      <c r="I8" s="33">
-        <f>IFERROR(VLOOKUP(B8,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I8" s="33" t="n">
+        <v>1479.7</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>212471386</v>
-      </c>
-      <c r="K8" s="9">
-        <f>IFERROR(ROUND(H8*I8,0),0)</f>
-        <v/>
-      </c>
-      <c r="L8" s="9">
-        <f>IFERROR(VLOOKUP(B8,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M8" s="9">
-        <f>IFERROR(VLOOKUP(B8,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>6620178</v>
+      </c>
+      <c r="K8" s="9" t="n">
+        <v>6620178</v>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>390</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>249</v>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
@@ -2692,24 +2697,20 @@
       <c r="H10" s="7" t="n">
         <v>252</v>
       </c>
-      <c r="I10" s="33">
-        <f>IFERROR(VLOOKUP(B10,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I10" s="33" t="n">
+        <v>1479</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>412788</v>
-      </c>
-      <c r="K10" s="9">
-        <f>IFERROR(ROUND(H10*I10,0),0)</f>
-        <v/>
-      </c>
-      <c r="L10" s="9">
-        <f>IFERROR(VLOOKUP(B10,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M10" s="9">
-        <f>IFERROR(VLOOKUP(B10,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>372708</v>
+      </c>
+      <c r="K10" s="9" t="n">
+        <v>372708</v>
+      </c>
+      <c r="L10" s="9" t="n">
+        <v>2500</v>
+      </c>
+      <c r="M10" s="9" t="n">
+        <v>8000</v>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
@@ -2823,24 +2824,20 @@
       <c r="H11" s="7" t="n">
         <v>2710</v>
       </c>
-      <c r="I11" s="33">
-        <f>IFERROR(VLOOKUP(B11,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I11" s="33" t="n">
+        <v>1475.7</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>5505104</v>
-      </c>
-      <c r="K11" s="9">
-        <f>IFERROR(ROUND(H11*I11,0),0)</f>
-        <v/>
-      </c>
-      <c r="L11" s="9">
-        <f>IFERROR(VLOOKUP(B11,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M11" s="9">
-        <f>IFERROR(VLOOKUP(B11,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>3999147</v>
+      </c>
+      <c r="K11" s="9" t="n">
+        <v>3999147</v>
+      </c>
+      <c r="L11" s="9" t="n">
+        <v>5493</v>
+      </c>
+      <c r="M11" s="9" t="n">
+        <v>5859</v>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
@@ -2954,24 +2951,20 @@
       <c r="H12" s="7" t="n">
         <v>5056.8</v>
       </c>
-      <c r="I12" s="33">
-        <f>IFERROR(VLOOKUP(B12,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I12" s="33" t="n">
+        <v>1445.5</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>7356514</v>
-      </c>
-      <c r="K12" s="9">
-        <f>IFERROR(ROUND(H12*I12,0),0)</f>
-        <v/>
-      </c>
-      <c r="L12" s="9">
-        <f>IFERROR(VLOOKUP(B12,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M12" s="9">
-        <f>IFERROR(VLOOKUP(B12,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>7309604</v>
+      </c>
+      <c r="K12" s="9" t="n">
+        <v>7309604</v>
+      </c>
+      <c r="L12" s="9" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M12" s="9" t="n">
+        <v>8000</v>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
@@ -3085,24 +3078,20 @@
       <c r="H13" s="7" t="n">
         <v>137850</v>
       </c>
-      <c r="I13" s="33">
-        <f>IFERROR(VLOOKUP(B13,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I13" s="33" t="n">
+        <v>1477.6</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>203737212</v>
-      </c>
-      <c r="K13" s="9">
-        <f>IFERROR(ROUND(H13*I13,0),0)</f>
-        <v/>
-      </c>
-      <c r="L13" s="9">
-        <f>IFERROR(VLOOKUP(B13,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M13" s="9">
-        <f>IFERROR(VLOOKUP(B13,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>203687160</v>
+      </c>
+      <c r="K13" s="9" t="n">
+        <v>203687160</v>
+      </c>
+      <c r="L13" s="9" t="n">
+        <v>12500</v>
+      </c>
+      <c r="M13" s="9" t="n">
+        <v>8000</v>
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
@@ -3216,24 +3205,20 @@
       <c r="H14" s="7" t="n">
         <v>20174</v>
       </c>
-      <c r="I14" s="33">
-        <f>IFERROR(VLOOKUP(B14,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I14" s="33" t="n">
+        <v>1454.7</v>
       </c>
       <c r="J14" s="9" t="n">
-        <v>36117425</v>
-      </c>
-      <c r="K14" s="9">
-        <f>IFERROR(ROUND(H14*I14,0),0)</f>
-        <v/>
-      </c>
-      <c r="L14" s="9">
-        <f>IFERROR(VLOOKUP(B14,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M14" s="9">
-        <f>IFERROR(VLOOKUP(B14,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>29347118</v>
+      </c>
+      <c r="K14" s="9" t="n">
+        <v>29347118</v>
+      </c>
+      <c r="L14" s="9" t="n">
+        <v>10171</v>
+      </c>
+      <c r="M14" s="9" t="n">
+        <v>6509</v>
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
@@ -3347,24 +3332,20 @@
       <c r="H15" s="7" t="n">
         <v>4620</v>
       </c>
-      <c r="I15" s="33">
-        <f>IFERROR(VLOOKUP(B15,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I15" s="33" t="n">
+        <v>1454.7</v>
       </c>
       <c r="J15" s="9" t="n">
-        <v>36117425</v>
-      </c>
-      <c r="K15" s="9">
-        <f>IFERROR(ROUND(H15*I15,0),0)</f>
-        <v/>
-      </c>
-      <c r="L15" s="9">
-        <f>IFERROR(VLOOKUP(B15,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M15" s="9">
-        <f>IFERROR(VLOOKUP(B15,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>6720714</v>
+      </c>
+      <c r="K15" s="9" t="n">
+        <v>6720714</v>
+      </c>
+      <c r="L15" s="9" t="n">
+        <v>2329</v>
+      </c>
+      <c r="M15" s="9" t="n">
+        <v>1491</v>
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
@@ -3478,24 +3459,20 @@
       <c r="H16" s="7" t="n">
         <v>9626.35</v>
       </c>
-      <c r="I16" s="33">
-        <f>IFERROR(VLOOKUP(B16,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I16" s="33" t="n">
+        <v>1476</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>14256012</v>
-      </c>
-      <c r="K16" s="9">
-        <f>IFERROR(ROUND(H16*I16,0),0)</f>
-        <v/>
-      </c>
-      <c r="L16" s="9">
-        <f>IFERROR(VLOOKUP(B16,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M16" s="9">
-        <f>IFERROR(VLOOKUP(B16,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>14208493</v>
+      </c>
+      <c r="K16" s="9" t="n">
+        <v>14208493</v>
+      </c>
+      <c r="L16" s="9" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M16" s="9" t="n">
+        <v>8000</v>
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
@@ -3609,24 +3586,20 @@
       <c r="H17" s="7" t="n">
         <v>4936</v>
       </c>
-      <c r="I17" s="33">
-        <f>IFERROR(VLOOKUP(B17,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I17" s="33" t="n">
+        <v>1480</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>22306800</v>
-      </c>
-      <c r="K17" s="9">
-        <f>IFERROR(ROUND(H17*I17,0),0)</f>
-        <v/>
-      </c>
-      <c r="L17" s="9">
-        <f>IFERROR(VLOOKUP(B17,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M17" s="9">
-        <f>IFERROR(VLOOKUP(B17,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>7305280</v>
+      </c>
+      <c r="K17" s="9" t="n">
+        <v>7305280</v>
+      </c>
+      <c r="L17" s="9" t="n">
+        <v>3282</v>
+      </c>
+      <c r="M17" s="9" t="n">
+        <v>2626</v>
       </c>
       <c r="N17" s="3" t="inlineStr">
         <is>
@@ -3740,24 +3713,20 @@
       <c r="H18" s="7" t="n">
         <v>2745</v>
       </c>
-      <c r="I18" s="33">
-        <f>IFERROR(VLOOKUP(B18,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I18" s="33" t="n">
+        <v>1451.7</v>
       </c>
       <c r="J18" s="9" t="n">
-        <v>25506948</v>
-      </c>
-      <c r="K18" s="9">
-        <f>IFERROR(ROUND(H18*I18,0),0)</f>
-        <v/>
-      </c>
-      <c r="L18" s="9">
-        <f>IFERROR(VLOOKUP(B18,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M18" s="9">
-        <f>IFERROR(VLOOKUP(B18,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>3984917</v>
+      </c>
+      <c r="K18" s="9" t="n">
+        <v>3984917</v>
+      </c>
+      <c r="L18" s="9" t="n">
+        <v>1565</v>
+      </c>
+      <c r="M18" s="9" t="n">
+        <v>1252</v>
       </c>
       <c r="N18" s="3" t="inlineStr">
         <is>
@@ -3871,24 +3840,20 @@
       <c r="H19" s="7" t="n">
         <v>1700</v>
       </c>
-      <c r="I19" s="33">
-        <f>IFERROR(VLOOKUP(B19,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I19" s="33" t="n">
+        <v>1506.4</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>9919642</v>
-      </c>
-      <c r="K19" s="9">
-        <f>IFERROR(ROUND(H19*I19,0),0)</f>
-        <v/>
-      </c>
-      <c r="L19" s="9">
-        <f>IFERROR(VLOOKUP(B19,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M19" s="9">
-        <f>IFERROR(VLOOKUP(B19,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>2560880</v>
+      </c>
+      <c r="K19" s="9" t="n">
+        <v>2560880</v>
+      </c>
+      <c r="L19" s="9" t="n">
+        <v>2594</v>
+      </c>
+      <c r="M19" s="9" t="n">
+        <v>2075</v>
       </c>
       <c r="N19" s="3" t="inlineStr">
         <is>
@@ -4131,10 +4096,10 @@
         <v>1482.8</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>424990980</v>
+        <v>424940824</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>424990980</v>
+        <v>424940824</v>
       </c>
       <c r="L21" s="9" t="n">
         <v>12038</v>
@@ -4252,24 +4217,20 @@
       <c r="H22" s="7" t="n">
         <v>9740</v>
       </c>
-      <c r="I22" s="33">
-        <f>IFERROR(VLOOKUP(B22,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I22" s="33" t="n">
+        <v>1505.7</v>
       </c>
       <c r="J22" s="9" t="n">
-        <v>51777431</v>
-      </c>
-      <c r="K22" s="9">
-        <f>IFERROR(ROUND(H22*I22,0),0)</f>
-        <v/>
-      </c>
-      <c r="L22" s="9">
-        <f>IFERROR(VLOOKUP(B22,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M22" s="9">
-        <f>IFERROR(VLOOKUP(B22,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>14665518</v>
+      </c>
+      <c r="K22" s="9" t="n">
+        <v>14665518</v>
+      </c>
+      <c r="L22" s="9" t="n">
+        <v>3544</v>
+      </c>
+      <c r="M22" s="9" t="n">
+        <v>2268</v>
       </c>
       <c r="N22" s="3" t="inlineStr">
         <is>
@@ -4498,24 +4459,20 @@
       <c r="H24" s="7" t="n">
         <v>36190</v>
       </c>
-      <c r="I24" s="33">
-        <f>IFERROR(VLOOKUP(B24,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I24" s="33" t="n">
+        <v>1481.9</v>
       </c>
       <c r="J24" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" s="9">
-        <f>IFERROR(ROUND(H24*I24,0),0)</f>
-        <v/>
-      </c>
-      <c r="L24" s="9">
-        <f>IFERROR(VLOOKUP(B24,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M24" s="9">
-        <f>IFERROR(VLOOKUP(B24,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>53629961</v>
+      </c>
+      <c r="K24" s="9" t="n">
+        <v>53629961</v>
+      </c>
+      <c r="L24" s="9" t="n">
+        <v>7847</v>
+      </c>
+      <c r="M24" s="9" t="n">
+        <v>5022</v>
       </c>
       <c r="N24" s="3" t="inlineStr">
         <is>
@@ -4629,24 +4586,20 @@
       <c r="H25" s="7" t="n">
         <v>180</v>
       </c>
-      <c r="I25" s="33">
-        <f>IFERROR(VLOOKUP(B25,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I25" s="33" t="n">
+        <v>1481.9</v>
       </c>
       <c r="J25" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" s="9">
-        <f>IFERROR(ROUND(H25*I25,0),0)</f>
-        <v/>
-      </c>
-      <c r="L25" s="9">
-        <f>IFERROR(VLOOKUP(B25,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M25" s="9">
-        <f>IFERROR(VLOOKUP(B25,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>266742</v>
+      </c>
+      <c r="K25" s="9" t="n">
+        <v>266742</v>
+      </c>
+      <c r="L25" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="M25" s="9" t="n">
+        <v>25</v>
       </c>
       <c r="N25" s="3" t="inlineStr">
         <is>
@@ -4760,24 +4713,20 @@
       <c r="H26" s="7" t="n">
         <v>21280</v>
       </c>
-      <c r="I26" s="33">
-        <f>IFERROR(VLOOKUP(B26,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I26" s="33" t="n">
+        <v>1481.9</v>
       </c>
       <c r="J26" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" s="9">
-        <f>IFERROR(ROUND(H26*I26,0),0)</f>
-        <v/>
-      </c>
-      <c r="L26" s="9">
-        <f>IFERROR(VLOOKUP(B26,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M26" s="9">
-        <f>IFERROR(VLOOKUP(B26,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>31534832</v>
+      </c>
+      <c r="K26" s="9" t="n">
+        <v>31534832</v>
+      </c>
+      <c r="L26" s="9" t="n">
+        <v>4614</v>
+      </c>
+      <c r="M26" s="9" t="n">
+        <v>2953</v>
       </c>
       <c r="N26" s="3" t="inlineStr">
         <is>
@@ -4891,24 +4840,20 @@
       <c r="H27" s="7" t="n">
         <v>2058</v>
       </c>
-      <c r="I27" s="33">
-        <f>IFERROR(VLOOKUP(B27,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I27" s="33" t="n">
+        <v>1474.9</v>
       </c>
       <c r="J27" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" s="9">
-        <f>IFERROR(ROUND(H27*I27,0),0)</f>
-        <v/>
-      </c>
-      <c r="L27" s="9">
-        <f>IFERROR(VLOOKUP(B27,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M27" s="9">
-        <f>IFERROR(VLOOKUP(B27,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>3035344</v>
+      </c>
+      <c r="K27" s="9" t="n">
+        <v>3035344</v>
+      </c>
+      <c r="L27" s="9" t="n">
+        <v>1200</v>
+      </c>
+      <c r="M27" s="9" t="n">
+        <v>768</v>
       </c>
       <c r="N27" s="3" t="inlineStr">
         <is>
@@ -5022,24 +4967,20 @@
       <c r="H28" s="7" t="n">
         <v>1977</v>
       </c>
-      <c r="I28" s="33">
-        <f>IFERROR(VLOOKUP(B28,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I28" s="33" t="n">
+        <v>1474.9</v>
       </c>
       <c r="J28" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" s="9">
-        <f>IFERROR(ROUND(H28*I28,0),0)</f>
-        <v/>
-      </c>
-      <c r="L28" s="9">
-        <f>IFERROR(VLOOKUP(B28,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M28" s="9">
-        <f>IFERROR(VLOOKUP(B28,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>2915877</v>
+      </c>
+      <c r="K28" s="9" t="n">
+        <v>2915877</v>
+      </c>
+      <c r="L28" s="9" t="n">
+        <v>1153</v>
+      </c>
+      <c r="M28" s="9" t="n">
+        <v>738</v>
       </c>
       <c r="N28" s="3" t="inlineStr">
         <is>
@@ -5153,22 +5094,20 @@
       <c r="H29" s="7" t="n">
         <v>4290</v>
       </c>
-      <c r="I29" s="33">
-        <f>IFERROR(VLOOKUP(B29,RemitTable2,7,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="J29" s="9" t="n"/>
-      <c r="K29" s="9">
-        <f>IFERROR(ROUND(H29*I29,0),0)</f>
-        <v/>
-      </c>
-      <c r="L29" s="9">
-        <f>IFERROR(VLOOKUP(B29,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M29" s="9">
-        <f>IFERROR(VLOOKUP(B29,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+      <c r="I29" s="33" t="n">
+        <v>1510.6</v>
+      </c>
+      <c r="J29" s="9" t="n">
+        <v>6480474</v>
+      </c>
+      <c r="K29" s="9" t="n">
+        <v>6480474</v>
+      </c>
+      <c r="L29" s="9" t="n">
+        <v>7500</v>
+      </c>
+      <c r="M29" s="9" t="n">
+        <v>8000</v>
       </c>
       <c r="N29" s="3" t="inlineStr">
         <is>
@@ -5270,24 +5209,20 @@
       <c r="H30" s="80" t="n">
         <v>78209</v>
       </c>
-      <c r="I30" s="180">
-        <f>IFERROR(VLOOKUP(B30,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I30" s="180" t="n">
+        <v>1502.7</v>
       </c>
       <c r="J30" s="82" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" s="82">
-        <f>IFERROR(ROUND(H30*I30,0),0)</f>
-        <v/>
-      </c>
-      <c r="L30" s="82">
-        <f>IFERROR(VLOOKUP(B30,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M30" s="82">
-        <f>IFERROR(VLOOKUP(B30,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>117524664</v>
+      </c>
+      <c r="K30" s="82" t="n">
+        <v>117524664</v>
+      </c>
+      <c r="L30" s="82" t="n">
+        <v>9619</v>
+      </c>
+      <c r="M30" s="82" t="n">
+        <v>6156</v>
       </c>
       <c r="N30" s="78" t="inlineStr">
         <is>
@@ -5389,24 +5324,20 @@
       <c r="H31" s="80" t="n">
         <v>8140</v>
       </c>
-      <c r="I31" s="180">
-        <f>IFERROR(VLOOKUP(B31,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I31" s="180" t="n">
+        <v>1502.7</v>
       </c>
       <c r="J31" s="82" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" s="82">
-        <f>IFERROR(ROUND(H31*I31,0),0)</f>
-        <v/>
-      </c>
-      <c r="L31" s="82">
-        <f>IFERROR(VLOOKUP(B31,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M31" s="82">
-        <f>IFERROR(VLOOKUP(B31,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>12231978</v>
+      </c>
+      <c r="K31" s="82" t="n">
+        <v>12231978</v>
+      </c>
+      <c r="L31" s="82" t="n">
+        <v>1001</v>
+      </c>
+      <c r="M31" s="82" t="n">
+        <v>641</v>
       </c>
       <c r="N31" s="78" t="inlineStr">
         <is>
@@ -5512,10 +5443,10 @@
         <v>1741.08</v>
       </c>
       <c r="J32" s="82" t="n">
-        <v>7702082</v>
+        <v>7640555</v>
       </c>
       <c r="K32" s="82" t="n">
-        <v>7702082</v>
+        <v>7640555</v>
       </c>
       <c r="L32" s="82" t="n">
         <v>10000</v>
@@ -5845,24 +5776,20 @@
       <c r="H35" s="126" t="n">
         <v>98800</v>
       </c>
-      <c r="I35" s="126">
-        <f>IFERROR(VLOOKUP(B35,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I35" s="126" t="n">
+        <v>1502.8</v>
       </c>
       <c r="J35" s="128" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" s="128">
-        <f>IFERROR(ROUND(H35*I35,0),0)</f>
-        <v/>
-      </c>
-      <c r="L35" s="128">
-        <f>IFERROR(VLOOKUP(B35,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M35" s="128">
-        <f>IFERROR(VLOOKUP(B35,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>148476640</v>
+      </c>
+      <c r="K35" s="128" t="n">
+        <v>148476640</v>
+      </c>
+      <c r="L35" s="128" t="n">
+        <v>12457</v>
+      </c>
+      <c r="M35" s="128" t="n">
+        <v>7973</v>
       </c>
       <c r="N35" s="129" t="n"/>
       <c r="O35" s="182" t="n">
@@ -5960,24 +5887,20 @@
       <c r="H36" s="126" t="n">
         <v>90</v>
       </c>
-      <c r="I36" s="126">
-        <f>IFERROR(VLOOKUP(B36,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I36" s="126" t="n">
+        <v>1502.8</v>
       </c>
       <c r="J36" s="128" t="n">
-        <v>0</v>
-      </c>
-      <c r="K36" s="128">
-        <f>IFERROR(ROUND(H36*I36,0),0)</f>
-        <v/>
-      </c>
-      <c r="L36" s="128">
-        <f>IFERROR(VLOOKUP(B36,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M36" s="128">
-        <f>IFERROR(VLOOKUP(B36,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>135252</v>
+      </c>
+      <c r="K36" s="128" t="n">
+        <v>135252</v>
+      </c>
+      <c r="L36" s="128" t="n">
+        <v>11</v>
+      </c>
+      <c r="M36" s="128" t="n">
+        <v>7</v>
       </c>
       <c r="N36" s="129" t="n"/>
       <c r="O36" s="129" t="n"/>
@@ -6061,24 +5984,20 @@
       <c r="H37" s="211" t="n">
         <v>69160</v>
       </c>
-      <c r="I37" s="212">
-        <f>IFERROR(VLOOKUP(B37,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I37" s="212" t="n">
+        <v>1525.3</v>
       </c>
       <c r="J37" s="213" t="n">
-        <v>0</v>
-      </c>
-      <c r="K37" s="213">
-        <f>IFERROR(ROUND(H37*I37,0),0)</f>
-        <v/>
-      </c>
-      <c r="L37" s="213">
-        <f>IFERROR(VLOOKUP(B37,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M37" s="213">
-        <f>IFERROR(VLOOKUP(B37,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>105489748</v>
+      </c>
+      <c r="K37" s="213" t="n">
+        <v>105489748</v>
+      </c>
+      <c r="L37" s="213" t="n">
+        <v>7261</v>
+      </c>
+      <c r="M37" s="213" t="n">
+        <v>4647</v>
       </c>
       <c r="N37" s="207" t="inlineStr">
         <is>
@@ -6180,24 +6099,20 @@
       <c r="H38" s="211" t="n">
         <v>49400</v>
       </c>
-      <c r="I38" s="212">
-        <f>IFERROR(VLOOKUP(B38,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I38" s="212" t="n">
+        <v>1525.3</v>
       </c>
       <c r="J38" s="213" t="n">
-        <v>0</v>
-      </c>
-      <c r="K38" s="213">
-        <f>IFERROR(ROUND(H38*I38,0),0)</f>
-        <v/>
-      </c>
-      <c r="L38" s="213">
-        <f>IFERROR(VLOOKUP(B38,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M38" s="213">
-        <f>IFERROR(VLOOKUP(B38,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>75349820</v>
+      </c>
+      <c r="K38" s="213" t="n">
+        <v>75349820</v>
+      </c>
+      <c r="L38" s="213" t="n">
+        <v>5186</v>
+      </c>
+      <c r="M38" s="213" t="n">
+        <v>3319</v>
       </c>
       <c r="N38" s="207" t="inlineStr">
         <is>
@@ -6420,24 +6335,20 @@
       <c r="H40" s="24" t="n">
         <v>5673</v>
       </c>
-      <c r="I40" s="185">
-        <f>IFERROR(VLOOKUP(B40,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I40" s="185" t="n">
+        <v>1441.6</v>
       </c>
       <c r="J40" s="26" t="n">
-        <v>205028994</v>
-      </c>
-      <c r="K40" s="26">
-        <f>IFERROR(ROUND(H40*I40,0),0)</f>
-        <v/>
-      </c>
-      <c r="L40" s="26">
-        <f>IFERROR(VLOOKUP(B40,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M40" s="26">
-        <f>IFERROR(VLOOKUP(B40,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>8178197</v>
+      </c>
+      <c r="K40" s="26" t="n">
+        <v>8178197</v>
+      </c>
+      <c r="L40" s="26" t="n">
+        <v>499</v>
+      </c>
+      <c r="M40" s="26" t="n">
+        <v>319</v>
       </c>
       <c r="N40" s="20" t="inlineStr">
         <is>
@@ -6551,24 +6462,20 @@
       <c r="H41" s="24" t="n">
         <v>350</v>
       </c>
-      <c r="I41" s="185">
-        <f>IFERROR(VLOOKUP(B41,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I41" s="185" t="n">
+        <v>1439.1</v>
       </c>
       <c r="J41" s="26" t="n">
-        <v>18264679</v>
-      </c>
-      <c r="K41" s="26">
-        <f>IFERROR(ROUND(H41*I41,0),0)</f>
-        <v/>
-      </c>
-      <c r="L41" s="26">
-        <f>IFERROR(VLOOKUP(B41,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M41" s="26">
-        <f>IFERROR(VLOOKUP(B41,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>503685</v>
+      </c>
+      <c r="K41" s="26" t="n">
+        <v>503685</v>
+      </c>
+      <c r="L41" s="26" t="n">
+        <v>253</v>
+      </c>
+      <c r="M41" s="26" t="n">
+        <v>202</v>
       </c>
       <c r="N41" s="20" t="inlineStr">
         <is>
@@ -6682,24 +6589,20 @@
       <c r="H42" s="24" t="n">
         <v>26358</v>
       </c>
-      <c r="I42" s="185">
-        <f>IFERROR(VLOOKUP(B42,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I42" s="185" t="n">
+        <v>1460.7</v>
       </c>
       <c r="J42" s="26" t="n">
-        <v>38550844</v>
-      </c>
-      <c r="K42" s="26">
-        <f>IFERROR(ROUND(H42*I42,0),0)</f>
-        <v/>
-      </c>
-      <c r="L42" s="26">
-        <f>IFERROR(VLOOKUP(B42,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M42" s="26">
-        <f>IFERROR(VLOOKUP(B42,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>38501131</v>
+      </c>
+      <c r="K42" s="26" t="n">
+        <v>38501131</v>
+      </c>
+      <c r="L42" s="26" t="n">
+        <v>12500</v>
+      </c>
+      <c r="M42" s="26" t="n">
+        <v>8000</v>
       </c>
       <c r="N42" s="20" t="inlineStr">
         <is>
@@ -6813,24 +6716,20 @@
       <c r="H43" s="24" t="n">
         <v>450</v>
       </c>
-      <c r="I43" s="185">
-        <f>IFERROR(VLOOKUP(B43,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I43" s="185" t="n">
+        <v>1475.7</v>
       </c>
       <c r="J43" s="26" t="n">
-        <v>5505104</v>
-      </c>
-      <c r="K43" s="26">
-        <f>IFERROR(ROUND(H43*I43,0),0)</f>
-        <v/>
-      </c>
-      <c r="L43" s="26">
-        <f>IFERROR(VLOOKUP(B43,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M43" s="26">
-        <f>IFERROR(VLOOKUP(B43,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>664065</v>
+      </c>
+      <c r="K43" s="26" t="n">
+        <v>664065</v>
+      </c>
+      <c r="L43" s="26" t="n">
+        <v>912</v>
+      </c>
+      <c r="M43" s="26" t="n">
+        <v>973</v>
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
@@ -6944,24 +6843,20 @@
       <c r="H44" s="24" t="n">
         <v>540</v>
       </c>
-      <c r="I44" s="185">
-        <f>IFERROR(VLOOKUP(B44,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I44" s="185" t="n">
+        <v>1475.7</v>
       </c>
       <c r="J44" s="26" t="n">
-        <v>5505104</v>
-      </c>
-      <c r="K44" s="26">
-        <f>IFERROR(ROUND(H44*I44,0),0)</f>
-        <v/>
-      </c>
-      <c r="L44" s="26">
-        <f>IFERROR(VLOOKUP(B44,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M44" s="26">
-        <f>IFERROR(VLOOKUP(B44,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>796878</v>
+      </c>
+      <c r="K44" s="26" t="n">
+        <v>796878</v>
+      </c>
+      <c r="L44" s="26" t="n">
+        <v>1095</v>
+      </c>
+      <c r="M44" s="26" t="n">
+        <v>1168</v>
       </c>
       <c r="N44" s="20" t="inlineStr">
         <is>
@@ -7075,24 +6970,20 @@
       <c r="H45" s="24" t="n">
         <v>136516</v>
       </c>
-      <c r="I45" s="185">
-        <f>IFERROR(VLOOKUP(B45,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I45" s="185" t="n">
+        <v>1441.6</v>
       </c>
       <c r="J45" s="26" t="n">
-        <v>205028994</v>
-      </c>
-      <c r="K45" s="26">
-        <f>IFERROR(ROUND(H45*I45,0),0)</f>
-        <v/>
-      </c>
-      <c r="L45" s="26">
-        <f>IFERROR(VLOOKUP(B45,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M45" s="26">
-        <f>IFERROR(VLOOKUP(B45,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>196801466</v>
+      </c>
+      <c r="K45" s="26" t="n">
+        <v>196801466</v>
+      </c>
+      <c r="L45" s="26" t="n">
+        <v>12001</v>
+      </c>
+      <c r="M45" s="26" t="n">
+        <v>7681</v>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
@@ -7339,24 +7230,20 @@
       <c r="H47" s="24" t="n">
         <v>14793</v>
       </c>
-      <c r="I47" s="185">
-        <f>IFERROR(VLOOKUP(B47,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I47" s="185" t="n">
+        <v>1451.7</v>
       </c>
       <c r="J47" s="26" t="n">
-        <v>25506948</v>
-      </c>
-      <c r="K47" s="26">
-        <f>IFERROR(ROUND(H47*I47,0),0)</f>
-        <v/>
-      </c>
-      <c r="L47" s="26">
-        <f>IFERROR(VLOOKUP(B47,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M47" s="26">
-        <f>IFERROR(VLOOKUP(B47,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>21474998</v>
+      </c>
+      <c r="K47" s="26" t="n">
+        <v>21474998</v>
+      </c>
+      <c r="L47" s="26" t="n">
+        <v>8435</v>
+      </c>
+      <c r="M47" s="26" t="n">
+        <v>6748</v>
       </c>
       <c r="N47" s="20" t="inlineStr">
         <is>
@@ -7603,24 +7490,20 @@
       <c r="H49" s="24" t="n">
         <v>1440</v>
       </c>
-      <c r="I49" s="185">
-        <f>IFERROR(VLOOKUP(B49,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I49" s="185" t="n">
+        <v>1453.6</v>
       </c>
       <c r="J49" s="26" t="n">
-        <v>16908206</v>
-      </c>
-      <c r="K49" s="26">
-        <f>IFERROR(ROUND(H49*I49,0),0)</f>
-        <v/>
-      </c>
-      <c r="L49" s="26">
-        <f>IFERROR(VLOOKUP(B49,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M49" s="26">
-        <f>IFERROR(VLOOKUP(B49,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>2093184</v>
+      </c>
+      <c r="K49" s="26" t="n">
+        <v>2093184</v>
+      </c>
+      <c r="L49" s="26" t="n">
+        <v>1241</v>
+      </c>
+      <c r="M49" s="26" t="n">
+        <v>993</v>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
@@ -7734,24 +7617,20 @@
       <c r="H50" s="24" t="n">
         <v>4489</v>
       </c>
-      <c r="I50" s="185">
-        <f>IFERROR(VLOOKUP(B50,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I50" s="185" t="n">
+        <v>1453.6</v>
       </c>
       <c r="J50" s="26" t="n">
-        <v>16908206</v>
-      </c>
-      <c r="K50" s="26">
-        <f>IFERROR(ROUND(H50*I50,0),0)</f>
-        <v/>
-      </c>
-      <c r="L50" s="26">
-        <f>IFERROR(VLOOKUP(B50,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M50" s="26">
-        <f>IFERROR(VLOOKUP(B50,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>6525210</v>
+      </c>
+      <c r="K50" s="26" t="n">
+        <v>6525210</v>
+      </c>
+      <c r="L50" s="26" t="n">
+        <v>3870</v>
+      </c>
+      <c r="M50" s="26" t="n">
+        <v>3096</v>
       </c>
       <c r="N50" s="20" t="inlineStr">
         <is>
@@ -7865,24 +7744,20 @@
       <c r="H51" s="24" t="n">
         <v>5670.57</v>
       </c>
-      <c r="I51" s="185">
-        <f>IFERROR(VLOOKUP(B51,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I51" s="185" t="n">
+        <v>1453.6</v>
       </c>
       <c r="J51" s="26" t="n">
-        <v>16908206</v>
-      </c>
-      <c r="K51" s="26">
-        <f>IFERROR(ROUND(H51*I51,0),0)</f>
-        <v/>
-      </c>
-      <c r="L51" s="26">
-        <f>IFERROR(VLOOKUP(B51,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M51" s="26">
-        <f>IFERROR(VLOOKUP(B51,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>8242741</v>
+      </c>
+      <c r="K51" s="26" t="n">
+        <v>8242741</v>
+      </c>
+      <c r="L51" s="26" t="n">
+        <v>4889</v>
+      </c>
+      <c r="M51" s="26" t="n">
+        <v>3911</v>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
@@ -7996,24 +7871,20 @@
       <c r="H52" s="24" t="n">
         <v>24614</v>
       </c>
-      <c r="I52" s="185">
-        <f>IFERROR(VLOOKUP(B52,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I52" s="185" t="n">
+        <v>1505.7</v>
       </c>
       <c r="J52" s="26" t="n">
-        <v>51777431</v>
-      </c>
-      <c r="K52" s="26">
-        <f>IFERROR(ROUND(H52*I52,0),0)</f>
-        <v/>
-      </c>
-      <c r="L52" s="26">
-        <f>IFERROR(VLOOKUP(B52,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M52" s="26">
-        <f>IFERROR(VLOOKUP(B52,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>37061300</v>
+      </c>
+      <c r="K52" s="26" t="n">
+        <v>37061300</v>
+      </c>
+      <c r="L52" s="26" t="n">
+        <v>8956</v>
+      </c>
+      <c r="M52" s="26" t="n">
+        <v>5732</v>
       </c>
       <c r="N52" s="20" t="inlineStr">
         <is>
@@ -8127,24 +7998,20 @@
       <c r="H53" s="24" t="n">
         <v>3993.05</v>
       </c>
-      <c r="I53" s="185">
-        <f>IFERROR(VLOOKUP(B53,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I53" s="185" t="n">
+        <v>1506.4</v>
       </c>
       <c r="J53" s="26" t="n">
-        <v>9919642</v>
-      </c>
-      <c r="K53" s="26">
-        <f>IFERROR(ROUND(H53*I53,0),0)</f>
-        <v/>
-      </c>
-      <c r="L53" s="26">
-        <f>IFERROR(VLOOKUP(B53,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M53" s="26">
-        <f>IFERROR(VLOOKUP(B53,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>6015131</v>
+      </c>
+      <c r="K53" s="26" t="n">
+        <v>6015131</v>
+      </c>
+      <c r="L53" s="26" t="n">
+        <v>6093</v>
+      </c>
+      <c r="M53" s="26" t="n">
+        <v>4875</v>
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
@@ -8258,24 +8125,20 @@
       <c r="H54" s="24" t="n">
         <v>360</v>
       </c>
-      <c r="I54" s="185">
-        <f>IFERROR(VLOOKUP(B54,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I54" s="185" t="n">
+        <v>1506.4</v>
       </c>
       <c r="J54" s="26" t="n">
-        <v>9919642</v>
-      </c>
-      <c r="K54" s="26">
-        <f>IFERROR(ROUND(H54*I54,0),0)</f>
-        <v/>
-      </c>
-      <c r="L54" s="26">
-        <f>IFERROR(VLOOKUP(B54,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M54" s="26">
-        <f>IFERROR(VLOOKUP(B54,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>542304</v>
+      </c>
+      <c r="K54" s="26" t="n">
+        <v>542304</v>
+      </c>
+      <c r="L54" s="26" t="n">
+        <v>549</v>
+      </c>
+      <c r="M54" s="26" t="n">
+        <v>439</v>
       </c>
       <c r="N54" s="20" t="inlineStr">
         <is>
@@ -8389,24 +8252,20 @@
       <c r="H55" s="24" t="n">
         <v>500</v>
       </c>
-      <c r="I55" s="185">
-        <f>IFERROR(VLOOKUP(B55,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I55" s="185" t="n">
+        <v>1506.4</v>
       </c>
       <c r="J55" s="26" t="n">
-        <v>9919642</v>
-      </c>
-      <c r="K55" s="26">
-        <f>IFERROR(ROUND(H55*I55,0),0)</f>
-        <v/>
-      </c>
-      <c r="L55" s="26">
-        <f>IFERROR(VLOOKUP(B55,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M55" s="26">
-        <f>IFERROR(VLOOKUP(B55,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>753200</v>
+      </c>
+      <c r="K55" s="26" t="n">
+        <v>753200</v>
+      </c>
+      <c r="L55" s="26" t="n">
+        <v>763</v>
+      </c>
+      <c r="M55" s="26" t="n">
+        <v>610</v>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
@@ -8520,24 +8379,20 @@
       <c r="H56" s="24" t="n">
         <v>17404</v>
       </c>
-      <c r="I56" s="185">
-        <f>IFERROR(VLOOKUP(B56,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I56" s="185" t="n">
+        <v>1474.9</v>
       </c>
       <c r="J56" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="K56" s="26">
-        <f>IFERROR(ROUND(H56*I56,0),0)</f>
-        <v/>
-      </c>
-      <c r="L56" s="26">
-        <f>IFERROR(VLOOKUP(B56,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M56" s="26">
-        <f>IFERROR(VLOOKUP(B56,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>25669160</v>
+      </c>
+      <c r="K56" s="26" t="n">
+        <v>25669160</v>
+      </c>
+      <c r="L56" s="26" t="n">
+        <v>10147</v>
+      </c>
+      <c r="M56" s="26" t="n">
+        <v>6494</v>
       </c>
       <c r="N56" s="20" t="inlineStr">
         <is>
@@ -8651,24 +8506,20 @@
       <c r="H57" s="87" t="n">
         <v>15289</v>
       </c>
-      <c r="I57" s="187">
-        <f>IFERROR(VLOOKUP(B57,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I57" s="187" t="n">
+        <v>1502.7</v>
       </c>
       <c r="J57" s="89" t="n">
-        <v>0</v>
-      </c>
-      <c r="K57" s="89">
-        <f>IFERROR(ROUND(H57*I57,0),0)</f>
-        <v/>
-      </c>
-      <c r="L57" s="89">
-        <f>IFERROR(VLOOKUP(B57,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M57" s="89">
-        <f>IFERROR(VLOOKUP(B57,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>22974780</v>
+      </c>
+      <c r="K57" s="89" t="n">
+        <v>22974780</v>
+      </c>
+      <c r="L57" s="89" t="n">
+        <v>1880</v>
+      </c>
+      <c r="M57" s="89" t="n">
+        <v>1203</v>
       </c>
       <c r="N57" s="85" t="inlineStr">
         <is>
@@ -8903,24 +8754,20 @@
       <c r="H59" s="134" t="n">
         <v>180</v>
       </c>
-      <c r="I59" s="134">
-        <f>IFERROR(VLOOKUP(B59,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I59" s="134" t="n">
+        <v>1518.9</v>
       </c>
       <c r="J59" s="136" t="n">
-        <v>0</v>
-      </c>
-      <c r="K59" s="136">
-        <f>IFERROR(ROUND(H59*I59,0),0)</f>
-        <v/>
-      </c>
-      <c r="L59" s="136">
-        <f>IFERROR(VLOOKUP(B59,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M59" s="136">
-        <f>IFERROR(VLOOKUP(B59,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>273402</v>
+      </c>
+      <c r="K59" s="136" t="n">
+        <v>273402</v>
+      </c>
+      <c r="L59" s="136" t="n">
+        <v>2500</v>
+      </c>
+      <c r="M59" s="136" t="n">
+        <v>8000</v>
       </c>
       <c r="N59" s="137" t="n"/>
       <c r="O59" s="137" t="n"/>
@@ -9012,24 +8859,20 @@
       <c r="H60" s="134" t="n">
         <v>250</v>
       </c>
-      <c r="I60" s="134">
-        <f>IFERROR(VLOOKUP(B60,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I60" s="134" t="n">
+        <v>1502.8</v>
       </c>
       <c r="J60" s="136" t="n">
-        <v>0</v>
-      </c>
-      <c r="K60" s="136">
-        <f>IFERROR(ROUND(H60*I60,0),0)</f>
-        <v/>
-      </c>
-      <c r="L60" s="136">
-        <f>IFERROR(VLOOKUP(B60,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M60" s="136">
-        <f>IFERROR(VLOOKUP(B60,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>375700</v>
+      </c>
+      <c r="K60" s="136" t="n">
+        <v>375700</v>
+      </c>
+      <c r="L60" s="136" t="n">
+        <v>32</v>
+      </c>
+      <c r="M60" s="136" t="n">
+        <v>20</v>
       </c>
       <c r="N60" s="137" t="n"/>
       <c r="O60" s="137" t="n"/>
@@ -9121,24 +8964,20 @@
       <c r="H61" s="134" t="n">
         <v>500</v>
       </c>
-      <c r="I61" s="134">
-        <f>IFERROR(VLOOKUP(B61,RemitTable2,7,FALSE),0)</f>
-        <v/>
+      <c r="I61" s="134" t="n">
+        <v>1525.3</v>
       </c>
       <c r="J61" s="136" t="n">
-        <v>0</v>
-      </c>
-      <c r="K61" s="136">
-        <f>IFERROR(ROUND(H61*I61,0),0)</f>
-        <v/>
-      </c>
-      <c r="L61" s="136">
-        <f>IFERROR(VLOOKUP(B61,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M61" s="136">
-        <f>IFERROR(VLOOKUP(B61,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>762650</v>
+      </c>
+      <c r="K61" s="136" t="n">
+        <v>762650</v>
+      </c>
+      <c r="L61" s="136" t="n">
+        <v>52</v>
+      </c>
+      <c r="M61" s="136" t="n">
+        <v>34</v>
       </c>
       <c r="N61" s="137" t="n"/>
       <c r="O61" s="137" t="n"/>
@@ -9491,19 +9330,16 @@
         <v/>
       </c>
       <c r="J64" s="222" t="n">
-        <v>0</v>
-      </c>
-      <c r="K64" s="222">
-        <f>IFERROR(ROUND(H64*I64,0),0)</f>
-        <v/>
-      </c>
-      <c r="L64" s="222">
-        <f>IFERROR(VLOOKUP(B64,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M64" s="222">
-        <f>IFERROR(VLOOKUP(B64,RemitTable2,11,FALSE),0)</f>
-        <v/>
+        <v>75818749</v>
+      </c>
+      <c r="K64" s="222" t="n">
+        <v>75818749</v>
+      </c>
+      <c r="L64" s="222" t="n">
+        <v>25000</v>
+      </c>
+      <c r="M64" s="222" t="n">
+        <v>16000</v>
       </c>
       <c r="N64" s="216" t="inlineStr">
         <is>
@@ -14744,33 +14580,26 @@
       <c r="E43" s="118" t="n">
         <v>143557</v>
       </c>
-      <c r="F43" s="122">
-        <f>D43/E43</f>
-        <v/>
-      </c>
-      <c r="G43" s="118">
-        <f>F10</f>
-        <v/>
-      </c>
-      <c r="H43" s="120">
-        <f>ROUND(D43*G43,0)</f>
-        <v/>
-      </c>
-      <c r="I43" s="120">
-        <f>ROUND(G10*F43*G43,0)</f>
-        <v/>
-      </c>
-      <c r="J43" s="120">
-        <f>ROUND(H10*F43,0)</f>
-        <v/>
-      </c>
-      <c r="K43" s="120">
-        <f>ROUND(I10*F43,0)</f>
-        <v/>
-      </c>
-      <c r="L43" s="121">
-        <f>H43+I43+J43+K43</f>
-        <v/>
+      <c r="F43" s="122" t="n">
+        <v>0.968835</v>
+      </c>
+      <c r="G43" s="118" t="n">
+        <v>1479.7</v>
+      </c>
+      <c r="H43" s="120" t="n">
+        <v>205801115</v>
+      </c>
+      <c r="I43" s="120" t="n">
+        <v>28672</v>
+      </c>
+      <c r="J43" s="120" t="n">
+        <v>12110</v>
+      </c>
+      <c r="K43" s="120" t="n">
+        <v>7751</v>
+      </c>
+      <c r="L43" s="121" t="n">
+        <v>205849648</v>
       </c>
       <c r="M43" s="115" t="n"/>
     </row>
@@ -14796,33 +14625,26 @@
       <c r="E44" s="118" t="n">
         <v>143557</v>
       </c>
-      <c r="F44" s="122">
-        <f>D44/E44</f>
-        <v/>
-      </c>
-      <c r="G44" s="118">
-        <f>F10</f>
-        <v/>
-      </c>
-      <c r="H44" s="120">
-        <f>ROUND(D44*G44,0)</f>
-        <v/>
-      </c>
-      <c r="I44" s="120">
-        <f>ROUND(G10*F44*G44,0)</f>
-        <v/>
-      </c>
-      <c r="J44" s="120">
-        <f>ROUND(H10*F44,0)</f>
-        <v/>
-      </c>
-      <c r="K44" s="120">
-        <f>ROUND(I10*F44,0)</f>
-        <v/>
-      </c>
-      <c r="L44" s="121">
-        <f>H44+I44+J44+K44</f>
-        <v/>
+      <c r="F44" s="122" t="n">
+        <v>0.031165</v>
+      </c>
+      <c r="G44" s="118" t="n">
+        <v>1479.7</v>
+      </c>
+      <c r="H44" s="120" t="n">
+        <v>6620178</v>
+      </c>
+      <c r="I44" s="120" t="n">
+        <v>922</v>
+      </c>
+      <c r="J44" s="120" t="n">
+        <v>390</v>
+      </c>
+      <c r="K44" s="120" t="n">
+        <v>249</v>
+      </c>
+      <c r="L44" s="121" t="n">
+        <v>6621739</v>
       </c>
       <c r="M44" s="115" t="n"/>
     </row>
@@ -14848,33 +14670,26 @@
       <c r="E45" s="118" t="n">
         <v>15040</v>
       </c>
-      <c r="F45" s="122">
-        <f>D45/E45</f>
-        <v/>
-      </c>
-      <c r="G45" s="118">
-        <f>F9</f>
-        <v/>
-      </c>
-      <c r="H45" s="120">
-        <f>ROUND(D45*G45,0)</f>
-        <v/>
-      </c>
-      <c r="I45" s="120">
-        <f>ROUND(G9*F45*G45,0)</f>
-        <v/>
-      </c>
-      <c r="J45" s="120">
-        <f>ROUND(H9*F45,0)</f>
-        <v/>
-      </c>
-      <c r="K45" s="120">
-        <f>ROUND(I9*F45,0)</f>
-        <v/>
-      </c>
-      <c r="L45" s="121">
-        <f>H45+I45+J45+K45</f>
-        <v/>
+      <c r="F45" s="122" t="n">
+        <v>0.328191</v>
+      </c>
+      <c r="G45" s="118" t="n">
+        <v>1480</v>
+      </c>
+      <c r="H45" s="120" t="n">
+        <v>7305280</v>
+      </c>
+      <c r="I45" s="120" t="n">
+        <v>9714</v>
+      </c>
+      <c r="J45" s="120" t="n">
+        <v>3282</v>
+      </c>
+      <c r="K45" s="120" t="n">
+        <v>2626</v>
+      </c>
+      <c r="L45" s="121" t="n">
+        <v>7320902</v>
       </c>
       <c r="M45" s="115" t="n"/>
     </row>
@@ -14900,33 +14715,26 @@
       <c r="E46" s="118" t="n">
         <v>13860</v>
       </c>
-      <c r="F46" s="122">
-        <f>D46/E46</f>
-        <v/>
-      </c>
-      <c r="G46" s="118">
-        <f>F12</f>
-        <v/>
-      </c>
-      <c r="H46" s="120">
-        <f>ROUND(D46*G46,0)</f>
-        <v/>
-      </c>
-      <c r="I46" s="120">
-        <f>ROUND(G12*F46*G46,0)</f>
-        <v/>
-      </c>
-      <c r="J46" s="120">
-        <f>ROUND(H12*F46,0)</f>
-        <v/>
-      </c>
-      <c r="K46" s="120">
-        <f>ROUND(I12*F46,0)</f>
-        <v/>
-      </c>
-      <c r="L46" s="121">
-        <f>H46+I46+J46+K46</f>
-        <v/>
+      <c r="F46" s="122" t="n">
+        <v>0.65368</v>
+      </c>
+      <c r="G46" s="118" t="n">
+        <v>1439.1</v>
+      </c>
+      <c r="H46" s="120" t="n">
+        <v>13038246</v>
+      </c>
+      <c r="I46" s="120" t="n">
+        <v>18814</v>
+      </c>
+      <c r="J46" s="120" t="n">
+        <v>6537</v>
+      </c>
+      <c r="K46" s="120" t="n">
+        <v>5229</v>
+      </c>
+      <c r="L46" s="121" t="n">
+        <v>13068826</v>
       </c>
       <c r="M46" s="115" t="n"/>
     </row>
@@ -14952,33 +14760,26 @@
       <c r="E47" s="118" t="n">
         <v>13860</v>
       </c>
-      <c r="F47" s="122">
-        <f>D47/E47</f>
-        <v/>
-      </c>
-      <c r="G47" s="118">
-        <f>F12</f>
-        <v/>
-      </c>
-      <c r="H47" s="120">
-        <f>ROUND(D47*G47,0)</f>
-        <v/>
-      </c>
-      <c r="I47" s="120">
-        <f>ROUND(G12*F47*G47,0)</f>
-        <v/>
-      </c>
-      <c r="J47" s="120">
-        <f>ROUND(H12*F47,0)</f>
-        <v/>
-      </c>
-      <c r="K47" s="120">
-        <f>ROUND(I12*F47,0)</f>
-        <v/>
-      </c>
-      <c r="L47" s="121">
-        <f>H47+I47+J47+K47</f>
-        <v/>
+      <c r="F47" s="122" t="n">
+        <v>0.025253</v>
+      </c>
+      <c r="G47" s="118" t="n">
+        <v>1439.1</v>
+      </c>
+      <c r="H47" s="120" t="n">
+        <v>503685</v>
+      </c>
+      <c r="I47" s="120" t="n">
+        <v>727</v>
+      </c>
+      <c r="J47" s="120" t="n">
+        <v>253</v>
+      </c>
+      <c r="K47" s="120" t="n">
+        <v>202</v>
+      </c>
+      <c r="L47" s="121" t="n">
+        <v>504867</v>
       </c>
       <c r="M47" s="115" t="n"/>
     </row>
@@ -15004,33 +14805,26 @@
       <c r="E48" s="118" t="n">
         <v>252</v>
       </c>
-      <c r="F48" s="122">
-        <f>D48/E48</f>
-        <v/>
-      </c>
-      <c r="G48" s="118">
-        <f>F14</f>
-        <v/>
-      </c>
-      <c r="H48" s="120">
-        <f>ROUND(D48*G48,0)</f>
-        <v/>
-      </c>
-      <c r="I48" s="120">
-        <f>ROUND(G14*F48*G48,0)</f>
-        <v/>
-      </c>
-      <c r="J48" s="120">
-        <f>ROUND(H14*F48,0)</f>
-        <v/>
-      </c>
-      <c r="K48" s="120">
-        <f>ROUND(I14*F48,0)</f>
-        <v/>
-      </c>
-      <c r="L48" s="121">
-        <f>H48+I48+J48+K48</f>
-        <v/>
+      <c r="F48" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="118" t="n">
+        <v>1479</v>
+      </c>
+      <c r="H48" s="120" t="n">
+        <v>372708</v>
+      </c>
+      <c r="I48" s="120" t="n">
+        <v>29580</v>
+      </c>
+      <c r="J48" s="120" t="n">
+        <v>2500</v>
+      </c>
+      <c r="K48" s="120" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L48" s="121" t="n">
+        <v>412788</v>
       </c>
       <c r="M48" s="115" t="n"/>
     </row>
@@ -15056,33 +14850,26 @@
       <c r="E49" s="118" t="n">
         <v>3700</v>
       </c>
-      <c r="F49" s="122">
-        <f>D49/E49</f>
-        <v/>
-      </c>
-      <c r="G49" s="118">
-        <f>F15</f>
-        <v/>
-      </c>
-      <c r="H49" s="120">
-        <f>ROUND(D49*G49,0)</f>
-        <v/>
-      </c>
-      <c r="I49" s="120">
-        <f>ROUND(G15*F49*G49,0)</f>
-        <v/>
-      </c>
-      <c r="J49" s="120">
-        <f>ROUND(H15*F49,0)</f>
-        <v/>
-      </c>
-      <c r="K49" s="120">
-        <f>ROUND(I15*F49,0)</f>
-        <v/>
-      </c>
-      <c r="L49" s="121">
-        <f>H49+I49+J49+K49</f>
-        <v/>
+      <c r="F49" s="122" t="n">
+        <v>0.121622</v>
+      </c>
+      <c r="G49" s="118" t="n">
+        <v>1475.7</v>
+      </c>
+      <c r="H49" s="120" t="n">
+        <v>664065</v>
+      </c>
+      <c r="I49" s="120" t="n">
+        <v>3590</v>
+      </c>
+      <c r="J49" s="120" t="n">
+        <v>912</v>
+      </c>
+      <c r="K49" s="120" t="n">
+        <v>973</v>
+      </c>
+      <c r="L49" s="121" t="n">
+        <v>669540</v>
       </c>
       <c r="M49" s="115" t="n"/>
     </row>
@@ -15108,33 +14895,26 @@
       <c r="E50" s="118" t="n">
         <v>3700</v>
       </c>
-      <c r="F50" s="122">
-        <f>D50/E50</f>
-        <v/>
-      </c>
-      <c r="G50" s="118">
-        <f>F15</f>
-        <v/>
-      </c>
-      <c r="H50" s="120">
-        <f>ROUND(D50*G50,0)</f>
-        <v/>
-      </c>
-      <c r="I50" s="120">
-        <f>ROUND(G15*F50*G50,0)</f>
-        <v/>
-      </c>
-      <c r="J50" s="120">
-        <f>ROUND(H15*F50,0)</f>
-        <v/>
-      </c>
-      <c r="K50" s="120">
-        <f>ROUND(I15*F50,0)</f>
-        <v/>
-      </c>
-      <c r="L50" s="121">
-        <f>H50+I50+J50+K50</f>
-        <v/>
+      <c r="F50" s="122" t="n">
+        <v>0.732432</v>
+      </c>
+      <c r="G50" s="118" t="n">
+        <v>1475.7</v>
+      </c>
+      <c r="H50" s="120" t="n">
+        <v>3999147</v>
+      </c>
+      <c r="I50" s="120" t="n">
+        <v>21617</v>
+      </c>
+      <c r="J50" s="120" t="n">
+        <v>5493</v>
+      </c>
+      <c r="K50" s="120" t="n">
+        <v>5859</v>
+      </c>
+      <c r="L50" s="121" t="n">
+        <v>4032116</v>
       </c>
       <c r="M50" s="115" t="n"/>
     </row>
@@ -15160,33 +14940,26 @@
       <c r="E51" s="118" t="n">
         <v>3700</v>
       </c>
-      <c r="F51" s="122">
-        <f>D51/E51</f>
-        <v/>
-      </c>
-      <c r="G51" s="118">
-        <f>F15</f>
-        <v/>
-      </c>
-      <c r="H51" s="120">
-        <f>ROUND(D51*G51,0)</f>
-        <v/>
-      </c>
-      <c r="I51" s="120">
-        <f>ROUND(G15*F51*G51,0)</f>
-        <v/>
-      </c>
-      <c r="J51" s="120">
-        <f>ROUND(H15*F51,0)</f>
-        <v/>
-      </c>
-      <c r="K51" s="120">
-        <f>ROUND(I15*F51,0)</f>
-        <v/>
-      </c>
-      <c r="L51" s="121">
-        <f>H51+I51+J51+K51</f>
-        <v/>
+      <c r="F51" s="122" t="n">
+        <v>0.145946</v>
+      </c>
+      <c r="G51" s="118" t="n">
+        <v>1475.7</v>
+      </c>
+      <c r="H51" s="120" t="n">
+        <v>796878</v>
+      </c>
+      <c r="I51" s="120" t="n">
+        <v>4307</v>
+      </c>
+      <c r="J51" s="120" t="n">
+        <v>1095</v>
+      </c>
+      <c r="K51" s="120" t="n">
+        <v>1168</v>
+      </c>
+      <c r="L51" s="121" t="n">
+        <v>803448</v>
       </c>
       <c r="M51" s="115" t="n"/>
     </row>
@@ -15212,33 +14985,26 @@
       <c r="E52" s="118" t="n">
         <v>9626.35</v>
       </c>
-      <c r="F52" s="122">
-        <f>D52/E52</f>
-        <v/>
-      </c>
-      <c r="G52" s="118">
-        <f>F16</f>
-        <v/>
-      </c>
-      <c r="H52" s="120">
-        <f>ROUND(D52*G52,0)</f>
-        <v/>
-      </c>
-      <c r="I52" s="120">
-        <f>ROUND(G16*F52*G52,0)</f>
-        <v/>
-      </c>
-      <c r="J52" s="120">
-        <f>ROUND(H16*F52,0)</f>
-        <v/>
-      </c>
-      <c r="K52" s="120">
-        <f>ROUND(I16*F52,0)</f>
-        <v/>
-      </c>
-      <c r="L52" s="121">
-        <f>H52+I52+J52+K52</f>
-        <v/>
+      <c r="F52" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="118" t="n">
+        <v>1476</v>
+      </c>
+      <c r="H52" s="120" t="n">
+        <v>14208493</v>
+      </c>
+      <c r="I52" s="120" t="n">
+        <v>29520</v>
+      </c>
+      <c r="J52" s="120" t="n">
+        <v>10000</v>
+      </c>
+      <c r="K52" s="120" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L52" s="121" t="n">
+        <v>14256013</v>
       </c>
       <c r="M52" s="115" t="n"/>
     </row>
@@ -15264,33 +15030,26 @@
       <c r="E53" s="118" t="n">
         <v>5056.8</v>
       </c>
-      <c r="F53" s="122">
-        <f>D53/E53</f>
-        <v/>
-      </c>
-      <c r="G53" s="118">
-        <f>F17</f>
-        <v/>
-      </c>
-      <c r="H53" s="120">
-        <f>ROUND(D53*G53,0)</f>
-        <v/>
-      </c>
-      <c r="I53" s="120">
-        <f>ROUND(G17*F53*G53,0)</f>
-        <v/>
-      </c>
-      <c r="J53" s="120">
-        <f>ROUND(H17*F53,0)</f>
-        <v/>
-      </c>
-      <c r="K53" s="120">
-        <f>ROUND(I17*F53,0)</f>
-        <v/>
-      </c>
-      <c r="L53" s="121">
-        <f>H53+I53+J53+K53</f>
-        <v/>
+      <c r="F53" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="118" t="n">
+        <v>1445.5</v>
+      </c>
+      <c r="H53" s="120" t="n">
+        <v>7309604</v>
+      </c>
+      <c r="I53" s="120" t="n">
+        <v>28910</v>
+      </c>
+      <c r="J53" s="120" t="n">
+        <v>10000</v>
+      </c>
+      <c r="K53" s="120" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L53" s="121" t="n">
+        <v>7356514</v>
       </c>
       <c r="M53" s="115" t="n"/>
     </row>
@@ -15316,33 +15075,26 @@
       <c r="E54" s="118" t="n">
         <v>24794</v>
       </c>
-      <c r="F54" s="122">
-        <f>D54/E54</f>
-        <v/>
-      </c>
-      <c r="G54" s="118">
-        <f>F19</f>
-        <v/>
-      </c>
-      <c r="H54" s="120">
-        <f>ROUND(D54*G54,0)</f>
-        <v/>
-      </c>
-      <c r="I54" s="120">
-        <f>ROUND(G19*F54*G54,0)</f>
-        <v/>
-      </c>
-      <c r="J54" s="120">
-        <f>ROUND(H19*F54,0)</f>
-        <v/>
-      </c>
-      <c r="K54" s="120">
-        <f>ROUND(I19*F54,0)</f>
-        <v/>
-      </c>
-      <c r="L54" s="121">
-        <f>H54+I54+J54+K54</f>
-        <v/>
+      <c r="F54" s="122" t="n">
+        <v>0.813665</v>
+      </c>
+      <c r="G54" s="118" t="n">
+        <v>1454.7</v>
+      </c>
+      <c r="H54" s="120" t="n">
+        <v>29347118</v>
+      </c>
+      <c r="I54" s="120" t="n">
+        <v>23673</v>
+      </c>
+      <c r="J54" s="120" t="n">
+        <v>10171</v>
+      </c>
+      <c r="K54" s="120" t="n">
+        <v>6509</v>
+      </c>
+      <c r="L54" s="121" t="n">
+        <v>29387471</v>
       </c>
       <c r="M54" s="115" t="n"/>
     </row>
@@ -15368,33 +15120,26 @@
       <c r="E55" s="118" t="n">
         <v>24794</v>
       </c>
-      <c r="F55" s="122">
-        <f>D55/E55</f>
-        <v/>
-      </c>
-      <c r="G55" s="118">
-        <f>F19</f>
-        <v/>
-      </c>
-      <c r="H55" s="120">
-        <f>ROUND(D55*G55,0)</f>
-        <v/>
-      </c>
-      <c r="I55" s="120">
-        <f>ROUND(G19*F55*G55,0)</f>
-        <v/>
-      </c>
-      <c r="J55" s="120">
-        <f>ROUND(H19*F55,0)</f>
-        <v/>
-      </c>
-      <c r="K55" s="120">
-        <f>ROUND(I19*F55,0)</f>
-        <v/>
-      </c>
-      <c r="L55" s="121">
-        <f>H55+I55+J55+K55</f>
-        <v/>
+      <c r="F55" s="122" t="n">
+        <v>0.186335</v>
+      </c>
+      <c r="G55" s="118" t="n">
+        <v>1454.7</v>
+      </c>
+      <c r="H55" s="120" t="n">
+        <v>6720714</v>
+      </c>
+      <c r="I55" s="120" t="n">
+        <v>5421</v>
+      </c>
+      <c r="J55" s="120" t="n">
+        <v>2329</v>
+      </c>
+      <c r="K55" s="120" t="n">
+        <v>1491</v>
+      </c>
+      <c r="L55" s="121" t="n">
+        <v>6729955</v>
       </c>
       <c r="M55" s="115" t="n"/>
     </row>
@@ -15420,33 +15165,26 @@
       <c r="E56" s="118" t="n">
         <v>11599.57</v>
       </c>
-      <c r="F56" s="122">
-        <f>D56/E56</f>
-        <v/>
-      </c>
-      <c r="G56" s="118">
-        <f>F20</f>
-        <v/>
-      </c>
-      <c r="H56" s="120">
-        <f>ROUND(D56*G56,0)</f>
-        <v/>
-      </c>
-      <c r="I56" s="120">
-        <f>ROUND(G20*F56*G56,0)</f>
-        <v/>
-      </c>
-      <c r="J56" s="120">
-        <f>ROUND(H20*F56,0)</f>
-        <v/>
-      </c>
-      <c r="K56" s="120">
-        <f>ROUND(I20*F56,0)</f>
-        <v/>
-      </c>
-      <c r="L56" s="121">
-        <f>H56+I56+J56+K56</f>
-        <v/>
+      <c r="F56" s="122" t="n">
+        <v>0.124143</v>
+      </c>
+      <c r="G56" s="118" t="n">
+        <v>1453.6</v>
+      </c>
+      <c r="H56" s="120" t="n">
+        <v>2093184</v>
+      </c>
+      <c r="I56" s="120" t="n">
+        <v>3609</v>
+      </c>
+      <c r="J56" s="120" t="n">
+        <v>1241</v>
+      </c>
+      <c r="K56" s="120" t="n">
+        <v>993</v>
+      </c>
+      <c r="L56" s="121" t="n">
+        <v>2099027</v>
       </c>
       <c r="M56" s="115" t="n"/>
     </row>
@@ -15472,33 +15210,26 @@
       <c r="E57" s="118" t="n">
         <v>11599.57</v>
       </c>
-      <c r="F57" s="122">
-        <f>D57/E57</f>
-        <v/>
-      </c>
-      <c r="G57" s="118">
-        <f>F20</f>
-        <v/>
-      </c>
-      <c r="H57" s="120">
-        <f>ROUND(D57*G57,0)</f>
-        <v/>
-      </c>
-      <c r="I57" s="120">
-        <f>ROUND(G20*F57*G57,0)</f>
-        <v/>
-      </c>
-      <c r="J57" s="120">
-        <f>ROUND(H20*F57,0)</f>
-        <v/>
-      </c>
-      <c r="K57" s="120">
-        <f>ROUND(I20*F57,0)</f>
-        <v/>
-      </c>
-      <c r="L57" s="121">
-        <f>H57+I57+J57+K57</f>
-        <v/>
+      <c r="F57" s="122" t="n">
+        <v>0.386997</v>
+      </c>
+      <c r="G57" s="118" t="n">
+        <v>1453.6</v>
+      </c>
+      <c r="H57" s="120" t="n">
+        <v>6525210</v>
+      </c>
+      <c r="I57" s="120" t="n">
+        <v>11251</v>
+      </c>
+      <c r="J57" s="120" t="n">
+        <v>3870</v>
+      </c>
+      <c r="K57" s="120" t="n">
+        <v>3096</v>
+      </c>
+      <c r="L57" s="121" t="n">
+        <v>6543427</v>
       </c>
       <c r="M57" s="115" t="n"/>
     </row>
@@ -15524,33 +15255,26 @@
       <c r="E58" s="118" t="n">
         <v>11599.57</v>
       </c>
-      <c r="F58" s="122">
-        <f>D58/E58</f>
-        <v/>
-      </c>
-      <c r="G58" s="118">
-        <f>F20</f>
-        <v/>
-      </c>
-      <c r="H58" s="120">
-        <f>ROUND(D58*G58,0)</f>
-        <v/>
-      </c>
-      <c r="I58" s="120">
-        <f>ROUND(G20*F58*G58,0)</f>
-        <v/>
-      </c>
-      <c r="J58" s="120">
-        <f>ROUND(H20*F58,0)</f>
-        <v/>
-      </c>
-      <c r="K58" s="120">
-        <f>ROUND(I20*F58,0)</f>
-        <v/>
-      </c>
-      <c r="L58" s="121">
-        <f>H58+I58+J58+K58</f>
-        <v/>
+      <c r="F58" s="122" t="n">
+        <v>0.48886</v>
+      </c>
+      <c r="G58" s="118" t="n">
+        <v>1453.6</v>
+      </c>
+      <c r="H58" s="120" t="n">
+        <v>8242741</v>
+      </c>
+      <c r="I58" s="120" t="n">
+        <v>14212</v>
+      </c>
+      <c r="J58" s="120" t="n">
+        <v>4889</v>
+      </c>
+      <c r="K58" s="120" t="n">
+        <v>3911</v>
+      </c>
+      <c r="L58" s="121" t="n">
+        <v>8265753</v>
       </c>
       <c r="M58" s="115" t="n"/>
     </row>
@@ -15576,33 +15300,26 @@
       <c r="E59" s="118" t="n">
         <v>26358</v>
       </c>
-      <c r="F59" s="122">
-        <f>D59/E59</f>
-        <v/>
-      </c>
-      <c r="G59" s="118">
-        <f>F21</f>
-        <v/>
-      </c>
-      <c r="H59" s="120">
-        <f>ROUND(D59*G59,0)</f>
-        <v/>
-      </c>
-      <c r="I59" s="120">
-        <f>ROUND(G21*F59*G59,0)</f>
-        <v/>
-      </c>
-      <c r="J59" s="120">
-        <f>ROUND(H21*F59,0)</f>
-        <v/>
-      </c>
-      <c r="K59" s="120">
-        <f>ROUND(I21*F59,0)</f>
-        <v/>
-      </c>
-      <c r="L59" s="121">
-        <f>H59+I59+J59+K59</f>
-        <v/>
+      <c r="F59" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="118" t="n">
+        <v>1460.7</v>
+      </c>
+      <c r="H59" s="120" t="n">
+        <v>38501131</v>
+      </c>
+      <c r="I59" s="120" t="n">
+        <v>29214</v>
+      </c>
+      <c r="J59" s="120" t="n">
+        <v>12500</v>
+      </c>
+      <c r="K59" s="120" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L59" s="121" t="n">
+        <v>38550845</v>
       </c>
       <c r="M59" s="115" t="n"/>
     </row>
@@ -15628,33 +15345,26 @@
       <c r="E60" s="118" t="n">
         <v>17538</v>
       </c>
-      <c r="F60" s="122">
-        <f>D60/E60</f>
-        <v/>
-      </c>
-      <c r="G60" s="118">
-        <f>F22</f>
-        <v/>
-      </c>
-      <c r="H60" s="120">
-        <f>ROUND(D60*G60,0)</f>
-        <v/>
-      </c>
-      <c r="I60" s="120">
-        <f>ROUND(G22*F60*G60,0)</f>
-        <v/>
-      </c>
-      <c r="J60" s="120">
-        <f>ROUND(H22*F60,0)</f>
-        <v/>
-      </c>
-      <c r="K60" s="120">
-        <f>ROUND(I22*F60,0)</f>
-        <v/>
-      </c>
-      <c r="L60" s="121">
-        <f>H60+I60+J60+K60</f>
-        <v/>
+      <c r="F60" s="122" t="n">
+        <v>0.843483</v>
+      </c>
+      <c r="G60" s="118" t="n">
+        <v>1451.7</v>
+      </c>
+      <c r="H60" s="120" t="n">
+        <v>21474998</v>
+      </c>
+      <c r="I60" s="120" t="n">
+        <v>24490</v>
+      </c>
+      <c r="J60" s="120" t="n">
+        <v>8435</v>
+      </c>
+      <c r="K60" s="120" t="n">
+        <v>6748</v>
+      </c>
+      <c r="L60" s="121" t="n">
+        <v>21514671</v>
       </c>
       <c r="M60" s="115" t="n"/>
     </row>
@@ -15680,33 +15390,26 @@
       <c r="E61" s="118" t="n">
         <v>17538</v>
       </c>
-      <c r="F61" s="122">
-        <f>D61/E61</f>
-        <v/>
-      </c>
-      <c r="G61" s="118">
-        <f>F22</f>
-        <v/>
-      </c>
-      <c r="H61" s="120">
-        <f>ROUND(D61*G61,0)</f>
-        <v/>
-      </c>
-      <c r="I61" s="120">
-        <f>ROUND(G22*F61*G61,0)</f>
-        <v/>
-      </c>
-      <c r="J61" s="120">
-        <f>ROUND(H22*F61,0)</f>
-        <v/>
-      </c>
-      <c r="K61" s="120">
-        <f>ROUND(I22*F61,0)</f>
-        <v/>
-      </c>
-      <c r="L61" s="121">
-        <f>H61+I61+J61+K61</f>
-        <v/>
+      <c r="F61" s="122" t="n">
+        <v>0.156517</v>
+      </c>
+      <c r="G61" s="118" t="n">
+        <v>1451.7</v>
+      </c>
+      <c r="H61" s="120" t="n">
+        <v>3984917</v>
+      </c>
+      <c r="I61" s="120" t="n">
+        <v>4544</v>
+      </c>
+      <c r="J61" s="120" t="n">
+        <v>1565</v>
+      </c>
+      <c r="K61" s="120" t="n">
+        <v>1252</v>
+      </c>
+      <c r="L61" s="121" t="n">
+        <v>3992278</v>
       </c>
       <c r="M61" s="115" t="n"/>
     </row>
@@ -15732,33 +15435,26 @@
       <c r="E62" s="118" t="n">
         <v>142189</v>
       </c>
-      <c r="F62" s="122">
-        <f>D62/E62</f>
-        <v/>
-      </c>
-      <c r="G62" s="118">
-        <f>F23</f>
-        <v/>
-      </c>
-      <c r="H62" s="120">
-        <f>ROUND(D62*G62,0)</f>
-        <v/>
-      </c>
-      <c r="I62" s="120">
-        <f>ROUND(G23*F62*G62,0)</f>
-        <v/>
-      </c>
-      <c r="J62" s="120">
-        <f>ROUND(H23*F62,0)</f>
-        <v/>
-      </c>
-      <c r="K62" s="120">
-        <f>ROUND(I23*F62,0)</f>
-        <v/>
-      </c>
-      <c r="L62" s="121">
-        <f>H62+I62+J62+K62</f>
-        <v/>
+      <c r="F62" s="122" t="n">
+        <v>0.039898</v>
+      </c>
+      <c r="G62" s="118" t="n">
+        <v>1441.6</v>
+      </c>
+      <c r="H62" s="120" t="n">
+        <v>8178197</v>
+      </c>
+      <c r="I62" s="120" t="n">
+        <v>1150</v>
+      </c>
+      <c r="J62" s="120" t="n">
+        <v>499</v>
+      </c>
+      <c r="K62" s="120" t="n">
+        <v>319</v>
+      </c>
+      <c r="L62" s="121" t="n">
+        <v>8180165</v>
       </c>
       <c r="M62" s="115" t="n"/>
     </row>
@@ -15784,33 +15480,26 @@
       <c r="E63" s="118" t="n">
         <v>142189</v>
       </c>
-      <c r="F63" s="122">
-        <f>D63/E63</f>
-        <v/>
-      </c>
-      <c r="G63" s="118">
-        <f>F23</f>
-        <v/>
-      </c>
-      <c r="H63" s="120">
-        <f>ROUND(D63*G63,0)</f>
-        <v/>
-      </c>
-      <c r="I63" s="120">
-        <f>ROUND(G23*F63*G63,0)</f>
-        <v/>
-      </c>
-      <c r="J63" s="120">
-        <f>ROUND(H23*F63,0)</f>
-        <v/>
-      </c>
-      <c r="K63" s="120">
-        <f>ROUND(I23*F63,0)</f>
-        <v/>
-      </c>
-      <c r="L63" s="121">
-        <f>H63+I63+J63+K63</f>
-        <v/>
+      <c r="F63" s="122" t="n">
+        <v>0.960102</v>
+      </c>
+      <c r="G63" s="118" t="n">
+        <v>1441.6</v>
+      </c>
+      <c r="H63" s="120" t="n">
+        <v>196801466</v>
+      </c>
+      <c r="I63" s="120" t="n">
+        <v>27682</v>
+      </c>
+      <c r="J63" s="120" t="n">
+        <v>12001</v>
+      </c>
+      <c r="K63" s="120" t="n">
+        <v>7681</v>
+      </c>
+      <c r="L63" s="121" t="n">
+        <v>196848830</v>
       </c>
       <c r="M63" s="115" t="n"/>
     </row>
@@ -15836,33 +15525,26 @@
       <c r="E64" s="118" t="n">
         <v>137850</v>
       </c>
-      <c r="F64" s="122">
-        <f>D64/E64</f>
-        <v/>
-      </c>
-      <c r="G64" s="118">
-        <f>F24</f>
-        <v/>
-      </c>
-      <c r="H64" s="120">
-        <f>ROUND(D64*G64,0)</f>
-        <v/>
-      </c>
-      <c r="I64" s="120">
-        <f>ROUND(G24*F64*G64,0)</f>
-        <v/>
-      </c>
-      <c r="J64" s="120">
-        <f>ROUND(H24*F64,0)</f>
-        <v/>
-      </c>
-      <c r="K64" s="120">
-        <f>ROUND(I24*F64,0)</f>
-        <v/>
-      </c>
-      <c r="L64" s="121">
-        <f>H64+I64+J64+K64</f>
-        <v/>
+      <c r="F64" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="118" t="n">
+        <v>1477.6</v>
+      </c>
+      <c r="H64" s="120" t="n">
+        <v>203687160</v>
+      </c>
+      <c r="I64" s="120" t="n">
+        <v>29552</v>
+      </c>
+      <c r="J64" s="120" t="n">
+        <v>12500</v>
+      </c>
+      <c r="K64" s="120" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L64" s="121" t="n">
+        <v>203737212</v>
       </c>
       <c r="M64" s="115" t="n"/>
     </row>
@@ -15888,33 +15570,26 @@
       <c r="E65" s="118" t="n">
         <v>34354</v>
       </c>
-      <c r="F65" s="122">
-        <f>D65/E65</f>
-        <v/>
-      </c>
-      <c r="G65" s="118">
-        <f>F25</f>
-        <v/>
-      </c>
-      <c r="H65" s="120">
-        <f>ROUND(D65*G65,0)</f>
-        <v/>
-      </c>
-      <c r="I65" s="120">
-        <f>ROUND(G25*F65*G65,0)</f>
-        <v/>
-      </c>
-      <c r="J65" s="120">
-        <f>ROUND(H25*F65,0)</f>
-        <v/>
-      </c>
-      <c r="K65" s="120">
-        <f>ROUND(I25*F65,0)</f>
-        <v/>
-      </c>
-      <c r="L65" s="121">
-        <f>H65+I65+J65+K65</f>
-        <v/>
+      <c r="F65" s="122" t="n">
+        <v>0.283519</v>
+      </c>
+      <c r="G65" s="118" t="n">
+        <v>1505.7</v>
+      </c>
+      <c r="H65" s="120" t="n">
+        <v>14665518</v>
+      </c>
+      <c r="I65" s="120" t="n">
+        <v>8538</v>
+      </c>
+      <c r="J65" s="120" t="n">
+        <v>3544</v>
+      </c>
+      <c r="K65" s="120" t="n">
+        <v>2268</v>
+      </c>
+      <c r="L65" s="121" t="n">
+        <v>14679868</v>
       </c>
       <c r="M65" s="115" t="n"/>
     </row>
@@ -15940,33 +15615,26 @@
       <c r="E66" s="118" t="n">
         <v>34354</v>
       </c>
-      <c r="F66" s="122">
-        <f>D66/E66</f>
-        <v/>
-      </c>
-      <c r="G66" s="118">
-        <f>F25</f>
-        <v/>
-      </c>
-      <c r="H66" s="120">
-        <f>ROUND(D66*G66,0)</f>
-        <v/>
-      </c>
-      <c r="I66" s="120">
-        <f>ROUND(G25*F66*G66,0)</f>
-        <v/>
-      </c>
-      <c r="J66" s="120">
-        <f>ROUND(H25*F66,0)</f>
-        <v/>
-      </c>
-      <c r="K66" s="120">
-        <f>ROUND(I25*F66,0)</f>
-        <v/>
-      </c>
-      <c r="L66" s="121">
-        <f>H66+I66+J66+K66</f>
-        <v/>
+      <c r="F66" s="122" t="n">
+        <v>0.716481</v>
+      </c>
+      <c r="G66" s="118" t="n">
+        <v>1505.7</v>
+      </c>
+      <c r="H66" s="120" t="n">
+        <v>37061300</v>
+      </c>
+      <c r="I66" s="120" t="n">
+        <v>21576</v>
+      </c>
+      <c r="J66" s="120" t="n">
+        <v>8956</v>
+      </c>
+      <c r="K66" s="120" t="n">
+        <v>5732</v>
+      </c>
+      <c r="L66" s="121" t="n">
+        <v>37097564</v>
       </c>
       <c r="M66" s="115" t="n"/>
     </row>
@@ -15992,33 +15660,26 @@
       <c r="E67" s="118" t="n">
         <v>6553.05</v>
       </c>
-      <c r="F67" s="122">
-        <f>D67/E67</f>
-        <v/>
-      </c>
-      <c r="G67" s="118">
-        <f>F26</f>
-        <v/>
-      </c>
-      <c r="H67" s="120">
-        <f>ROUND(D67*G67,0)</f>
-        <v/>
-      </c>
-      <c r="I67" s="120">
-        <f>ROUND(G26*F67*G67,0)</f>
-        <v/>
-      </c>
-      <c r="J67" s="120">
-        <f>ROUND(H26*F67,0)</f>
-        <v/>
-      </c>
-      <c r="K67" s="120">
-        <f>ROUND(I26*F67,0)</f>
-        <v/>
-      </c>
-      <c r="L67" s="121">
-        <f>H67+I67+J67+K67</f>
-        <v/>
+      <c r="F67" s="122" t="n">
+        <v>0.259421</v>
+      </c>
+      <c r="G67" s="118" t="n">
+        <v>1506.4</v>
+      </c>
+      <c r="H67" s="120" t="n">
+        <v>2560880</v>
+      </c>
+      <c r="I67" s="120" t="n">
+        <v>7816</v>
+      </c>
+      <c r="J67" s="120" t="n">
+        <v>2594</v>
+      </c>
+      <c r="K67" s="120" t="n">
+        <v>2075</v>
+      </c>
+      <c r="L67" s="121" t="n">
+        <v>2573365</v>
       </c>
       <c r="M67" s="115" t="n"/>
     </row>
@@ -16044,33 +15705,26 @@
       <c r="E68" s="118" t="n">
         <v>6553.05</v>
       </c>
-      <c r="F68" s="122">
-        <f>D68/E68</f>
-        <v/>
-      </c>
-      <c r="G68" s="118">
-        <f>F26</f>
-        <v/>
-      </c>
-      <c r="H68" s="120">
-        <f>ROUND(D68*G68,0)</f>
-        <v/>
-      </c>
-      <c r="I68" s="120">
-        <f>ROUND(G26*F68*G68,0)</f>
-        <v/>
-      </c>
-      <c r="J68" s="120">
-        <f>ROUND(H26*F68,0)</f>
-        <v/>
-      </c>
-      <c r="K68" s="120">
-        <f>ROUND(I26*F68,0)</f>
-        <v/>
-      </c>
-      <c r="L68" s="121">
-        <f>H68+I68+J68+K68</f>
-        <v/>
+      <c r="F68" s="122" t="n">
+        <v>0.6093420000000001</v>
+      </c>
+      <c r="G68" s="118" t="n">
+        <v>1506.4</v>
+      </c>
+      <c r="H68" s="120" t="n">
+        <v>6015131</v>
+      </c>
+      <c r="I68" s="120" t="n">
+        <v>18358</v>
+      </c>
+      <c r="J68" s="120" t="n">
+        <v>6093</v>
+      </c>
+      <c r="K68" s="120" t="n">
+        <v>4875</v>
+      </c>
+      <c r="L68" s="121" t="n">
+        <v>6044457</v>
       </c>
       <c r="M68" s="115" t="n"/>
     </row>
@@ -16096,33 +15750,26 @@
       <c r="E69" s="118" t="n">
         <v>6553.05</v>
       </c>
-      <c r="F69" s="122">
-        <f>D69/E69</f>
-        <v/>
-      </c>
-      <c r="G69" s="118">
-        <f>F26</f>
-        <v/>
-      </c>
-      <c r="H69" s="120">
-        <f>ROUND(D69*G69,0)</f>
-        <v/>
-      </c>
-      <c r="I69" s="120">
-        <f>ROUND(G26*F69*G69,0)</f>
-        <v/>
-      </c>
-      <c r="J69" s="120">
-        <f>ROUND(H26*F69,0)</f>
-        <v/>
-      </c>
-      <c r="K69" s="120">
-        <f>ROUND(I26*F69,0)</f>
-        <v/>
-      </c>
-      <c r="L69" s="121">
-        <f>H69+I69+J69+K69</f>
-        <v/>
+      <c r="F69" s="122" t="n">
+        <v>0.054936</v>
+      </c>
+      <c r="G69" s="118" t="n">
+        <v>1506.4</v>
+      </c>
+      <c r="H69" s="120" t="n">
+        <v>542304</v>
+      </c>
+      <c r="I69" s="120" t="n">
+        <v>1655</v>
+      </c>
+      <c r="J69" s="120" t="n">
+        <v>549</v>
+      </c>
+      <c r="K69" s="120" t="n">
+        <v>439</v>
+      </c>
+      <c r="L69" s="121" t="n">
+        <v>544947</v>
       </c>
       <c r="M69" s="115" t="n"/>
     </row>
@@ -16148,33 +15795,26 @@
       <c r="E70" s="118" t="n">
         <v>6553.05</v>
       </c>
-      <c r="F70" s="122">
-        <f>D70/E70</f>
-        <v/>
-      </c>
-      <c r="G70" s="118">
-        <f>F26</f>
-        <v/>
-      </c>
-      <c r="H70" s="120">
-        <f>ROUND(D70*G70,0)</f>
-        <v/>
-      </c>
-      <c r="I70" s="120">
-        <f>ROUND(G26*F70*G70,0)</f>
-        <v/>
-      </c>
-      <c r="J70" s="120">
-        <f>ROUND(H26*F70,0)</f>
-        <v/>
-      </c>
-      <c r="K70" s="120">
-        <f>ROUND(I26*F70,0)</f>
-        <v/>
-      </c>
-      <c r="L70" s="121">
-        <f>H70+I70+J70+K70</f>
-        <v/>
+      <c r="F70" s="122" t="n">
+        <v>0.07630000000000001</v>
+      </c>
+      <c r="G70" s="118" t="n">
+        <v>1506.4</v>
+      </c>
+      <c r="H70" s="120" t="n">
+        <v>753200</v>
+      </c>
+      <c r="I70" s="120" t="n">
+        <v>2299</v>
+      </c>
+      <c r="J70" s="120" t="n">
+        <v>763</v>
+      </c>
+      <c r="K70" s="120" t="n">
+        <v>610</v>
+      </c>
+      <c r="L70" s="121" t="n">
+        <v>756872</v>
       </c>
       <c r="M70" s="115" t="n"/>
     </row>
@@ -16200,33 +15840,26 @@
       <c r="E71" s="118" t="n">
         <v>57650</v>
       </c>
-      <c r="F71" s="122">
-        <f>D71/E71</f>
-        <v/>
-      </c>
-      <c r="G71" s="118">
-        <f>F27</f>
-        <v/>
-      </c>
-      <c r="H71" s="120">
-        <f>ROUND(D71*G71,0)</f>
-        <v/>
-      </c>
-      <c r="I71" s="120">
-        <f>ROUND(G27*F71*G71,0)</f>
-        <v/>
-      </c>
-      <c r="J71" s="120">
-        <f>ROUND(H27*F71,0)</f>
-        <v/>
-      </c>
-      <c r="K71" s="120">
-        <f>ROUND(I27*F71,0)</f>
-        <v/>
-      </c>
-      <c r="L71" s="121">
-        <f>H71+I71+J71+K71</f>
-        <v/>
+      <c r="F71" s="122" t="n">
+        <v>0.627754</v>
+      </c>
+      <c r="G71" s="118" t="n">
+        <v>1481.9</v>
+      </c>
+      <c r="H71" s="120" t="n">
+        <v>53629961</v>
+      </c>
+      <c r="I71" s="120" t="n">
+        <v>18605</v>
+      </c>
+      <c r="J71" s="120" t="n">
+        <v>7847</v>
+      </c>
+      <c r="K71" s="120" t="n">
+        <v>5022</v>
+      </c>
+      <c r="L71" s="121" t="n">
+        <v>53661435</v>
       </c>
       <c r="M71" s="115" t="n"/>
     </row>
@@ -16252,33 +15885,26 @@
       <c r="E72" s="118" t="n">
         <v>57650</v>
       </c>
-      <c r="F72" s="122">
-        <f>D72/E72</f>
-        <v/>
-      </c>
-      <c r="G72" s="118">
-        <f>F27</f>
-        <v/>
-      </c>
-      <c r="H72" s="120">
-        <f>ROUND(D72*G72,0)</f>
-        <v/>
-      </c>
-      <c r="I72" s="120">
-        <f>ROUND(G27*F72*G72,0)</f>
-        <v/>
-      </c>
-      <c r="J72" s="120">
-        <f>ROUND(H27*F72,0)</f>
-        <v/>
-      </c>
-      <c r="K72" s="120">
-        <f>ROUND(I27*F72,0)</f>
-        <v/>
-      </c>
-      <c r="L72" s="121">
-        <f>H72+I72+J72+K72</f>
-        <v/>
+      <c r="F72" s="122" t="n">
+        <v>0.003122</v>
+      </c>
+      <c r="G72" s="118" t="n">
+        <v>1481.9</v>
+      </c>
+      <c r="H72" s="120" t="n">
+        <v>266742</v>
+      </c>
+      <c r="I72" s="120" t="n">
+        <v>93</v>
+      </c>
+      <c r="J72" s="120" t="n">
+        <v>39</v>
+      </c>
+      <c r="K72" s="120" t="n">
+        <v>25</v>
+      </c>
+      <c r="L72" s="121" t="n">
+        <v>266899</v>
       </c>
       <c r="M72" s="115" t="n"/>
     </row>
@@ -16304,33 +15930,26 @@
       <c r="E73" s="118" t="n">
         <v>57650</v>
       </c>
-      <c r="F73" s="122">
-        <f>D73/E73</f>
-        <v/>
-      </c>
-      <c r="G73" s="118">
-        <f>F27</f>
-        <v/>
-      </c>
-      <c r="H73" s="120">
-        <f>ROUND(D73*G73,0)</f>
-        <v/>
-      </c>
-      <c r="I73" s="120">
-        <f>ROUND(G27*F73*G73,0)</f>
-        <v/>
-      </c>
-      <c r="J73" s="120">
-        <f>ROUND(H27*F73,0)</f>
-        <v/>
-      </c>
-      <c r="K73" s="120">
-        <f>ROUND(I27*F73,0)</f>
-        <v/>
-      </c>
-      <c r="L73" s="121">
-        <f>H73+I73+J73+K73</f>
-        <v/>
+      <c r="F73" s="122" t="n">
+        <v>0.369124</v>
+      </c>
+      <c r="G73" s="118" t="n">
+        <v>1481.9</v>
+      </c>
+      <c r="H73" s="120" t="n">
+        <v>31534832</v>
+      </c>
+      <c r="I73" s="120" t="n">
+        <v>10940</v>
+      </c>
+      <c r="J73" s="120" t="n">
+        <v>4614</v>
+      </c>
+      <c r="K73" s="120" t="n">
+        <v>2953</v>
+      </c>
+      <c r="L73" s="121" t="n">
+        <v>31553339</v>
       </c>
       <c r="M73" s="115" t="n"/>
     </row>
@@ -16356,33 +15975,26 @@
       <c r="E74" s="118" t="n">
         <v>297580</v>
       </c>
-      <c r="F74" s="122">
-        <f>D74/E74</f>
-        <v/>
-      </c>
-      <c r="G74" s="118">
-        <f>F31</f>
-        <v/>
-      </c>
-      <c r="H74" s="120">
-        <f>ROUND(D74*G74,0)</f>
-        <v/>
-      </c>
-      <c r="I74" s="120">
-        <f>ROUND(G31*F74*G74,0)</f>
-        <v/>
-      </c>
-      <c r="J74" s="120">
-        <f>ROUND(H31*F74,0)</f>
-        <v/>
-      </c>
-      <c r="K74" s="120">
-        <f>ROUND(I31*F74,0)</f>
-        <v/>
-      </c>
-      <c r="L74" s="121">
-        <f>H74+I74+J74+K74</f>
-        <v/>
+      <c r="F74" s="122" t="n">
+        <v>0.036965</v>
+      </c>
+      <c r="G74" s="118" t="n">
+        <v>1482.8</v>
+      </c>
+      <c r="H74" s="120" t="n">
+        <v>16310800</v>
+      </c>
+      <c r="I74" s="120" t="n">
+        <v>1096</v>
+      </c>
+      <c r="J74" s="120" t="n">
+        <v>462</v>
+      </c>
+      <c r="K74" s="120" t="n">
+        <v>296</v>
+      </c>
+      <c r="L74" s="121" t="n">
+        <v>16312654</v>
       </c>
       <c r="M74" s="115" t="n"/>
     </row>
@@ -16408,33 +16020,26 @@
       <c r="E75" s="118" t="n">
         <v>297580</v>
       </c>
-      <c r="F75" s="122">
-        <f>D75/E75</f>
-        <v/>
-      </c>
-      <c r="G75" s="118">
-        <f>F31</f>
-        <v/>
-      </c>
-      <c r="H75" s="120">
-        <f>ROUND(D75*G75,0)</f>
-        <v/>
-      </c>
-      <c r="I75" s="120">
-        <f>ROUND(G31*F75*G75,0)</f>
-        <v/>
-      </c>
-      <c r="J75" s="120">
-        <f>ROUND(H31*F75,0)</f>
-        <v/>
-      </c>
-      <c r="K75" s="120">
-        <f>ROUND(I31*F75,0)</f>
-        <v/>
-      </c>
-      <c r="L75" s="121">
-        <f>H75+I75+J75+K75</f>
-        <v/>
+      <c r="F75" s="122" t="n">
+        <v>0.963035</v>
+      </c>
+      <c r="G75" s="118" t="n">
+        <v>1482.8</v>
+      </c>
+      <c r="H75" s="120" t="n">
+        <v>424940824</v>
+      </c>
+      <c r="I75" s="120" t="n">
+        <v>28560</v>
+      </c>
+      <c r="J75" s="120" t="n">
+        <v>12038</v>
+      </c>
+      <c r="K75" s="120" t="n">
+        <v>7704</v>
+      </c>
+      <c r="L75" s="121" t="n">
+        <v>424989126</v>
       </c>
       <c r="M75" s="115" t="n"/>
     </row>
@@ -16460,33 +16065,26 @@
       <c r="E76" s="118" t="n">
         <v>4388.4</v>
       </c>
-      <c r="F76" s="122">
-        <f>D76/E76</f>
-        <v/>
-      </c>
-      <c r="G76" s="118">
-        <f>F32</f>
-        <v/>
-      </c>
-      <c r="H76" s="120">
-        <f>ROUND(D76*G76,0)</f>
-        <v/>
-      </c>
-      <c r="I76" s="120">
-        <f>ROUND(G32*F76*G76,0)</f>
-        <v/>
-      </c>
-      <c r="J76" s="120">
-        <f>ROUND(H32*F76,0)</f>
-        <v/>
-      </c>
-      <c r="K76" s="120">
-        <f>ROUND(I32*F76,0)</f>
-        <v/>
-      </c>
-      <c r="L76" s="121">
-        <f>H76+I76+J76+K76</f>
-        <v/>
+      <c r="F76" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" s="118" t="n">
+        <v>1741.08</v>
+      </c>
+      <c r="H76" s="120" t="n">
+        <v>7640555</v>
+      </c>
+      <c r="I76" s="120" t="n">
+        <v>43527</v>
+      </c>
+      <c r="J76" s="120" t="n">
+        <v>10000</v>
+      </c>
+      <c r="K76" s="120" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L76" s="121" t="n">
+        <v>7702082</v>
       </c>
     </row>
     <row r="77" ht="15.75" customHeight="1">
@@ -16511,33 +16109,26 @@
       <c r="E77" s="118" t="n">
         <v>21439</v>
       </c>
-      <c r="F77" s="122">
-        <f>D77/E77</f>
-        <v/>
-      </c>
-      <c r="G77" s="118">
-        <f>F33</f>
-        <v/>
-      </c>
-      <c r="H77" s="120">
-        <f>ROUND(D77*G77,0)</f>
-        <v/>
-      </c>
-      <c r="I77" s="120">
-        <f>ROUND(G33*F77*G77,0)</f>
-        <v/>
-      </c>
-      <c r="J77" s="120">
-        <f>ROUND(H33*F77,0)</f>
-        <v/>
-      </c>
-      <c r="K77" s="120">
-        <f>ROUND(I33*F77,0)</f>
-        <v/>
-      </c>
-      <c r="L77" s="121">
-        <f>H77+I77+J77+K77</f>
-        <v/>
+      <c r="F77" s="122" t="n">
+        <v>0.811792</v>
+      </c>
+      <c r="G77" s="118" t="n">
+        <v>1474.9</v>
+      </c>
+      <c r="H77" s="120" t="n">
+        <v>25669160</v>
+      </c>
+      <c r="I77" s="120" t="n">
+        <v>23946</v>
+      </c>
+      <c r="J77" s="120" t="n">
+        <v>10147</v>
+      </c>
+      <c r="K77" s="120" t="n">
+        <v>6494</v>
+      </c>
+      <c r="L77" s="121" t="n">
+        <v>25709747</v>
       </c>
     </row>
     <row r="78" ht="15.75" customHeight="1">
@@ -16562,33 +16153,26 @@
       <c r="E78" s="118" t="n">
         <v>21439</v>
       </c>
-      <c r="F78" s="122">
-        <f>D78/E78</f>
-        <v/>
-      </c>
-      <c r="G78" s="118">
-        <f>F33</f>
-        <v/>
-      </c>
-      <c r="H78" s="120">
-        <f>ROUND(D78*G78,0)</f>
-        <v/>
-      </c>
-      <c r="I78" s="120">
-        <f>ROUND(G33*F78*G78,0)</f>
-        <v/>
-      </c>
-      <c r="J78" s="120">
-        <f>ROUND(H33*F78,0)</f>
-        <v/>
-      </c>
-      <c r="K78" s="120">
-        <f>ROUND(I33*F78,0)</f>
-        <v/>
-      </c>
-      <c r="L78" s="121">
-        <f>H78+I78+J78+K78</f>
-        <v/>
+      <c r="F78" s="122" t="n">
+        <v>0.09599299999999999</v>
+      </c>
+      <c r="G78" s="118" t="n">
+        <v>1474.9</v>
+      </c>
+      <c r="H78" s="120" t="n">
+        <v>3035344</v>
+      </c>
+      <c r="I78" s="120" t="n">
+        <v>2832</v>
+      </c>
+      <c r="J78" s="120" t="n">
+        <v>1200</v>
+      </c>
+      <c r="K78" s="120" t="n">
+        <v>768</v>
+      </c>
+      <c r="L78" s="121" t="n">
+        <v>3040144</v>
       </c>
     </row>
     <row r="79" ht="15.75" customHeight="1">
@@ -16613,33 +16197,26 @@
       <c r="E79" s="118" t="n">
         <v>21439</v>
       </c>
-      <c r="F79" s="122">
-        <f>D79/E79</f>
-        <v/>
-      </c>
-      <c r="G79" s="118">
-        <f>F33</f>
-        <v/>
-      </c>
-      <c r="H79" s="120">
-        <f>ROUND(D79*G79,0)</f>
-        <v/>
-      </c>
-      <c r="I79" s="120">
-        <f>ROUND(G33*F79*G79,0)</f>
-        <v/>
-      </c>
-      <c r="J79" s="120">
-        <f>ROUND(H33*F79,0)</f>
-        <v/>
-      </c>
-      <c r="K79" s="120">
-        <f>ROUND(I33*F79,0)</f>
-        <v/>
-      </c>
-      <c r="L79" s="121">
-        <f>H79+I79+J79+K79</f>
-        <v/>
+      <c r="F79" s="122" t="n">
+        <v>0.09221500000000001</v>
+      </c>
+      <c r="G79" s="118" t="n">
+        <v>1474.9</v>
+      </c>
+      <c r="H79" s="120" t="n">
+        <v>2915877</v>
+      </c>
+      <c r="I79" s="120" t="n">
+        <v>2720</v>
+      </c>
+      <c r="J79" s="120" t="n">
+        <v>1153</v>
+      </c>
+      <c r="K79" s="120" t="n">
+        <v>738</v>
+      </c>
+      <c r="L79" s="121" t="n">
+        <v>2920488</v>
       </c>
     </row>
     <row r="80" ht="15.75" customHeight="1">
@@ -16664,33 +16241,26 @@
       <c r="E80" s="118" t="n">
         <v>6800</v>
       </c>
-      <c r="F80" s="122">
-        <f>D80/E80</f>
-        <v/>
-      </c>
-      <c r="G80" s="118">
-        <f>F34</f>
-        <v/>
-      </c>
-      <c r="H80" s="120">
-        <f>ROUND(D80*G80,0)</f>
-        <v/>
-      </c>
-      <c r="I80" s="120">
-        <f>ROUND(G34*F80*G80,0)</f>
-        <v/>
-      </c>
-      <c r="J80" s="120">
-        <f>ROUND(H34*F80,0)</f>
-        <v/>
-      </c>
-      <c r="K80" s="120">
-        <f>ROUND(I34*F80,0)</f>
-        <v/>
-      </c>
-      <c r="L80" s="121">
-        <f>H80+I80+J80+K80</f>
-        <v/>
+      <c r="F80" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" s="118" t="n">
+        <v>1475.2</v>
+      </c>
+      <c r="H80" s="120" t="n">
+        <v>10031360</v>
+      </c>
+      <c r="I80" s="120" t="n">
+        <v>29504</v>
+      </c>
+      <c r="J80" s="120" t="n">
+        <v>10000</v>
+      </c>
+      <c r="K80" s="120" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L80" s="121" t="n">
+        <v>10078864</v>
       </c>
     </row>
     <row r="81" ht="15.75" customHeight="1">
@@ -16715,33 +16285,26 @@
       <c r="E81" s="118" t="n">
         <v>180</v>
       </c>
-      <c r="F81" s="122">
-        <f>D81/E81</f>
-        <v/>
-      </c>
-      <c r="G81" s="118">
-        <f>F36</f>
-        <v/>
-      </c>
-      <c r="H81" s="120">
-        <f>ROUND(D81*G81,0)</f>
-        <v/>
-      </c>
-      <c r="I81" s="120">
-        <f>ROUND(G36*F81*G81,0)</f>
-        <v/>
-      </c>
-      <c r="J81" s="120">
-        <f>ROUND(H36*F81,0)</f>
-        <v/>
-      </c>
-      <c r="K81" s="120">
-        <f>ROUND(I36*F81,0)</f>
-        <v/>
-      </c>
-      <c r="L81" s="121">
-        <f>H81+I81+J81+K81</f>
-        <v/>
+      <c r="F81" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="G81" s="118" t="n">
+        <v>1518.9</v>
+      </c>
+      <c r="H81" s="120" t="n">
+        <v>273402</v>
+      </c>
+      <c r="I81" s="120" t="n">
+        <v>30378</v>
+      </c>
+      <c r="J81" s="120" t="n">
+        <v>2500</v>
+      </c>
+      <c r="K81" s="120" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L81" s="121" t="n">
+        <v>314280</v>
       </c>
     </row>
     <row r="82" ht="15.75" customHeight="1">
@@ -16766,33 +16329,26 @@
       <c r="E82" s="118" t="n">
         <v>4290</v>
       </c>
-      <c r="F82" s="122">
-        <f>D82/E82</f>
-        <v/>
-      </c>
-      <c r="G82" s="118">
-        <f>F37</f>
-        <v/>
-      </c>
-      <c r="H82" s="120">
-        <f>ROUND(D82*G82,0)</f>
-        <v/>
-      </c>
-      <c r="I82" s="120">
-        <f>ROUND(G37*F82*G82,0)</f>
-        <v/>
-      </c>
-      <c r="J82" s="120">
-        <f>ROUND(H37*F82,0)</f>
-        <v/>
-      </c>
-      <c r="K82" s="120">
-        <f>ROUND(I37*F82,0)</f>
-        <v/>
-      </c>
-      <c r="L82" s="121">
-        <f>H82+I82+J82+K82</f>
-        <v/>
+      <c r="F82" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" s="118" t="n">
+        <v>1510.6</v>
+      </c>
+      <c r="H82" s="120" t="n">
+        <v>6480474</v>
+      </c>
+      <c r="I82" s="120" t="n">
+        <v>30212</v>
+      </c>
+      <c r="J82" s="120" t="n">
+        <v>7500</v>
+      </c>
+      <c r="K82" s="120" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L82" s="121" t="n">
+        <v>6526186</v>
       </c>
       <c r="M82" s="40" t="n"/>
     </row>
@@ -16818,33 +16374,26 @@
       <c r="E83" s="118" t="n">
         <v>99140</v>
       </c>
-      <c r="F83" s="122">
-        <f>D83/E83</f>
-        <v/>
-      </c>
-      <c r="G83" s="118">
-        <f>F38</f>
-        <v/>
-      </c>
-      <c r="H83" s="120">
-        <f>ROUND(D83*G83,0)</f>
-        <v/>
-      </c>
-      <c r="I83" s="120">
-        <f>ROUND(G38*F83*G83,0)</f>
-        <v/>
-      </c>
-      <c r="J83" s="120">
-        <f>ROUND(H38*F83,0)</f>
-        <v/>
-      </c>
-      <c r="K83" s="120">
-        <f>ROUND(I38*F83,0)</f>
-        <v/>
-      </c>
-      <c r="L83" s="121">
-        <f>H83+I83+J83+K83</f>
-        <v/>
+      <c r="F83" s="122" t="n">
+        <v>0.996571</v>
+      </c>
+      <c r="G83" s="118" t="n">
+        <v>1502.8</v>
+      </c>
+      <c r="H83" s="120" t="n">
+        <v>148476640</v>
+      </c>
+      <c r="I83" s="120" t="n">
+        <v>29953</v>
+      </c>
+      <c r="J83" s="120" t="n">
+        <v>12457</v>
+      </c>
+      <c r="K83" s="120" t="n">
+        <v>7973</v>
+      </c>
+      <c r="L83" s="121" t="n">
+        <v>148527023</v>
       </c>
     </row>
     <row r="84" ht="15.75" customHeight="1">
@@ -16869,33 +16418,26 @@
       <c r="E84" s="118" t="n">
         <v>99140</v>
       </c>
-      <c r="F84" s="122">
-        <f>D84/E84</f>
-        <v/>
-      </c>
-      <c r="G84" s="118">
-        <f>F38</f>
-        <v/>
-      </c>
-      <c r="H84" s="120">
-        <f>ROUND(D84*G84,0)</f>
-        <v/>
-      </c>
-      <c r="I84" s="120">
-        <f>ROUND(G38*F84*G84,0)</f>
-        <v/>
-      </c>
-      <c r="J84" s="120">
-        <f>ROUND(H38*F84,0)</f>
-        <v/>
-      </c>
-      <c r="K84" s="120">
-        <f>ROUND(I38*F84,0)</f>
-        <v/>
-      </c>
-      <c r="L84" s="121">
-        <f>H84+I84+J84+K84</f>
-        <v/>
+      <c r="F84" s="122" t="n">
+        <v>0.002522</v>
+      </c>
+      <c r="G84" s="118" t="n">
+        <v>1502.8</v>
+      </c>
+      <c r="H84" s="120" t="n">
+        <v>375700</v>
+      </c>
+      <c r="I84" s="120" t="n">
+        <v>76</v>
+      </c>
+      <c r="J84" s="120" t="n">
+        <v>32</v>
+      </c>
+      <c r="K84" s="120" t="n">
+        <v>20</v>
+      </c>
+      <c r="L84" s="121" t="n">
+        <v>375828</v>
       </c>
     </row>
     <row r="85" ht="15.75" customHeight="1">
@@ -16920,33 +16462,26 @@
       <c r="E85" s="118" t="n">
         <v>99140</v>
       </c>
-      <c r="F85" s="122">
-        <f>D85/E85</f>
-        <v/>
-      </c>
-      <c r="G85" s="118">
-        <f>F38</f>
-        <v/>
-      </c>
-      <c r="H85" s="120">
-        <f>ROUND(D85*G85,0)</f>
-        <v/>
-      </c>
-      <c r="I85" s="120">
-        <f>ROUND(G38*F85*G85,0)</f>
-        <v/>
-      </c>
-      <c r="J85" s="120">
-        <f>ROUND(H38*F85,0)</f>
-        <v/>
-      </c>
-      <c r="K85" s="120">
-        <f>ROUND(I38*F85,0)</f>
-        <v/>
-      </c>
-      <c r="L85" s="121">
-        <f>H85+I85+J85+K85</f>
-        <v/>
+      <c r="F85" s="122" t="n">
+        <v>0.000908</v>
+      </c>
+      <c r="G85" s="118" t="n">
+        <v>1502.8</v>
+      </c>
+      <c r="H85" s="120" t="n">
+        <v>135252</v>
+      </c>
+      <c r="I85" s="120" t="n">
+        <v>27</v>
+      </c>
+      <c r="J85" s="120" t="n">
+        <v>11</v>
+      </c>
+      <c r="K85" s="120" t="n">
+        <v>7</v>
+      </c>
+      <c r="L85" s="121" t="n">
+        <v>135297</v>
       </c>
     </row>
     <row r="86" ht="15.75" customHeight="1">
@@ -16971,33 +16506,26 @@
       <c r="E86" s="118" t="n">
         <v>101638</v>
       </c>
-      <c r="F86" s="122">
-        <f>D86/E86</f>
-        <v/>
-      </c>
-      <c r="G86" s="118">
-        <f>F39</f>
-        <v/>
-      </c>
-      <c r="H86" s="120">
-        <f>ROUND(D86*G86,0)</f>
-        <v/>
-      </c>
-      <c r="I86" s="120">
-        <f>ROUND(G39*F86*G86,0)</f>
-        <v/>
-      </c>
-      <c r="J86" s="120">
-        <f>ROUND(H39*F86,0)</f>
-        <v/>
-      </c>
-      <c r="K86" s="120">
-        <f>ROUND(I39*F86,0)</f>
-        <v/>
-      </c>
-      <c r="L86" s="121">
-        <f>H86+I86+J86+K86</f>
-        <v/>
+      <c r="F86" s="122" t="n">
+        <v>0.150426</v>
+      </c>
+      <c r="G86" s="118" t="n">
+        <v>1502.7</v>
+      </c>
+      <c r="H86" s="120" t="n">
+        <v>22974780</v>
+      </c>
+      <c r="I86" s="120" t="n">
+        <v>4521</v>
+      </c>
+      <c r="J86" s="120" t="n">
+        <v>1880</v>
+      </c>
+      <c r="K86" s="120" t="n">
+        <v>1203</v>
+      </c>
+      <c r="L86" s="121" t="n">
+        <v>22982384</v>
       </c>
     </row>
     <row r="87" ht="15.75" customHeight="1">
@@ -17022,33 +16550,26 @@
       <c r="E87" s="118" t="n">
         <v>101638</v>
       </c>
-      <c r="F87" s="122">
-        <f>D87/E87</f>
-        <v/>
-      </c>
-      <c r="G87" s="118">
-        <f>F39</f>
-        <v/>
-      </c>
-      <c r="H87" s="120">
-        <f>ROUND(D87*G87,0)</f>
-        <v/>
-      </c>
-      <c r="I87" s="120">
-        <f>ROUND(G39*F87*G87,0)</f>
-        <v/>
-      </c>
-      <c r="J87" s="120">
-        <f>ROUND(H39*F87,0)</f>
-        <v/>
-      </c>
-      <c r="K87" s="120">
-        <f>ROUND(I39*F87,0)</f>
-        <v/>
-      </c>
-      <c r="L87" s="121">
-        <f>H87+I87+J87+K87</f>
-        <v/>
+      <c r="F87" s="122" t="n">
+        <v>0.769486</v>
+      </c>
+      <c r="G87" s="118" t="n">
+        <v>1502.7</v>
+      </c>
+      <c r="H87" s="120" t="n">
+        <v>117524664</v>
+      </c>
+      <c r="I87" s="120" t="n">
+        <v>23126</v>
+      </c>
+      <c r="J87" s="120" t="n">
+        <v>9619</v>
+      </c>
+      <c r="K87" s="120" t="n">
+        <v>6156</v>
+      </c>
+      <c r="L87" s="121" t="n">
+        <v>117563565</v>
       </c>
     </row>
     <row r="88">
@@ -17073,33 +16594,26 @@
       <c r="E88" s="118" t="n">
         <v>101638</v>
       </c>
-      <c r="F88" s="122">
-        <f>D88/E88</f>
-        <v/>
-      </c>
-      <c r="G88" s="118">
-        <f>F39</f>
-        <v/>
-      </c>
-      <c r="H88" s="120">
-        <f>ROUND(D88*G88,0)</f>
-        <v/>
-      </c>
-      <c r="I88" s="120">
-        <f>ROUND(G39*F88*G88,0)</f>
-        <v/>
-      </c>
-      <c r="J88" s="120">
-        <f>ROUND(H39*F88,0)</f>
-        <v/>
-      </c>
-      <c r="K88" s="120">
-        <f>ROUND(I39*F88,0)</f>
-        <v/>
-      </c>
-      <c r="L88" s="121">
-        <f>H88+I88+J88+K88</f>
-        <v/>
+      <c r="F88" s="122" t="n">
+        <v>0.08008800000000001</v>
+      </c>
+      <c r="G88" s="118" t="n">
+        <v>1502.7</v>
+      </c>
+      <c r="H88" s="120" t="n">
+        <v>12231978</v>
+      </c>
+      <c r="I88" s="120" t="n">
+        <v>2407</v>
+      </c>
+      <c r="J88" s="120" t="n">
+        <v>1001</v>
+      </c>
+      <c r="K88" s="120" t="n">
+        <v>641</v>
+      </c>
+      <c r="L88" s="121" t="n">
+        <v>12236027</v>
       </c>
     </row>
     <row r="89">
@@ -17124,33 +16638,26 @@
       <c r="E89" s="236" t="n">
         <v>119060</v>
       </c>
-      <c r="F89" s="240">
-        <f>D89/E89</f>
-        <v/>
-      </c>
-      <c r="G89" s="236">
-        <f>F40</f>
-        <v/>
-      </c>
-      <c r="H89" s="238">
-        <f>ROUND(D89*G89,0)</f>
-        <v/>
-      </c>
-      <c r="I89" s="238">
-        <f>ROUND(G40*F89*G89,0)</f>
-        <v/>
-      </c>
-      <c r="J89" s="238">
-        <f>ROUND(H40*F89,0)</f>
-        <v/>
-      </c>
-      <c r="K89" s="238">
-        <f>ROUND(I40*F89,0)</f>
-        <v/>
-      </c>
-      <c r="L89" s="239">
-        <f>H89+I89+J89+K89</f>
-        <v/>
+      <c r="F89" s="240" t="n">
+        <v>0.0042</v>
+      </c>
+      <c r="G89" s="236" t="n">
+        <v>1525.3</v>
+      </c>
+      <c r="H89" s="238" t="n">
+        <v>762650</v>
+      </c>
+      <c r="I89" s="238" t="n">
+        <v>128</v>
+      </c>
+      <c r="J89" s="238" t="n">
+        <v>52</v>
+      </c>
+      <c r="K89" s="238" t="n">
+        <v>34</v>
+      </c>
+      <c r="L89" s="239" t="n">
+        <v>762864</v>
       </c>
     </row>
     <row r="90">
@@ -17175,33 +16682,26 @@
       <c r="E90" s="236" t="n">
         <v>119060</v>
       </c>
-      <c r="F90" s="240">
-        <f>D90/E90</f>
-        <v/>
-      </c>
-      <c r="G90" s="236">
-        <f>F40</f>
-        <v/>
-      </c>
-      <c r="H90" s="238">
-        <f>ROUND(D90*G90,0)</f>
-        <v/>
-      </c>
-      <c r="I90" s="238">
-        <f>ROUND(G40*F90*G90,0)</f>
-        <v/>
-      </c>
-      <c r="J90" s="238">
-        <f>ROUND(H40*F90,0)</f>
-        <v/>
-      </c>
-      <c r="K90" s="238">
-        <f>ROUND(I40*F90,0)</f>
-        <v/>
-      </c>
-      <c r="L90" s="239">
-        <f>H90+I90+J90+K90</f>
-        <v/>
+      <c r="F90" s="240" t="n">
+        <v>0.580884</v>
+      </c>
+      <c r="G90" s="236" t="n">
+        <v>1525.3</v>
+      </c>
+      <c r="H90" s="238" t="n">
+        <v>105489748</v>
+      </c>
+      <c r="I90" s="238" t="n">
+        <v>17720</v>
+      </c>
+      <c r="J90" s="238" t="n">
+        <v>7261</v>
+      </c>
+      <c r="K90" s="238" t="n">
+        <v>4647</v>
+      </c>
+      <c r="L90" s="239" t="n">
+        <v>105519376</v>
       </c>
     </row>
     <row r="91">
@@ -17226,33 +16726,26 @@
       <c r="E91" s="236" t="n">
         <v>119060</v>
       </c>
-      <c r="F91" s="240">
-        <f>D91/E91</f>
-        <v/>
-      </c>
-      <c r="G91" s="236">
-        <f>F40</f>
-        <v/>
-      </c>
-      <c r="H91" s="238">
-        <f>ROUND(D91*G91,0)</f>
-        <v/>
-      </c>
-      <c r="I91" s="238">
-        <f>ROUND(G40*F91*G91,0)</f>
-        <v/>
-      </c>
-      <c r="J91" s="238">
-        <f>ROUND(H40*F91,0)</f>
-        <v/>
-      </c>
-      <c r="K91" s="238">
-        <f>ROUND(I40*F91,0)</f>
-        <v/>
-      </c>
-      <c r="L91" s="239">
-        <f>H91+I91+J91+K91</f>
-        <v/>
+      <c r="F91" s="240" t="n">
+        <v>0.414917</v>
+      </c>
+      <c r="G91" s="236" t="n">
+        <v>1525.3</v>
+      </c>
+      <c r="H91" s="238" t="n">
+        <v>75349820</v>
+      </c>
+      <c r="I91" s="238" t="n">
+        <v>12657</v>
+      </c>
+      <c r="J91" s="238" t="n">
+        <v>5186</v>
+      </c>
+      <c r="K91" s="238" t="n">
+        <v>3319</v>
+      </c>
+      <c r="L91" s="239" t="n">
+        <v>75370982</v>
       </c>
     </row>
   </sheetData>
@@ -17317,7 +16810,7 @@
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="163" t="inlineStr">
         <is>
-          <t>기준일: 2026-06-10  |  상환 완료 건은 초록색 표시  |  상환예정일 = 신한은행 PDF 만기일 기준</t>
+          <t>기준일: 2026-06-16  |  상환 완료 건은 초록색 표시  |  상환예정일 = 신한은행 PDF 만기일 기준</t>
         </is>
       </c>
     </row>
@@ -17604,64 +17097,76 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="59" t="n">
+      <c r="A16" s="276" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="59" t="inlineStr">
+      <c r="B16" s="276" t="inlineStr">
         <is>
           <t>CPO-672</t>
         </is>
       </c>
-      <c r="C16" s="74" t="inlineStr">
+      <c r="C16" s="277" t="inlineStr">
         <is>
           <t>Christie</t>
         </is>
       </c>
-      <c r="D16" s="60" t="n">
+      <c r="D16" s="278" t="n">
         <v>221868</v>
       </c>
-      <c r="E16" s="59" t="inlineStr">
+      <c r="E16" s="276" t="inlineStr">
         <is>
           <t>신한은행</t>
         </is>
       </c>
-      <c r="F16" s="59" t="inlineStr">
+      <c r="F16" s="276" t="inlineStr">
         <is>
           <t>M88JX2510NU00018</t>
         </is>
       </c>
-      <c r="G16" s="59" t="inlineStr">
+      <c r="G16" s="276" t="inlineStr">
         <is>
           <t>2025-10-16</t>
         </is>
       </c>
-      <c r="H16" s="59" t="inlineStr">
+      <c r="H16" s="276" t="inlineStr">
         <is>
           <t>2026-04-14</t>
         </is>
       </c>
-      <c r="I16" s="59" t="inlineStr">
+      <c r="I16" s="276" t="inlineStr">
         <is>
           <t>180 Days</t>
         </is>
       </c>
-      <c r="J16" s="59" t="inlineStr">
+      <c r="J16" s="276" t="inlineStr">
         <is>
           <t>2025-12-16</t>
         </is>
       </c>
-      <c r="K16" s="59" t="inlineStr">
+      <c r="K16" s="276" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="L16" s="200" t="n">
-        <v>67</v>
-      </c>
-      <c r="M16" s="59" t="n"/>
-      <c r="N16" s="201" t="n"/>
-      <c r="O16" s="63" t="n"/>
-      <c r="P16" s="59" t="n"/>
+      <c r="L16" s="279" t="inlineStr">
+        <is>
+          <t>상환완료</t>
+        </is>
+      </c>
+      <c r="M16" s="280" t="n">
+        <v>46189</v>
+      </c>
+      <c r="N16" s="278" t="n">
+        <v>1517.2</v>
+      </c>
+      <c r="O16" s="281" t="n">
+        <v>336629315</v>
+      </c>
+      <c r="P16" s="276" t="inlineStr">
+        <is>
+          <t>6/16 만기 상환 완료 (외국환 거래표 2026-06-16, REF M88JX2510NU00018). 원금 USD 221,868.99 → 원화 336,629,315 (적용환율 1,517.20). 미결제잔액 USD 0.00</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="245" t="n">
@@ -19602,7 +19107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="15" customWidth="1" style="40" min="1" max="2"/>
@@ -19645,7 +19150,7 @@
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="205" t="inlineStr">
         <is>
-          <t>업데이트: 2026-06-02 (관세청 고시환율)</t>
+          <t>업데이트: 2026-06-16 (관세청 고시환율)</t>
         </is>
       </c>
       <c r="B4" s="148" t="n"/>
@@ -20249,6 +19754,22 @@
       </c>
       <c r="D42" s="211" t="n">
         <v>1514.68</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="282" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B43" s="282" t="n">
+        <v>46193</v>
+      </c>
+      <c r="C43" s="207" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D43" s="211" t="n">
+        <v>1531.46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update latest.xlsx: 취득원가 기준(부가세 제외) 2026-07-07
</commit_message>
<xml_diff>
--- a/latest.xlsx
+++ b/latest.xlsx
@@ -1901,7 +1901,7 @@
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="170" t="inlineStr">
         <is>
-          <t>회계처리용 통합 데이터  |  기준일: 2026-07-02  |  노란색=미확인  |  보라색=라이센스/워런티  |  날짜→해당항목 좌측 배치</t>
+          <t>회계처리용 통합 데이터  |  기준일: 2026-07-07  |  노란색=미확인  |  보라색=라이센스/워런티  |  날짜→해당항목 좌측 배치</t>
         </is>
       </c>
       <c r="B2" s="148" t="n"/>
@@ -2092,7 +2092,7 @@
       </c>
       <c r="T4" s="155" t="inlineStr">
         <is>
-          <t>부가세(KRW)</t>
+          <t>부가세(KRW,참고)</t>
         </is>
       </c>
       <c r="U4" s="150" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="Z4" s="155" t="inlineStr">
         <is>
-          <t>소계:관부가세+통관(KRW)</t>
+          <t>소계:관세+통관(KRW)</t>
         </is>
       </c>
       <c r="AA4" s="155" t="inlineStr">
@@ -2251,7 +2251,7 @@
         <v>0</v>
       </c>
       <c r="Z5" s="9">
-        <f>S5+T5+W5</f>
+        <f>S5+W5</f>
         <v/>
       </c>
       <c r="AA5" s="123">
@@ -2378,7 +2378,7 @@
         <v>2470670</v>
       </c>
       <c r="Z6" s="9">
-        <f>S6+T6+W6</f>
+        <f>S6+W6</f>
         <v/>
       </c>
       <c r="AA6" s="10">
@@ -2505,7 +2505,7 @@
         <v>0</v>
       </c>
       <c r="Z7" s="9">
-        <f>S7+T7+W7</f>
+        <f>S7+W7</f>
         <v/>
       </c>
       <c r="AA7" s="10">
@@ -2632,7 +2632,7 @@
         <v>590823</v>
       </c>
       <c r="Z8" s="9">
-        <f>S8+T8+W8</f>
+        <f>S8+W8</f>
         <v/>
       </c>
       <c r="AA8" s="10">
@@ -2757,7 +2757,7 @@
         <v>0</v>
       </c>
       <c r="Z9" s="18">
-        <f>S9+T9+W9</f>
+        <f>S9+W9</f>
         <v/>
       </c>
       <c r="AA9" s="18">
@@ -2880,7 +2880,7 @@
         <v>4477</v>
       </c>
       <c r="Z10" s="9">
-        <f>S10+T10+W10</f>
+        <f>S10+W10</f>
         <v/>
       </c>
       <c r="AA10" s="10">
@@ -3007,7 +3007,7 @@
         <v>0</v>
       </c>
       <c r="Z11" s="9">
-        <f>S11+T11+W11</f>
+        <f>S11+W11</f>
         <v/>
       </c>
       <c r="AA11" s="10">
@@ -3134,7 +3134,7 @@
         <v>581438</v>
       </c>
       <c r="Z12" s="9">
-        <f>S12+T12+W12</f>
+        <f>S12+W12</f>
         <v/>
       </c>
       <c r="AA12" s="10">
@@ -3261,7 +3261,7 @@
         <v>2385057</v>
       </c>
       <c r="Z13" s="9">
-        <f>S13+T13+W13</f>
+        <f>S13+W13</f>
         <v/>
       </c>
       <c r="AA13" s="10">
@@ -3388,7 +3388,7 @@
         <v>1864148</v>
       </c>
       <c r="Z14" s="9">
-        <f>S14+T14+W14</f>
+        <f>S14+W14</f>
         <v/>
       </c>
       <c r="AA14" s="10">
@@ -3515,7 +3515,7 @@
         <v>426904</v>
       </c>
       <c r="Z15" s="9">
-        <f>S15+T15+W15</f>
+        <f>S15+W15</f>
         <v/>
       </c>
       <c r="AA15" s="10">
@@ -3642,7 +3642,7 @@
         <v>2690702</v>
       </c>
       <c r="Z16" s="9">
-        <f>S16+T16+W16</f>
+        <f>S16+W16</f>
         <v/>
       </c>
       <c r="AA16" s="10">
@@ -3769,7 +3769,7 @@
         <v>1379682</v>
       </c>
       <c r="Z17" s="9">
-        <f>S17+T17+W17</f>
+        <f>S17+W17</f>
         <v/>
       </c>
       <c r="AA17" s="10">
@@ -3896,7 +3896,7 @@
         <v>162080</v>
       </c>
       <c r="Z18" s="9">
-        <f>S18+T18+W18</f>
+        <f>S18+W18</f>
         <v/>
       </c>
       <c r="AA18" s="10">
@@ -4023,7 +4023,7 @@
         <v>136050</v>
       </c>
       <c r="Z19" s="9">
-        <f>S19+T19+W19</f>
+        <f>S19+W19</f>
         <v/>
       </c>
       <c r="AA19" s="10">
@@ -4150,7 +4150,7 @@
         <v>1553086</v>
       </c>
       <c r="Z20" s="9">
-        <f>S20+T20+W20</f>
+        <f>S20+W20</f>
         <v/>
       </c>
       <c r="AA20" s="10">
@@ -4277,7 +4277,7 @@
         <v>2649525</v>
       </c>
       <c r="Z21" s="9">
-        <f>S21+T21+W21</f>
+        <f>S21+W21</f>
         <v/>
       </c>
       <c r="AA21" s="10">
@@ -4404,7 +4404,7 @@
         <v>1561040</v>
       </c>
       <c r="Z22" s="9">
-        <f>S22+T22+W22</f>
+        <f>S22+W22</f>
         <v/>
       </c>
       <c r="AA22" s="10">
@@ -4529,7 +4529,7 @@
         <v>0</v>
       </c>
       <c r="Z23" s="18">
-        <f>S23+T23+W23</f>
+        <f>S23+W23</f>
         <v/>
       </c>
       <c r="AA23" s="18">
@@ -4652,7 +4652,7 @@
         <v>1232133</v>
       </c>
       <c r="Z24" s="9">
-        <f>S24+T24+W24</f>
+        <f>S24+W24</f>
         <v/>
       </c>
       <c r="AA24" s="10">
@@ -4779,7 +4779,7 @@
         <v>6128</v>
       </c>
       <c r="Z25" s="9">
-        <f>S25+T25+W25</f>
+        <f>S25+W25</f>
         <v/>
       </c>
       <c r="AA25" s="10">
@@ -4906,7 +4906,7 @@
         <v>904960</v>
       </c>
       <c r="Z26" s="9">
-        <f>S26+T26+W26</f>
+        <f>S26+W26</f>
         <v/>
       </c>
       <c r="AA26" s="10">
@@ -5033,7 +5033,7 @@
         <v>6264783</v>
       </c>
       <c r="Z27" s="9">
-        <f>S27+T27+W27</f>
+        <f>S27+W27</f>
         <v/>
       </c>
       <c r="AA27" s="10">
@@ -5160,7 +5160,7 @@
         <v>1454605</v>
       </c>
       <c r="Z28" s="9">
-        <f>S28+T28+W28</f>
+        <f>S28+W28</f>
         <v/>
       </c>
       <c r="AA28" s="10">
@@ -5283,7 +5283,7 @@
         <v>174806</v>
       </c>
       <c r="Z29" s="9">
-        <f>S29+T29+W29</f>
+        <f>S29+W29</f>
         <v/>
       </c>
       <c r="AA29" s="10">
@@ -5398,7 +5398,7 @@
         <v>3909069</v>
       </c>
       <c r="Z30" s="82">
-        <f>S30+T30+W30</f>
+        <f>S30+W30</f>
         <v/>
       </c>
       <c r="AA30" s="83">
@@ -5513,7 +5513,7 @@
         <v>846621</v>
       </c>
       <c r="Z31" s="82">
-        <f>S31+T31+W31</f>
+        <f>S31+W31</f>
         <v/>
       </c>
       <c r="AA31" s="83">
@@ -5622,7 +5622,7 @@
         <v>0</v>
       </c>
       <c r="Z32" s="82">
-        <f>S32+T32+W32</f>
+        <f>S32+W32</f>
         <v/>
       </c>
       <c r="AA32" s="83">
@@ -5729,7 +5729,7 @@
         <v>3103207</v>
       </c>
       <c r="Z33" s="128">
-        <f>S33+T33+W33</f>
+        <f>S33+W33</f>
         <v/>
       </c>
       <c r="AA33" s="131">
@@ -5846,7 +5846,7 @@
         <v>3270326</v>
       </c>
       <c r="Z34" s="128">
-        <f>S34+T34+W34</f>
+        <f>S34+W34</f>
         <v/>
       </c>
       <c r="AA34" s="131">
@@ -5957,7 +5957,7 @@
         <v>3636072</v>
       </c>
       <c r="Z35" s="128">
-        <f>S35+T35+W35</f>
+        <f>S35+W35</f>
         <v/>
       </c>
       <c r="AA35" s="131">
@@ -6058,7 +6058,7 @@
         <v>0</v>
       </c>
       <c r="Z36" s="128">
-        <f>S36+T36+W36</f>
+        <f>S36+W36</f>
         <v/>
       </c>
       <c r="AA36" s="131">
@@ -6169,7 +6169,7 @@
         <v>3759954</v>
       </c>
       <c r="Z37" s="213">
-        <f>S37+T37+W37</f>
+        <f>S37+W37</f>
         <v/>
       </c>
       <c r="AA37" s="214">
@@ -6284,7 +6284,7 @@
         <v>2259958</v>
       </c>
       <c r="Z38" s="213">
-        <f>S38+T38+W38</f>
+        <f>S38+W38</f>
         <v/>
       </c>
       <c r="AA38" s="214">
@@ -6401,7 +6401,7 @@
         <v>159250</v>
       </c>
       <c r="Z39" s="128">
-        <f>S39+T39+W39</f>
+        <f>S39+W39</f>
         <v/>
       </c>
       <c r="AA39" s="131">
@@ -6526,7 +6526,7 @@
         <v>2898404</v>
       </c>
       <c r="Z40" s="128">
-        <f>S40+T40+W40</f>
+        <f>S40+W40</f>
         <v/>
       </c>
       <c r="AA40" s="131">
@@ -6641,7 +6641,7 @@
         <v>14471173</v>
       </c>
       <c r="Z41" s="128">
-        <f>S41+T41+W41</f>
+        <f>S41+W41</f>
         <v/>
       </c>
       <c r="AA41" s="131">
@@ -6756,7 +6756,7 @@
         <v>3412382</v>
       </c>
       <c r="Z42" s="128">
-        <f>S42+T42+W42</f>
+        <f>S42+W42</f>
         <v/>
       </c>
       <c r="AA42" s="131">
@@ -6873,7 +6873,7 @@
         <v>692650</v>
       </c>
       <c r="Z43" s="128">
-        <f>S43+T43+W43</f>
+        <f>S43+W43</f>
         <v/>
       </c>
       <c r="AA43" s="131">
@@ -6984,7 +6984,7 @@
         <v>0</v>
       </c>
       <c r="Z44" s="128">
-        <f>S44+T44+W44</f>
+        <f>S44+W44</f>
         <v/>
       </c>
       <c r="AA44" s="131">
@@ -7099,7 +7099,7 @@
         <v>0</v>
       </c>
       <c r="Z45" s="302">
-        <f>S45+T45+W45</f>
+        <f>S45+W45</f>
         <v/>
       </c>
       <c r="AA45" s="302">
@@ -7226,7 +7226,7 @@
         <v>0</v>
       </c>
       <c r="Z46" s="302">
-        <f>S46+T46+W46</f>
+        <f>S46+W46</f>
         <v/>
       </c>
       <c r="AA46" s="302">
@@ -7353,7 +7353,7 @@
         <v>0</v>
       </c>
       <c r="Z47" s="302">
-        <f>S47+T47+W47</f>
+        <f>S47+W47</f>
         <v/>
       </c>
       <c r="AA47" s="302">
@@ -7480,7 +7480,7 @@
         <v>0</v>
       </c>
       <c r="Z48" s="302">
-        <f>S48+T48+W48</f>
+        <f>S48+W48</f>
         <v/>
       </c>
       <c r="AA48" s="302">
@@ -7607,7 +7607,7 @@
         <v>0</v>
       </c>
       <c r="Z49" s="302">
-        <f>S49+T49+W49</f>
+        <f>S49+W49</f>
         <v/>
       </c>
       <c r="AA49" s="302">
@@ -7734,7 +7734,7 @@
         <v>0</v>
       </c>
       <c r="Z50" s="302">
-        <f>S50+T50+W50</f>
+        <f>S50+W50</f>
         <v/>
       </c>
       <c r="AA50" s="302">
@@ -7867,7 +7867,7 @@
         <v>0</v>
       </c>
       <c r="Z51" s="302">
-        <f>S51+T51+W51</f>
+        <f>S51+W51</f>
         <v/>
       </c>
       <c r="AA51" s="302">
@@ -7994,7 +7994,7 @@
         <v>0</v>
       </c>
       <c r="Z52" s="302">
-        <f>S52+T52+W52</f>
+        <f>S52+W52</f>
         <v/>
       </c>
       <c r="AA52" s="302">
@@ -8127,7 +8127,7 @@
         <v>0</v>
       </c>
       <c r="Z53" s="302">
-        <f>S53+T53+W53</f>
+        <f>S53+W53</f>
         <v/>
       </c>
       <c r="AA53" s="302">
@@ -8254,7 +8254,7 @@
         <v>0</v>
       </c>
       <c r="Z54" s="302">
-        <f>S54+T54+W54</f>
+        <f>S54+W54</f>
         <v/>
       </c>
       <c r="AA54" s="302">
@@ -8381,7 +8381,7 @@
         <v>0</v>
       </c>
       <c r="Z55" s="302">
-        <f>S55+T55+W55</f>
+        <f>S55+W55</f>
         <v/>
       </c>
       <c r="AA55" s="302">
@@ -8508,7 +8508,7 @@
         <v>0</v>
       </c>
       <c r="Z56" s="302">
-        <f>S56+T56+W56</f>
+        <f>S56+W56</f>
         <v/>
       </c>
       <c r="AA56" s="302">
@@ -8635,7 +8635,7 @@
         <v>0</v>
       </c>
       <c r="Z57" s="302">
-        <f>S57+T57+W57</f>
+        <f>S57+W57</f>
         <v/>
       </c>
       <c r="AA57" s="302">
@@ -8762,7 +8762,7 @@
         <v>0</v>
       </c>
       <c r="Z58" s="302">
-        <f>S58+T58+W58</f>
+        <f>S58+W58</f>
         <v/>
       </c>
       <c r="AA58" s="302">
@@ -8889,7 +8889,7 @@
         <v>0</v>
       </c>
       <c r="Z59" s="302">
-        <f>S59+T59+W59</f>
+        <f>S59+W59</f>
         <v/>
       </c>
       <c r="AA59" s="302">
@@ -9016,7 +9016,7 @@
         <v>0</v>
       </c>
       <c r="Z60" s="302">
-        <f>S60+T60+W60</f>
+        <f>S60+W60</f>
         <v/>
       </c>
       <c r="AA60" s="302">
@@ -9143,7 +9143,7 @@
         <v>0</v>
       </c>
       <c r="Z61" s="302">
-        <f>S61+T61+W61</f>
+        <f>S61+W61</f>
         <v/>
       </c>
       <c r="AA61" s="302">
@@ -9268,7 +9268,7 @@
         <v>0</v>
       </c>
       <c r="Z62" s="308">
-        <f>S62+T62+W62</f>
+        <f>S62+W62</f>
         <v/>
       </c>
       <c r="AA62" s="308">
@@ -9395,7 +9395,7 @@
         <v>0</v>
       </c>
       <c r="Z63" s="308">
-        <f>S63+T63+W63</f>
+        <f>S63+W63</f>
         <v/>
       </c>
       <c r="AA63" s="308">
@@ -9500,7 +9500,7 @@
         <v>0</v>
       </c>
       <c r="Z64" s="136">
-        <f>S64+T64+W64</f>
+        <f>S64+W64</f>
         <v/>
       </c>
       <c r="AA64" s="136">
@@ -9605,7 +9605,7 @@
         <v>0</v>
       </c>
       <c r="Z65" s="136">
-        <f>S65+T65+W65</f>
+        <f>S65+W65</f>
         <v/>
       </c>
       <c r="AA65" s="136">
@@ -9710,7 +9710,7 @@
         <v>0</v>
       </c>
       <c r="Z66" s="136">
-        <f>S66+T66+W66</f>
+        <f>S66+W66</f>
         <v/>
       </c>
       <c r="AA66" s="136">
@@ -9823,7 +9823,7 @@
         <v>0</v>
       </c>
       <c r="Z67" s="136">
-        <f>S67+T67+W67</f>
+        <f>S67+W67</f>
         <v/>
       </c>
       <c r="AA67" s="136">
@@ -9938,7 +9938,7 @@
         <v>0</v>
       </c>
       <c r="Z68" s="136">
-        <f>S68+T68+W68</f>
+        <f>S68+W68</f>
         <v/>
       </c>
       <c r="AA68" s="136">
@@ -10053,7 +10053,7 @@
         <v>0</v>
       </c>
       <c r="Z69" s="136">
-        <f>S69+T69+W69</f>
+        <f>S69+W69</f>
         <v/>
       </c>
       <c r="AA69" s="136">
@@ -10168,7 +10168,7 @@
         <v>0</v>
       </c>
       <c r="Z70" s="136">
-        <f>S70+T70+W70</f>
+        <f>S70+W70</f>
         <v/>
       </c>
       <c r="AA70" s="136">
@@ -10283,7 +10283,7 @@
         <v>0</v>
       </c>
       <c r="Z71" s="136">
-        <f>S71+T71+W71</f>
+        <f>S71+W71</f>
         <v/>
       </c>
       <c r="AA71" s="136">
@@ -10412,7 +10412,7 @@
         <v>0</v>
       </c>
       <c r="Z72" s="290">
-        <f>S72+T72+W72</f>
+        <f>S72+W72</f>
         <v/>
       </c>
       <c r="AA72" s="290">
@@ -10539,7 +10539,7 @@
         <v>216006</v>
       </c>
       <c r="Z73" s="290">
-        <f>S73+T73+W73</f>
+        <f>S73+W73</f>
         <v/>
       </c>
       <c r="AA73" s="290">
@@ -10655,7 +10655,7 @@
         <v>5002612</v>
       </c>
       <c r="Z74" s="222">
-        <f>S74+T74+W74</f>
+        <f>S74+W74</f>
         <v/>
       </c>
       <c r="AA74" s="222">
@@ -10760,7 +10760,7 @@
         <v>0</v>
       </c>
       <c r="Z75" s="290">
-        <f>S75+T75+W75</f>
+        <f>S75+W75</f>
         <v/>
       </c>
       <c r="AA75" s="290">
@@ -11062,6 +11062,19 @@
       <c r="AE79" s="145" t="n"/>
       <c r="AF79" s="145" t="n"/>
     </row>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
     <row r="93">
       <c r="M93" s="40" t="n"/>
     </row>

</xml_diff>

<commit_message>
Update latest.xlsx 2026-09-09 11:09
</commit_message>
<xml_diff>
--- a/latest.xlsx
+++ b/latest.xlsx
@@ -5914,7 +5914,7 @@
         <v>75349820</v>
       </c>
       <c r="L34" s="213" t="n">
-        <v>5186</v>
+        <v>5187</v>
       </c>
       <c r="M34" s="213" t="n">
         <v>3319</v>
@@ -6591,10 +6591,10 @@
         <v>1517.3</v>
       </c>
       <c r="J40" s="128" t="n">
-        <v>74558330</v>
+        <v>74558301</v>
       </c>
       <c r="K40" s="128" t="n">
-        <v>74558330</v>
+        <v>74558301</v>
       </c>
       <c r="L40" s="128" t="n">
         <v>10115</v>
@@ -6706,10 +6706,10 @@
         <v>1517.3</v>
       </c>
       <c r="J41" s="128" t="n">
-        <v>17582284</v>
+        <v>17581259</v>
       </c>
       <c r="K41" s="128" t="n">
-        <v>17582284</v>
+        <v>17581259</v>
       </c>
       <c r="L41" s="128" t="n">
         <v>2385</v>
@@ -7114,7 +7114,7 @@
         </is>
       </c>
       <c r="Y44" s="128" t="n">
-        <v>593662</v>
+        <v>593664</v>
       </c>
       <c r="Z44" s="128">
         <f>S44+W44</f>
@@ -8479,7 +8479,7 @@
         </is>
       </c>
       <c r="Y55" s="128" t="n">
-        <v>45948</v>
+        <v>45946</v>
       </c>
       <c r="Z55" s="128">
         <f>S55+W55</f>
@@ -8626,15 +8626,11 @@
           <t>2025-09</t>
         </is>
       </c>
-      <c r="AE56" s="299" t="inlineStr">
-        <is>
-          <t>2025-09-13</t>
-        </is>
-      </c>
-      <c r="AF56" s="298" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="AE56" s="299" t="n">
+        <v>45913</v>
+      </c>
+      <c r="AF56" s="298" t="n">
+        <v>46262</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
@@ -8751,15 +8747,11 @@
           <t>2025-12</t>
         </is>
       </c>
-      <c r="AE57" s="299" t="inlineStr">
-        <is>
-          <t>2025-12-01</t>
-        </is>
-      </c>
-      <c r="AF57" s="298" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
+      <c r="AE57" s="299" t="n">
+        <v>45992</v>
+      </c>
+      <c r="AF57" s="298" t="n">
+        <v>46356</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
@@ -8876,15 +8868,11 @@
           <t>2025-12</t>
         </is>
       </c>
-      <c r="AE58" s="299" t="inlineStr">
-        <is>
-          <t>2025-12-22</t>
-        </is>
-      </c>
-      <c r="AF58" s="298" t="inlineStr">
-        <is>
-          <t>2026-12-21</t>
-        </is>
+      <c r="AE58" s="299" t="n">
+        <v>46013</v>
+      </c>
+      <c r="AF58" s="298" t="n">
+        <v>46377</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
@@ -9001,15 +8989,11 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE59" s="299" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="AF59" s="298" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="AE59" s="299" t="n">
+        <v>46023</v>
+      </c>
+      <c r="AF59" s="298" t="n">
+        <v>46387</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
@@ -9126,15 +9110,11 @@
           <t>2025-11</t>
         </is>
       </c>
-      <c r="AE60" s="299" t="inlineStr">
-        <is>
-          <t>2025-11-01</t>
-        </is>
-      </c>
-      <c r="AF60" s="298" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
+      <c r="AE60" s="299" t="n">
+        <v>45962</v>
+      </c>
+      <c r="AF60" s="298" t="n">
+        <v>46325</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
@@ -9251,15 +9231,11 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE61" s="299" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="AF61" s="298" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="AE61" s="299" t="n">
+        <v>46023</v>
+      </c>
+      <c r="AF61" s="298" t="n">
+        <v>46387</v>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
@@ -9382,15 +9358,11 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE62" s="299" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="AF62" s="298" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="AE62" s="299" t="n">
+        <v>46023</v>
+      </c>
+      <c r="AF62" s="298" t="n">
+        <v>46387</v>
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
@@ -9507,15 +9479,11 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE63" s="299" t="inlineStr">
-        <is>
-          <t>2026-01-30</t>
-        </is>
-      </c>
-      <c r="AF63" s="298" t="inlineStr">
-        <is>
-          <t>2027-01-29</t>
-        </is>
+      <c r="AE63" s="299" t="n">
+        <v>46052</v>
+      </c>
+      <c r="AF63" s="298" t="n">
+        <v>46416</v>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
@@ -9763,15 +9731,11 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE65" s="299" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="AF65" s="298" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="AE65" s="299" t="n">
+        <v>46023</v>
+      </c>
+      <c r="AF65" s="298" t="n">
+        <v>46387</v>
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
@@ -9888,15 +9852,11 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE66" s="299" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="AF66" s="298" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="AE66" s="299" t="n">
+        <v>46023</v>
+      </c>
+      <c r="AF66" s="298" t="n">
+        <v>46387</v>
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
@@ -10013,15 +9973,11 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE67" s="299" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="AF67" s="298" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="AE67" s="299" t="n">
+        <v>46023</v>
+      </c>
+      <c r="AF67" s="298" t="n">
+        <v>46387</v>
       </c>
     </row>
     <row r="68" ht="15.75" customHeight="1">
@@ -10138,15 +10094,11 @@
           <t>2026-03</t>
         </is>
       </c>
-      <c r="AE68" s="299" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-      <c r="AF68" s="298" t="inlineStr">
-        <is>
-          <t>2027-02-28</t>
-        </is>
+      <c r="AE68" s="299" t="n">
+        <v>46082</v>
+      </c>
+      <c r="AF68" s="298" t="n">
+        <v>46446</v>
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
@@ -10263,15 +10215,11 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE69" s="299" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="AF69" s="298" t="inlineStr">
-        <is>
-          <t>2027-02-22</t>
-        </is>
+      <c r="AE69" s="299" t="n">
+        <v>46023</v>
+      </c>
+      <c r="AF69" s="298" t="n">
+        <v>46440</v>
       </c>
     </row>
     <row r="70" ht="15.75" customHeight="1">
@@ -10388,15 +10336,11 @@
           <t>2026-03</t>
         </is>
       </c>
-      <c r="AE70" s="299" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-      <c r="AF70" s="298" t="inlineStr">
-        <is>
-          <t>2027-02-28</t>
-        </is>
+      <c r="AE70" s="299" t="n">
+        <v>46082</v>
+      </c>
+      <c r="AF70" s="298" t="n">
+        <v>46446</v>
       </c>
     </row>
     <row r="71" ht="15.75" customHeight="1">
@@ -10442,10 +10386,10 @@
         <v>753200</v>
       </c>
       <c r="L71" s="302" t="n">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="M71" s="302" t="n">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="N71" s="296" t="inlineStr">
         <is>
@@ -10638,15 +10582,11 @@
           <t>2026-04</t>
         </is>
       </c>
-      <c r="AE72" s="299" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="AF72" s="298" t="inlineStr">
-        <is>
-          <t>2027-03-31</t>
-        </is>
+      <c r="AE72" s="299" t="n">
+        <v>46113</v>
+      </c>
+      <c r="AF72" s="298" t="n">
+        <v>46477</v>
       </c>
     </row>
     <row r="73" ht="15.75" customHeight="1">
@@ -11101,7 +11041,7 @@
       </c>
       <c r="AD76" s="304" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="AE76" s="305" t="n">
@@ -13154,14 +13094,6 @@
     <row r="102">
       <c r="M102" s="40" t="n"/>
     </row>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="A93:G93"/>
@@ -13363,7 +13295,7 @@
         <v>45982</v>
       </c>
       <c r="H4" s="184" t="n">
-        <v>46014</v>
+        <v>46020</v>
       </c>
       <c r="I4" s="184" t="n">
         <v>45992</v>
@@ -14718,43 +14650,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
     <row r="70">
       <c r="M70" s="40" t="n"/>
     </row>
@@ -17116,22 +17011,6 @@
         </is>
       </c>
     </row>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
     <row r="71">
       <c r="M71" s="40" t="n"/>
     </row>
@@ -17151,7 +17030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M131"/>
+  <dimension ref="A1:M120"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="12.83203125" customWidth="1" style="160" min="1" max="1"/>
@@ -19450,17 +19329,17 @@
           <t>② PO별 비용 안분 내역</t>
         </is>
       </c>
-      <c r="B50" s="333" t="n"/>
-      <c r="C50" s="333" t="n"/>
-      <c r="D50" s="333" t="n"/>
-      <c r="E50" s="333" t="n"/>
-      <c r="F50" s="333" t="n"/>
-      <c r="G50" s="333" t="n"/>
-      <c r="H50" s="333" t="n"/>
-      <c r="I50" s="333" t="n"/>
-      <c r="J50" s="333" t="n"/>
-      <c r="K50" s="333" t="n"/>
-      <c r="L50" s="333" t="n"/>
+      <c r="B50" s="148" t="n"/>
+      <c r="C50" s="148" t="n"/>
+      <c r="D50" s="148" t="n"/>
+      <c r="E50" s="148" t="n"/>
+      <c r="F50" s="148" t="n"/>
+      <c r="G50" s="148" t="n"/>
+      <c r="H50" s="148" t="n"/>
+      <c r="I50" s="148" t="n"/>
+      <c r="J50" s="148" t="n"/>
+      <c r="K50" s="148" t="n"/>
+      <c r="L50" s="149" t="n"/>
       <c r="M50" s="228" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
@@ -20831,10 +20710,10 @@
         <v>2299</v>
       </c>
       <c r="J79" s="238" t="n">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="K79" s="238" t="n">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="L79" s="239">
         <f>H79+I79+J79+K79</f>
@@ -21865,7 +21744,7 @@
         <v>12657</v>
       </c>
       <c r="J101" s="238" t="n">
-        <v>5186</v>
+        <v>5187</v>
       </c>
       <c r="K101" s="238" t="n">
         <v>3319</v>
@@ -22000,7 +21879,7 @@
         <v>1517.3</v>
       </c>
       <c r="H104" s="238" t="n">
-        <v>74558330</v>
+        <v>74558301</v>
       </c>
       <c r="I104" s="238" t="n">
         <v>24555</v>
@@ -22047,7 +21926,7 @@
         <v>1517.3</v>
       </c>
       <c r="H105" s="238" t="n">
-        <v>17582284</v>
+        <v>17581259</v>
       </c>
       <c r="I105" s="238" t="n">
         <v>5791</v>
@@ -22761,17 +22640,6 @@
         <v/>
       </c>
     </row>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A50:L50"/>

</xml_diff>